<commit_message>
feat(tools): rediseno ejecutivo del Excel de Declaracion Patrimonial
Dashboard premium con tarjetas KPI y resumen separado en tres bloques:
ACTIVOS, PASIVOS y PATRIMONIO NETO. Hojas de grupo con estilo ejecutivo,
filas alternadas y totales por color de categoria.

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -21,10 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%;0.0%"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,35 +37,85 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007A7A7A"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A1A1A"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001E6B52"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <color rgb="007A7A7A"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00A23B3B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0020507D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="001A1A1A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007A7A7A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001A1A1A"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="0010243E"/>
       <sz val="12"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -73,27 +124,57 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="0010243E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00C8A24B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="001F3B5C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FCEFC9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E6B52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A23B3B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F0EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0020507D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EAF2"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,69 +188,216 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D3D8"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D3D8"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D3D8"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D3D8"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -259,7 +487,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Total por grupo: 2025 vs 2026</a:t>
+              <a:t>Activos / Pasivos / Patrimonio: 2025 vs 2026</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -274,7 +502,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!B4</f>
+              <f>'Dashboard'!D35</f>
             </strRef>
           </tx>
           <spPr>
@@ -284,12 +512,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$5:$A$8</f>
+              <f>'Dashboard'!$B$36:$B$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$5:$B$8</f>
+              <f>'Dashboard'!$D$36:$D$38</f>
             </numRef>
           </val>
         </ser>
@@ -298,7 +526,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!C4</f>
+              <f>'Dashboard'!E35</f>
             </strRef>
           </tx>
           <spPr>
@@ -308,12 +536,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$5:$A$8</f>
+              <f>'Dashboard'!$B$36:$B$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$C$5:$C$8</f>
+              <f>'Dashboard'!$E$36:$E$38</f>
             </numRef>
           </val>
         </ser>
@@ -384,15 +612,18 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$5:$A$7</f>
+              <f>'Dashboard'!$B$13:$B$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$5:$B$7</f>
+              <f>'Dashboard'!$D$13:$D$15</f>
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showPercent val="1"/>
+        </dLbls>
         <firstSliceAng val="0"/>
       </pieChart>
     </plotArea>
@@ -418,7 +649,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Variacion proyectada por grupo (2025-&gt;2026)</a:t>
+              <a:t>Variacion proyectada (2025 -&gt; 2026)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -433,7 +664,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!D4</f>
+              <f>'Dashboard'!F35</f>
             </strRef>
           </tx>
           <spPr>
@@ -443,12 +674,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$5:$A$8</f>
+              <f>'Dashboard'!$B$36:$B$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$D$5:$D$8</f>
+              <f>'Dashboard'!$F$36:$F$38</f>
             </numRef>
           </val>
         </ser>
@@ -492,12 +723,12 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="3240000"/>
+    <ext cx="5400000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -514,12 +745,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>21</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5040000" cy="3240000"/>
+    <ext cx="5040000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -536,12 +767,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>38</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="3240000"/>
+    <ext cx="5400000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -848,276 +1079,636 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DASHBOARD - DECLARACION PATRIMONIAL 2025 vs 2026</t>
+          <t>DECLARACION PATRIMONIAL  -  TABLERO EJECUTIVO</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Declarante: GONZALEZ NAVAS MARCO VINICIO  |  R - RUC: 1709164899001  |  SOC - Sociedad conyugal</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Edite la columna amarilla en cada hoja de grupo; los totales, variaciones y graficos se actualizan solos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Grupo</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+          <t>GONZALEZ NAVAS MARCO VINICIO   |   R - RUC: 1709164899001   |   SOC - Sociedad conyugal   |   Comparativo 2025 vs 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="5" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+    </row>
+    <row r="5" ht="6" customHeight="1">
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL ACTIVOS</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL PASIVOS</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>PATRIMONIO NETO</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="14">
+        <f>D17</f>
+        <v/>
+      </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="15">
+        <f>D22</f>
+        <v/>
+      </c>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="16">
+        <f>D28</f>
+        <v/>
+      </c>
+      <c r="G7" s="13" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Var. proyectada</t>
+        </is>
+      </c>
+      <c r="C8" s="18">
+        <f>G17</f>
+        <v/>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Var. proyectada</t>
+        </is>
+      </c>
+      <c r="E8" s="20">
+        <f>G22</f>
+        <v/>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>Var. proyectada</t>
+        </is>
+      </c>
+      <c r="G8" s="22">
+        <f>G28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>ACTIVOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="n"/>
+      <c r="D12" s="26" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="E12" s="26" t="inlineStr">
         <is>
           <t>Total 2026</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="F12" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="G12" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Dinero</t>
-        </is>
-      </c>
-      <c r="B5" s="6">
-        <f>'Dinero'!E8</f>
-        <v/>
-      </c>
-      <c r="C5" s="6">
-        <f>'Dinero'!F8</f>
-        <v/>
-      </c>
-      <c r="D5" s="6">
-        <f>C5-B5</f>
-        <v/>
-      </c>
-      <c r="E5" s="7">
-        <f>IF(B5=0,"",(C5-B5)/B5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>Dinero e inversiones</t>
+        </is>
+      </c>
+      <c r="D13" s="28">
+        <f>'Dinero'!E10</f>
+        <v/>
+      </c>
+      <c r="E13" s="28">
+        <f>'Dinero'!F10</f>
+        <v/>
+      </c>
+      <c r="F13" s="28">
+        <f>E13-D13</f>
+        <v/>
+      </c>
+      <c r="G13" s="29">
+        <f>IF(D13=0,"",(E13-D13)/D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>Vehiculos</t>
         </is>
       </c>
-      <c r="B6" s="6">
-        <f>'Vehiculos'!D7</f>
-        <v/>
-      </c>
-      <c r="C6" s="6">
-        <f>'Vehiculos'!E7</f>
-        <v/>
-      </c>
-      <c r="D6" s="6">
-        <f>C6-B6</f>
-        <v/>
-      </c>
-      <c r="E6" s="7">
-        <f>IF(B6=0,"",(C6-B6)/B6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Bienes Inmuebles</t>
-        </is>
-      </c>
-      <c r="B7" s="6">
-        <f>'Bienes Inmuebles'!E8</f>
-        <v/>
-      </c>
-      <c r="C7" s="6">
-        <f>'Bienes Inmuebles'!F8</f>
-        <v/>
-      </c>
-      <c r="D7" s="6">
-        <f>C7-B7</f>
-        <v/>
-      </c>
-      <c r="E7" s="7">
-        <f>IF(B7=0,"",(C7-B7)/B7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Pasivo</t>
-        </is>
-      </c>
-      <c r="B8" s="6">
-        <f>'Pasivo'!E6</f>
-        <v/>
-      </c>
-      <c r="C8" s="6">
-        <f>'Pasivo'!F6</f>
-        <v/>
-      </c>
-      <c r="D8" s="6">
-        <f>C8-B8</f>
-        <v/>
-      </c>
-      <c r="E8" s="7">
-        <f>IF(B8=0,"",(C8-B8)/B8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="D14" s="28">
+        <f>'Vehiculos'!D9</f>
+        <v/>
+      </c>
+      <c r="E14" s="28">
+        <f>'Vehiculos'!E9</f>
+        <v/>
+      </c>
+      <c r="F14" s="28">
+        <f>E14-D14</f>
+        <v/>
+      </c>
+      <c r="G14" s="29">
+        <f>IF(D14=0,"",(E14-D14)/D14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>Bienes inmuebles</t>
+        </is>
+      </c>
+      <c r="D15" s="28">
+        <f>'Bienes Inmuebles'!E10</f>
+        <v/>
+      </c>
+      <c r="E15" s="28">
+        <f>'Bienes Inmuebles'!F10</f>
+        <v/>
+      </c>
+      <c r="F15" s="28">
+        <f>E15-D15</f>
+        <v/>
+      </c>
+      <c r="G15" s="29">
+        <f>IF(D15=0,"",(E15-D15)/D15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>Total bruto de activos</t>
+        </is>
+      </c>
+      <c r="D16" s="28">
+        <f>SUM(D13:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="28">
+        <f>SUM(E13:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="28">
+        <f>E16-D16</f>
+        <v/>
+      </c>
+      <c r="G16" s="29">
+        <f>IF(D16=0,"",(E16-D16)/D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>TOTAL ACTIVOS</t>
         </is>
       </c>
-      <c r="B9" s="9">
-        <f>SUM(B5:B7)</f>
-        <v/>
-      </c>
-      <c r="C9" s="9">
-        <f>SUM(C5:C7)</f>
-        <v/>
-      </c>
-      <c r="D9" s="9">
-        <f>SUM(D5:D7)</f>
-        <v/>
-      </c>
-      <c r="E9" s="10">
-        <f>IF(B9=0,"",(C9-B9)/B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>PATRIMONIO NETO (Activos - Pasivo)</t>
-        </is>
-      </c>
-      <c r="B10" s="12">
-        <f>B9-B8</f>
-        <v/>
-      </c>
-      <c r="C10" s="12">
-        <f>C9-C8</f>
-        <v/>
-      </c>
-      <c r="D10" s="12">
-        <f>D9-D8</f>
-        <v/>
-      </c>
-      <c r="E10" s="13">
-        <f>IF(B10=0,"",(C10-B10)/B10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>INDICADORES CLAVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>Patrimonio declarado 2025</t>
-        </is>
-      </c>
-      <c r="B13" s="16">
-        <f>B10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Patrimonio declarado (XML) 2025</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="n">
+      <c r="D17" s="31">
+        <f>D16</f>
+        <v/>
+      </c>
+      <c r="E17" s="31">
+        <f>E16</f>
+        <v/>
+      </c>
+      <c r="F17" s="31">
+        <f>E17-D17</f>
+        <v/>
+      </c>
+      <c r="G17" s="32">
+        <f>IF(D17=0,"",(E17-D17)/D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>PASIVOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Total 2025</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>Total 2026</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>Variacion</t>
+        </is>
+      </c>
+      <c r="G20" s="26" t="inlineStr">
+        <is>
+          <t>Variacion %</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t>Deudas y obligaciones</t>
+        </is>
+      </c>
+      <c r="D21" s="35">
+        <f>'Pasivo'!E8</f>
+        <v/>
+      </c>
+      <c r="E21" s="35">
+        <f>'Pasivo'!F8</f>
+        <v/>
+      </c>
+      <c r="F21" s="35">
+        <f>E21-D21</f>
+        <v/>
+      </c>
+      <c r="G21" s="36">
+        <f>IF(D21=0,"",(E21-D21)/D21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="37" t="inlineStr">
+        <is>
+          <t>TOTAL PASIVOS</t>
+        </is>
+      </c>
+      <c r="D22" s="38">
+        <f>D21</f>
+        <v/>
+      </c>
+      <c r="E22" s="38">
+        <f>E21</f>
+        <v/>
+      </c>
+      <c r="F22" s="38">
+        <f>E22-D22</f>
+        <v/>
+      </c>
+      <c r="G22" s="39">
+        <f>IF(D22=0,"",(E22-D22)/D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="40" t="inlineStr">
+        <is>
+          <t>PATRIMONIO NETO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="26" t="inlineStr">
+        <is>
+          <t>Total 2025</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>Total 2026</t>
+        </is>
+      </c>
+      <c r="F25" s="26" t="inlineStr">
+        <is>
+          <t>Variacion</t>
+        </is>
+      </c>
+      <c r="G25" s="26" t="inlineStr">
+        <is>
+          <t>Variacion %</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>(+) Total activos</t>
+        </is>
+      </c>
+      <c r="D26" s="42">
+        <f>D17</f>
+        <v/>
+      </c>
+      <c r="E26" s="42">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="F26" s="42">
+        <f>E26-D26</f>
+        <v/>
+      </c>
+      <c r="G26" s="43">
+        <f>IF(D26=0,"",(E26-D26)/D26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="41" t="inlineStr">
+        <is>
+          <t>(-) Total pasivos</t>
+        </is>
+      </c>
+      <c r="D27" s="42">
+        <f>D22</f>
+        <v/>
+      </c>
+      <c r="E27" s="42">
+        <f>E22</f>
+        <v/>
+      </c>
+      <c r="F27" s="42">
+        <f>E27-D27</f>
+        <v/>
+      </c>
+      <c r="G27" s="43">
+        <f>IF(D27=0,"",(E27-D27)/D27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t>(=) PATRIMONIO NETO</t>
+        </is>
+      </c>
+      <c r="D28" s="45">
+        <f>D26-D27</f>
+        <v/>
+      </c>
+      <c r="E28" s="45">
+        <f>E26-E27</f>
+        <v/>
+      </c>
+      <c r="F28" s="45">
+        <f>E28-D28</f>
+        <v/>
+      </c>
+      <c r="G28" s="46">
+        <f>IF(D28=0,"",(E28-D28)/D28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="B29" s="47" t="inlineStr">
+        <is>
+          <t>Patrimonio declarado en el XML (2025)</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="48" t="n">
         <v>883285.5600000001</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Patrimonio anio anterior</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="n">
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="B30" s="47" t="inlineStr">
+        <is>
+          <t>Patrimonio neto del anio anterior</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="48" t="n">
         <v>801569.97</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Crecimiento patrimonial (XML)</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="n">
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="B31" s="47" t="inlineStr">
+        <is>
+          <t>Crecimiento patrimonial declarado (XML)</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="48" t="n">
         <v>81715.59</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Variacion proyectada 2025-&gt;2026</t>
-        </is>
-      </c>
-      <c r="B17" s="16">
-        <f>D10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>Variacion % proyectada 2025-&gt;2026</t>
-        </is>
-      </c>
-      <c r="B18" s="17">
-        <f>E10</f>
-        <v/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>CONSOLIDADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C35" s="25" t="n"/>
+      <c r="D35" s="26" t="inlineStr">
+        <is>
+          <t>Total 2025</t>
+        </is>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <t>Total 2026</t>
+        </is>
+      </c>
+      <c r="F35" s="26" t="inlineStr">
+        <is>
+          <t>Variacion</t>
+        </is>
+      </c>
+      <c r="G35" s="26" t="inlineStr">
+        <is>
+          <t>Variacion %</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="B36" s="50" t="inlineStr">
+        <is>
+          <t>Activos</t>
+        </is>
+      </c>
+      <c r="D36" s="51">
+        <f>D17</f>
+        <v/>
+      </c>
+      <c r="E36" s="51">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="F36" s="51">
+        <f>E36-D36</f>
+        <v/>
+      </c>
+      <c r="G36" s="52">
+        <f>IF(D36=0,"",(E36-D36)/D36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="B37" s="53" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="D37" s="54">
+        <f>D22</f>
+        <v/>
+      </c>
+      <c r="E37" s="54">
+        <f>E22</f>
+        <v/>
+      </c>
+      <c r="F37" s="54">
+        <f>E37-D37</f>
+        <v/>
+      </c>
+      <c r="G37" s="55">
+        <f>IF(D37=0,"",(E37-D37)/D37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="B38" s="56" t="inlineStr">
+        <is>
+          <t>Patrimonio neto</t>
+        </is>
+      </c>
+      <c r="D38" s="57">
+        <f>D28</f>
+        <v/>
+      </c>
+      <c r="E38" s="57">
+        <f>E28</f>
+        <v/>
+      </c>
+      <c r="F38" s="57">
+        <f>E38-D38</f>
+        <v/>
+      </c>
+      <c r="G38" s="58">
+        <f>IF(D38=0,"",(E38-D38)/D38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="59" t="inlineStr">
+        <is>
+          <t>Edite la columna amarilla en las hojas de cada grupo; las tarjetas, secciones y graficos se recalculan solos.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="36">
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B11:G11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1130,240 +1721,252 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DINERO E INVERSIONES</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Declaracion 2025  -  columna 2026 editable</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="5" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Institucion / detalle</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Moneda</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Valor 2026  (editable)</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>Valor 2026</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>IFI - Institucion financiera / ECU - Ecuador</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>3 - Inversion / poliza</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>1029</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E6" s="61" t="n">
         <v>130.2</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F6" s="62" t="n">
         <v>130.2</v>
       </c>
-      <c r="G4" s="6">
-        <f>F4-E4</f>
-        <v/>
-      </c>
-      <c r="H4" s="7">
-        <f>IF(E4=0,"",(F4-E4)/E4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="G6" s="61">
+        <f>F6-E6</f>
+        <v/>
+      </c>
+      <c r="H6" s="63">
+        <f>IF(E6=0,"",(F6-E6)/E6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>IFI - Institucion financiera / ECU - Ecuador</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>4 - Deposito a plazo</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>1029</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D7" s="64" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E7" s="65" t="n">
         <v>5590.32</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F7" s="62" t="n">
         <v>5590.32</v>
       </c>
-      <c r="G5" s="6">
-        <f>F5-E5</f>
-        <v/>
-      </c>
-      <c r="H5" s="7">
-        <f>IF(E5=0,"",(F5-E5)/E5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="G7" s="65">
+        <f>F7-E7</f>
+        <v/>
+      </c>
+      <c r="H7" s="66">
+        <f>IF(E7=0,"",(F7-E7)/E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>IFI - Institucion financiera / ECU - Ecuador</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>3 - Inversion / poliza</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>1418</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E8" s="61" t="n">
         <v>53237.31</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F8" s="62" t="n">
         <v>53237.31</v>
       </c>
-      <c r="G6" s="6">
-        <f>F6-E6</f>
-        <v/>
-      </c>
-      <c r="H6" s="7">
-        <f>IF(E6=0,"",(F6-E6)/E6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="G8" s="61">
+        <f>F8-E8</f>
+        <v/>
+      </c>
+      <c r="H8" s="63">
+        <f>IF(E8=0,"",(F8-E8)/E8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="64" t="inlineStr">
         <is>
           <t>IFI - Institucion financiera / EXT - Exterior</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B9" s="64" t="inlineStr">
         <is>
           <t>2 - Cuenta corriente</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C9" s="64" t="inlineStr">
         <is>
           <t>BANCO PICHINCHA CA</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D9" s="64" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E9" s="65" t="n">
         <v>189049.31</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F9" s="62" t="n">
         <v>189049.31</v>
       </c>
-      <c r="G7" s="6">
-        <f>F7-E7</f>
-        <v/>
-      </c>
-      <c r="H7" s="7">
-        <f>IF(E7=0,"",(F7-E7)/E7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="G9" s="65">
+        <f>F9-E9</f>
+        <v/>
+      </c>
+      <c r="H9" s="66">
+        <f>IF(E9=0,"",(F9-E9)/E9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n"/>
-      <c r="C8" s="20" t="n"/>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="21">
-        <f>SUM(E4:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="21">
-        <f>SUM(F4:F7)</f>
-        <v/>
-      </c>
-      <c r="G8" s="21">
-        <f>F8-E8</f>
-        <v/>
-      </c>
-      <c r="H8" s="22">
-        <f>IF(E8=0,"",(F8-E8)/E8)</f>
+      <c r="B10" s="67" t="n"/>
+      <c r="C10" s="67" t="n"/>
+      <c r="D10" s="67" t="n"/>
+      <c r="E10" s="31">
+        <f>SUM(E6:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="31">
+        <f>SUM(F6:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="31">
+        <f>F10-E10</f>
+        <v/>
+      </c>
+      <c r="H10" s="32">
+        <f>IF(E10=0,"",(F10-E10)/E10)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1376,182 +1979,194 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>VEHICULOS</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Declaracion 2025  -  columna 2026 editable</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="5" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Tipo de vehiculo</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Placa</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Valor 2026  (editable)</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>Valor 2026</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>1 - Vehiculo terrestre</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>PBO7092</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>ECU - Ecuador</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D6" s="61" t="n">
         <v>12000</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E6" s="62" t="n">
         <v>12000</v>
       </c>
-      <c r="F4" s="6">
-        <f>E4-D4</f>
-        <v/>
-      </c>
-      <c r="G4" s="7">
-        <f>IF(D4=0,"",(E4-D4)/D4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="F6" s="61">
+        <f>E6-D6</f>
+        <v/>
+      </c>
+      <c r="G6" s="63">
+        <f>IF(D6=0,"",(E6-D6)/D6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>1 - Vehiculo terrestre</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>PBF9690</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>ECU - Ecuador</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D7" s="65" t="n">
         <v>20000</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E7" s="62" t="n">
         <v>20000</v>
       </c>
-      <c r="F5" s="6">
-        <f>E5-D5</f>
-        <v/>
-      </c>
-      <c r="G5" s="7">
-        <f>IF(D5=0,"",(E5-D5)/D5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="F7" s="65">
+        <f>E7-D7</f>
+        <v/>
+      </c>
+      <c r="G7" s="66">
+        <f>IF(D7=0,"",(E7-D7)/D7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>1 - Vehiculo terrestre</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>PFC8683</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>ECU - Ecuador</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D8" s="61" t="n">
         <v>32000</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E8" s="62" t="n">
         <v>32000</v>
       </c>
-      <c r="F6" s="6">
-        <f>E6-D6</f>
-        <v/>
-      </c>
-      <c r="G6" s="7">
-        <f>IF(D6=0,"",(E6-D6)/D6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="F8" s="61">
+        <f>E8-D8</f>
+        <v/>
+      </c>
+      <c r="G8" s="63">
+        <f>IF(D8=0,"",(E8-D8)/D8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="20" t="n"/>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="21">
-        <f>SUM(D4:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="21">
-        <f>SUM(E4:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="21">
-        <f>E7-D7</f>
-        <v/>
-      </c>
-      <c r="G7" s="22">
-        <f>IF(D7=0,"",(E7-D7)/D7)</f>
+      <c r="B9" s="67" t="n"/>
+      <c r="C9" s="67" t="n"/>
+      <c r="D9" s="31">
+        <f>SUM(D6:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="31">
+        <f>SUM(E6:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="31">
+        <f>E9-D9</f>
+        <v/>
+      </c>
+      <c r="G9" s="32">
+        <f>IF(D9=0,"",(E9-D9)/D9)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1564,232 +2179,244 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>BIENES INMUEBLES</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Declaracion 2025  -  columna 2026 editable</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="5" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Tipo de inmueble</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Clave catastral</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Inscripcion</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Valor 2026  (editable)</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>Valor 2026</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>3 - Terreno</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>ECU - Ecuador</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>1042203018</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>22/10/2008</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E6" s="61" t="n">
         <v>267340.8</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F6" s="62" t="n">
         <v>267340.8</v>
       </c>
-      <c r="G4" s="6">
-        <f>F4-E4</f>
-        <v/>
-      </c>
-      <c r="H4" s="7">
-        <f>IF(E4=0,"",(F4-E4)/E4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="G6" s="61">
+        <f>F6-E6</f>
+        <v/>
+      </c>
+      <c r="H6" s="63">
+        <f>IF(E6=0,"",(F6-E6)/E6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>1 - Edificacion / casa</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>ECU - Ecuador</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>1012005008000000000</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D7" s="64" t="inlineStr">
         <is>
           <t>13/03/1997</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E7" s="65" t="n">
         <v>198118.55</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F7" s="62" t="n">
         <v>198118.55</v>
       </c>
-      <c r="G5" s="6">
-        <f>F5-E5</f>
-        <v/>
-      </c>
-      <c r="H5" s="7">
-        <f>IF(E5=0,"",(F5-E5)/E5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="G7" s="65">
+        <f>F7-E7</f>
+        <v/>
+      </c>
+      <c r="H7" s="66">
+        <f>IF(E7=0,"",(F7-E7)/E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>1 - Edificacion / casa</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>ECU - Ecuador</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>1042203018</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr"/>
-      <c r="E6" s="6" t="n">
+      <c r="D8" s="60" t="inlineStr"/>
+      <c r="E8" s="61" t="n">
         <v>33634.04</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F8" s="62" t="n">
         <v>33634.04</v>
       </c>
-      <c r="G6" s="6">
-        <f>F6-E6</f>
-        <v/>
-      </c>
-      <c r="H6" s="7">
-        <f>IF(E6=0,"",(F6-E6)/E6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="G8" s="61">
+        <f>F8-E8</f>
+        <v/>
+      </c>
+      <c r="H8" s="63">
+        <f>IF(E8=0,"",(F8-E8)/E8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="64" t="inlineStr">
         <is>
           <t>3 - Terreno</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B9" s="64" t="inlineStr">
         <is>
           <t>ECU - Ecuador</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C9" s="64" t="inlineStr">
         <is>
           <t>1012005008000000000</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr"/>
-      <c r="E7" s="6" t="n">
+      <c r="D9" s="64" t="inlineStr"/>
+      <c r="E9" s="65" t="n">
         <v>82624.22</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F9" s="62" t="n">
         <v>82624.22</v>
       </c>
-      <c r="G7" s="6">
-        <f>F7-E7</f>
-        <v/>
-      </c>
-      <c r="H7" s="7">
-        <f>IF(E7=0,"",(F7-E7)/E7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="G9" s="65">
+        <f>F9-E9</f>
+        <v/>
+      </c>
+      <c r="H9" s="66">
+        <f>IF(E9=0,"",(F9-E9)/E9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n"/>
-      <c r="C8" s="20" t="n"/>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="21">
-        <f>SUM(E4:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="21">
-        <f>SUM(F4:F7)</f>
-        <v/>
-      </c>
-      <c r="G8" s="21">
-        <f>F8-E8</f>
-        <v/>
-      </c>
-      <c r="H8" s="22">
-        <f>IF(E8=0,"",(F8-E8)/E8)</f>
+      <c r="B10" s="67" t="n"/>
+      <c r="C10" s="67" t="n"/>
+      <c r="D10" s="67" t="n"/>
+      <c r="E10" s="31">
+        <f>SUM(E6:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="31">
+        <f>SUM(F6:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="31">
+        <f>F10-E10</f>
+        <v/>
+      </c>
+      <c r="H10" s="32">
+        <f>IF(E10=0,"",(F10-E10)/E10)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1802,168 +2429,180 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PASIVOS / DEUDAS</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Declaracion 2025  -  columna 2026 editable</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="5" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Tipo de acreedor</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Acreedor</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Domicilio</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Identificacion</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Valor 2026  (editable)</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>Valor 2026</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>IFI - Institucion financiera</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>DINERS CLUB DEL ECUADOR</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>ECU - Ecuador</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>1792260957001</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E6" s="61" t="n">
         <v>4891.88</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F6" s="62" t="n">
         <v>4891.88</v>
       </c>
-      <c r="G4" s="6">
-        <f>F4-E4</f>
-        <v/>
-      </c>
-      <c r="H4" s="7">
-        <f>IF(E4=0,"",(F4-E4)/E4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="G6" s="61">
+        <f>F6-E6</f>
+        <v/>
+      </c>
+      <c r="H6" s="63">
+        <f>IF(E6=0,"",(F6-E6)/E6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>IFI - Institucion financiera</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>BANCO DEL PICHINCHA</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>ECU - Ecuador</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D7" s="64" t="inlineStr">
         <is>
           <t>1790010937001</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E7" s="65" t="n">
         <v>5547.31</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F7" s="62" t="n">
         <v>5547.31</v>
       </c>
-      <c r="G5" s="6">
-        <f>F5-E5</f>
-        <v/>
-      </c>
-      <c r="H5" s="7">
-        <f>IF(E5=0,"",(F5-E5)/E5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="G7" s="65">
+        <f>F7-E7</f>
+        <v/>
+      </c>
+      <c r="H7" s="66">
+        <f>IF(E7=0,"",(F7-E7)/E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="68" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="21">
-        <f>SUM(E4:E5)</f>
-        <v/>
-      </c>
-      <c r="F6" s="21">
-        <f>SUM(F4:F5)</f>
-        <v/>
-      </c>
-      <c r="G6" s="21">
-        <f>F6-E6</f>
-        <v/>
-      </c>
-      <c r="H6" s="22">
-        <f>IF(E6=0,"",(F6-E6)/E6)</f>
+      <c r="B8" s="68" t="n"/>
+      <c r="C8" s="68" t="n"/>
+      <c r="D8" s="68" t="n"/>
+      <c r="E8" s="38">
+        <f>SUM(E6:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="38">
+        <f>SUM(F6:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="38">
+        <f>F8-E8</f>
+        <v/>
+      </c>
+      <c r="H8" s="39">
+        <f>IF(E8=0,"",(F8-E8)/E8)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1976,219 +2615,223 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DATOS GENERALES DE LA DECLARACION</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+    <row r="3" ht="5" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="69" t="inlineStr">
         <is>
           <t>Anio de la declaracion</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B5" s="70" t="n">
         <v>2025</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="69" t="inlineStr">
         <is>
           <t>Tipo de declaracion</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B6" s="70" t="inlineStr">
         <is>
           <t>SOC - Sociedad conyugal</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="69" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B7" s="70" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="69" t="inlineStr">
         <is>
           <t>Numero de identificacion</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B8" s="70" t="inlineStr">
         <is>
           <t>1709164899001</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="69" t="inlineStr">
         <is>
           <t>Nombre del declarante</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B9" s="70" t="inlineStr">
         <is>
           <t>GONZALEZ NAVAS MARCO VINICIO</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="69" t="inlineStr">
         <is>
           <t>Identificacion del conyuge</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B10" s="70" t="inlineStr">
         <is>
           <t>C - Cedula</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="69" t="inlineStr">
         <is>
           <t>Numero ident. conyuge</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B11" s="70" t="inlineStr">
         <is>
           <t>1709784225</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="69" t="inlineStr">
         <is>
           <t>Nombre del conyuge</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B12" s="70" t="inlineStr">
         <is>
           <t>HIDALGO LOZA ROSA CONSUELO</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="69" t="inlineStr">
         <is>
           <t>Total creditos</t>
         </is>
       </c>
-      <c r="B11" s="24" t="n">
+      <c r="B13" s="71" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="23" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="72" t="inlineStr"/>
+      <c r="B14" s="73" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="69" t="inlineStr">
         <is>
           <t>Patrimonio total declarado</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n">
+      <c r="B15" s="71" t="n">
         <v>883285.5600000001</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="69" t="inlineStr">
         <is>
           <t>Atribuible a hijos</t>
         </is>
       </c>
-      <c r="B14" s="24" t="n">
+      <c r="B16" s="71" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="69" t="inlineStr">
         <is>
           <t>Sociedad conyugal</t>
         </is>
       </c>
-      <c r="B15" s="24" t="n">
+      <c r="B17" s="71" t="n">
         <v>883285.5600000001</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="69" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="B16" s="24" t="n">
+      <c r="B18" s="71" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="69" t="inlineStr">
         <is>
           <t>Patrimonio anio anterior</t>
         </is>
       </c>
-      <c r="B17" s="24" t="n">
+      <c r="B19" s="71" t="n">
         <v>801569.97</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="69" t="inlineStr">
         <is>
           <t>Crecimiento patrimonial</t>
         </is>
       </c>
-      <c r="B18" s="24" t="n">
+      <c r="B20" s="71" t="n">
         <v>81715.59</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="74" t="inlineStr">
         <is>
           <t>Justificacion de la variacion patrimonial</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="73" t="inlineStr">
         <is>
           <t>- 1 - Ingresos por trabajo en relacion de dependencia</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="73" t="inlineStr">
         <is>
           <t>- 6 - Otros ingresos / variaciones de mercado</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="59" t="inlineStr">
         <is>
           <t>Nota: las descripciones de codigos son de referencia; verificar contra el catalogo oficial del SRI.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(tools): agrega generador de XML del SRI desde el Excel
Nuevo script generar_xml_sri.py que reconstruye el XML de la Declaracion
Patrimonial a partir del libro Excel lleno, para los modulos con etiquetas
confirmadas (dinero, vehiculos, bienes inmuebles y pasivos) mas cabecera,
patrimonio y justificacion. Las instituciones financieras cuyo codigo no
consta en el catalogo del SRI se dejan en blanco para elegirlas de la lista.

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -9509,11 +9509,7 @@
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr">
-        <is>
-          <t>1029</t>
-        </is>
-      </c>
+      <c r="E6" s="59" t="inlineStr"/>
       <c r="F6" s="59" t="inlineStr">
         <is>
           <t>DOLARES</t>
@@ -9560,11 +9556,7 @@
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E7" s="63" t="inlineStr">
-        <is>
-          <t>1029</t>
-        </is>
-      </c>
+      <c r="E7" s="63" t="inlineStr"/>
       <c r="F7" s="63" t="inlineStr">
         <is>
           <t>DOLARES</t>
@@ -9611,11 +9603,7 @@
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E8" s="59" t="inlineStr">
-        <is>
-          <t>1418</t>
-        </is>
-      </c>
+      <c r="E8" s="59" t="inlineStr"/>
       <c r="F8" s="59" t="inlineStr">
         <is>
           <t>DOLARES</t>

</xml_diff>

<commit_message>
feat(tools): motor VBA y hoja con boton para generar el XML del SRI
Agrega GenerarXmlSRI.bas, una macro VBA que reconstruye el XML de la
Declaracion Patrimonial leyendo las hojas del libro y el mapa de
etiquetas (_Mapa). Incorpora la hoja "Generar XML" con el boton y las
instrucciones de instalacion de la macro, para generar el archivo .xml
con un clic desde Excel.

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -18,8 +18,10 @@
     <sheet name="Otros Activos" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Pasivos" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Justificacion" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Datos del XML" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Catalogos" sheetId="13" state="hidden" r:id="rId13"/>
+    <sheet name="Generar XML" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Datos del XML" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="_Mapa" sheetId="14" state="hidden" r:id="rId14"/>
+    <sheet name="Catalogos" sheetId="15" state="hidden" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +34,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="+0.0%;-0.0%;0.0%"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -119,6 +121,16 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007A7A7A"/>
+      <sz val="8"/>
     </font>
     <font>
       <b val="1"/>
@@ -215,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -425,6 +437,12 @@
     <xf numFmtId="164" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -434,8 +452,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2539,6 +2555,161 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GENERAR XML PARA EL SRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Convierte este libro en el archivo XML de la Declaracion Patrimonial, listo para subir al portal del SRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="5" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="77" t="inlineStr">
+        <is>
+          <t>►   GENERAR XML</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="78" t="inlineStr">
+        <is>
+          <t>Dibuje el boton sobre este recuadro y asignele la macro GenerarXmlSRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="79" t="inlineStr">
+        <is>
+          <t>CONFIGURACION POR UNICA VEZ (activa el boton)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="80" t="inlineStr">
+        <is>
+          <t>1. Abra el editor de macros con la tecla  Alt + F11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="80" t="inlineStr">
+        <is>
+          <t>2. Menu Archivo &gt; Importar archivo... y seleccione el archivo GenerarXmlSRI.bas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="80" t="inlineStr">
+        <is>
+          <t>3. Cierre el editor y guarde este libro como  'Libro de Excel habilitado para macros (*.xlsm)'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="80" t="inlineStr">
+        <is>
+          <t>4. Active la pestana Programador:  Archivo &gt; Opciones &gt; Personalizar cinta de opciones &gt; marque 'Programador'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="80" t="inlineStr">
+        <is>
+          <t>5. Programador &gt; Insertar &gt; Boton (control de formulario) y dibujelo sobre el recuadro verde de arriba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="80" t="inlineStr">
+        <is>
+          <t>6. Cuando Excel lo solicite, asigne la macro  GenerarXmlSRI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="80" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="79" t="inlineStr">
+        <is>
+          <t>USO DIARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="80" t="inlineStr">
+        <is>
+          <t>7. Llene las columnas amarillas de cada modulo y la hoja Justificacion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="80" t="inlineStr">
+        <is>
+          <t>8. Pulse el boton GENERAR XML, indique el anio y elija donde guardar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="80" t="inlineStr">
+        <is>
+          <t>9. El archivo .xml queda listo para subir al portal del SRI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="80" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="80" t="inlineStr">
+        <is>
+          <t>Alternativa sin macros:  ejecutar  python tools/generar_xml_sri.py  desde la terminal.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B5:D6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2557,108 +2728,108 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="77" t="inlineStr">
+      <c r="A5" s="81" t="inlineStr">
         <is>
           <t>IDENTIFICACION</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="78" t="inlineStr">
+      <c r="A6" s="82" t="inlineStr">
         <is>
           <t>Anio de la declaracion</t>
         </is>
       </c>
-      <c r="B6" s="79" t="n">
+      <c r="B6" s="83" t="n">
         <v>2025</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="78" t="inlineStr">
+      <c r="A7" s="82" t="inlineStr">
         <is>
           <t>Tipo de declaracion</t>
         </is>
       </c>
-      <c r="B7" s="79" t="inlineStr">
+      <c r="B7" s="83" t="inlineStr">
         <is>
           <t>SOC - Sociedad conyugal o union de hecho</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="78" t="inlineStr">
+      <c r="A8" s="82" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="B8" s="79" t="inlineStr">
+      <c r="B8" s="83" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="78" t="inlineStr">
+      <c r="A9" s="82" t="inlineStr">
         <is>
           <t>Numero de identificacion</t>
         </is>
       </c>
-      <c r="B9" s="79" t="inlineStr">
+      <c r="B9" s="83" t="inlineStr">
         <is>
           <t>1709164899001</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="78" t="inlineStr">
+      <c r="A10" s="82" t="inlineStr">
         <is>
           <t>Nombre del declarante</t>
         </is>
       </c>
-      <c r="B10" s="79" t="inlineStr">
+      <c r="B10" s="83" t="inlineStr">
         <is>
           <t>GONZALEZ NAVAS MARCO VINICIO</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="78" t="inlineStr">
+      <c r="A11" s="82" t="inlineStr">
         <is>
           <t>Identificacion del conyuge</t>
         </is>
       </c>
-      <c r="B11" s="79" t="inlineStr">
+      <c r="B11" s="83" t="inlineStr">
         <is>
           <t>C - Cedula</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="78" t="inlineStr">
+      <c r="A12" s="82" t="inlineStr">
         <is>
           <t>Numero ident. conyuge</t>
         </is>
       </c>
-      <c r="B12" s="79" t="inlineStr">
+      <c r="B12" s="83" t="inlineStr">
         <is>
           <t>1709784225</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="78" t="inlineStr">
+      <c r="A13" s="82" t="inlineStr">
         <is>
           <t>Nombre del conyuge</t>
         </is>
       </c>
-      <c r="B13" s="79" t="inlineStr">
+      <c r="B13" s="83" t="inlineStr">
         <is>
           <t>HIDALGO LOZA ROSA CONSUELO</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="78" t="inlineStr">
+      <c r="A14" s="82" t="inlineStr">
         <is>
           <t>Total creditos / cuentas por cobrar</t>
         </is>
@@ -2668,14 +2839,14 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="77" t="inlineStr">
+      <c r="A16" s="81" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO (enlazado a la hoja Dashboard)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="78" t="inlineStr">
+      <c r="A17" s="82" t="inlineStr">
         <is>
           <t>Patrimonio neto 2025</t>
         </is>
@@ -2686,7 +2857,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="78" t="inlineStr">
+      <c r="A18" s="82" t="inlineStr">
         <is>
           <t>Patrimonio neto 2026 (proyectado)</t>
         </is>
@@ -2697,7 +2868,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="78" t="inlineStr">
+      <c r="A19" s="82" t="inlineStr">
         <is>
           <t>Variacion proyectada</t>
         </is>
@@ -2708,7 +2879,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="78" t="inlineStr">
+      <c r="A20" s="82" t="inlineStr">
         <is>
           <t>Variacion % proyectada</t>
         </is>
@@ -2719,14 +2890,14 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="77" t="inlineStr">
+      <c r="A22" s="81" t="inlineStr">
         <is>
           <t>PATRIMONIO DECLARADO EN EL XML</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="78" t="inlineStr">
+      <c r="A23" s="82" t="inlineStr">
         <is>
           <t>Patrimonio total declarado</t>
         </is>
@@ -2736,7 +2907,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="78" t="inlineStr">
+      <c r="A24" s="82" t="inlineStr">
         <is>
           <t>Atribuible a hijos no emancipados</t>
         </is>
@@ -2746,7 +2917,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="78" t="inlineStr">
+      <c r="A25" s="82" t="inlineStr">
         <is>
           <t>Patrimonio en la sociedad conyugal</t>
         </is>
@@ -2756,7 +2927,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="78" t="inlineStr">
+      <c r="A26" s="82" t="inlineStr">
         <is>
           <t>Patrimonio individual del declarante</t>
         </is>
@@ -2766,7 +2937,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="78" t="inlineStr">
+      <c r="A27" s="82" t="inlineStr">
         <is>
           <t>Patrimonio del anio anterior</t>
         </is>
@@ -2776,7 +2947,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="78" t="inlineStr">
+      <c r="A28" s="82" t="inlineStr">
         <is>
           <t>Crecimiento / decremento patrimonial</t>
         </is>
@@ -2786,21 +2957,21 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="80" t="inlineStr">
+      <c r="A30" s="79" t="inlineStr">
         <is>
           <t>Justificacion de la variacion (ver hoja Justificacion)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="81" t="inlineStr">
+      <c r="A31" s="80" t="inlineStr">
         <is>
           <t>- 1 - Ingresos locales</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="81" t="inlineStr">
+      <c r="A32" s="80" t="inlineStr">
         <is>
           <t>- 6 - Otros</t>
         </is>
@@ -2825,7 +2996,3250 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hoja</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>contenedor</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>detalle</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>clase</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ordenXml</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>xmlTag</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>descIndex</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>dineroEn</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>tipoInversion</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>pais</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>_ifi</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>tipoMoneda</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>saldo</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>partesRelacionadas</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>regularizacionActivos</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dinero</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>dinero</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>detalleDinero</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>anioFiscalAdquisicion</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>tipoInversion</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>codpais</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>nombempresa</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>porcentpart</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>numAcc</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>relacionadas</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>regularizacionActivos</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>drc</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Derechos de Capital</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>inversiones</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>detalleInversiones</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>anioFiscalAdquisicion</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>nombreDeudor</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>tipoDeudor</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>tipoIdentificacion</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>numeroIdentificacion</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>pais</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>partesRelacionadas</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>saldo</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>regularizacionActivos</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>cxc</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Cuentas por Cobrar</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ctasXCobrar</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>detalleCtasXCobrar</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>anioFiscalAdquisicion</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>muebles</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Bienes Muebles</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>otrosBienes</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>detalleOtrosBienes</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>tipoBien</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>muebles</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Bienes Muebles</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>otrosBienes</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>detalleOtrosBienes</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>4</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>muebles</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Bienes Muebles</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>otrosBienes</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>detalleOtrosBienes</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>4</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>pais</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>muebles</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Bienes Muebles</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>otrosBienes</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>detalleOtrosBienes</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>4</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>muebles</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Bienes Muebles</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>otrosBienes</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>detalleOtrosBienes</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>4</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>regularizacionActivos</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>muebles</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Bienes Muebles</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>otrosBienes</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>detalleOtrosBienes</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>4</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>anioFiscalAdquisicion</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Vehiculos</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>detalleVehiculos</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>3</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>tipoVehiculo</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Vehiculos</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>detalleVehiculos</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>3</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>placa</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Vehiculos</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>detalleVehiculos</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Vehiculos</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>detalleVehiculos</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>pais</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Vehiculos</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>detalleVehiculos</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Vehiculos</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>detalleVehiculos</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>regularizacionActivos</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Vehiculos</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>vehiculos</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>detalleVehiculos</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>3</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>anioFiscalAdquisicion</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Derechos</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>detalleDerechos</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>8</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>tipoDerecho</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Derechos</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>detalleDerechos</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>8</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Derechos</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>detalleDerechos</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>8</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>pais</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Derechos</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>detalleDerechos</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>8</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Derechos</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>detalleDerechos</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>8</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>regularizacionActivos</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Derechos</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>derechos</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>detalleDerechos</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>8</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>anioFiscalAdquisicion</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>5</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>tipoInmueble</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>5</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>5</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>codPais</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>5</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>provincia</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>5</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>canton</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>5</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>fechaInscripcion</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>5</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>claveCat</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>5</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>5</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>regularizacionActivos</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>inmuebles</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Bienes Inmuebles</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>bienesInmuebles</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>detalleBienesInmuebles</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>5</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>anioFiscalAdquisicion</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Otros Activos</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>otrosActivos</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>detalleOtrosActivos</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>7</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Otros Activos</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>otrosActivos</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>detalleOtrosActivos</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>7</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>pais</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Otros Activos</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>otrosActivos</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>detalleOtrosActivos</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>7</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>descripcion</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Otros Activos</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>otrosActivos</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>detalleOtrosActivos</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>7</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>valorTotal</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Otros Activos</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>otrosActivos</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>detalleOtrosActivos</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>7</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>regularizacionActivos</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Otros Activos</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>otrosActivos</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>detalleOtrosActivos</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>7</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>anioFiscalAdquisicion</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>detallePasivo</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>6</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>tipoAcreedor</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>detallePasivo</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>6</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>domicilioAcreedor</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>detallePasivo</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>6</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>valorDeuda</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>detallePasivo</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>6</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>paisAcreedor</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>detallePasivo</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>6</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>nombreAcreedor</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>detallePasivo</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>6</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>tipoIdentificacionAcreedor</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>detallePasivo</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>6</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>numeroIdentificacionAcreedor</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>detallePasivo</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>6</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>txt</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>numeroRegistroBancoCentral</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Pasivos</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>detallePasivo</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>pasivo</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>6</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>cod</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>partesRelacionadas</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2835,97 +6249,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="82" t="inlineStr">
+      <c r="A1" s="84" t="inlineStr">
         <is>
           <t>DINERO_EN</t>
         </is>
       </c>
-      <c r="B1" s="82" t="inlineStr">
+      <c r="B1" s="84" t="inlineStr">
         <is>
           <t>TIPO_INVERSION</t>
         </is>
       </c>
-      <c r="C1" s="82" t="inlineStr">
+      <c r="C1" s="84" t="inlineStr">
         <is>
           <t>UBICACION</t>
         </is>
       </c>
-      <c r="D1" s="82" t="inlineStr">
+      <c r="D1" s="84" t="inlineStr">
         <is>
           <t>PAIS</t>
         </is>
       </c>
-      <c r="E1" s="82" t="inlineStr">
+      <c r="E1" s="84" t="inlineStr">
         <is>
           <t>INSTITUCION_FINANCIERA</t>
         </is>
       </c>
-      <c r="F1" s="82" t="inlineStr">
+      <c r="F1" s="84" t="inlineStr">
         <is>
           <t>PARTES_RELACIONADAS</t>
         </is>
       </c>
-      <c r="G1" s="82" t="inlineStr">
+      <c r="G1" s="84" t="inlineStr">
         <is>
           <t>TIPO_DRC</t>
         </is>
       </c>
-      <c r="H1" s="82" t="inlineStr">
+      <c r="H1" s="84" t="inlineStr">
         <is>
           <t>TIPO_PERSONA</t>
         </is>
       </c>
-      <c r="I1" s="82" t="inlineStr">
+      <c r="I1" s="84" t="inlineStr">
         <is>
           <t>TIPO_BIEN_MUEBLE</t>
         </is>
       </c>
-      <c r="J1" s="82" t="inlineStr">
+      <c r="J1" s="84" t="inlineStr">
         <is>
           <t>TIPO_VEHICULO</t>
         </is>
       </c>
-      <c r="K1" s="82" t="inlineStr">
+      <c r="K1" s="84" t="inlineStr">
         <is>
           <t>TIPO_DERECHO</t>
         </is>
       </c>
-      <c r="L1" s="82" t="inlineStr">
+      <c r="L1" s="84" t="inlineStr">
         <is>
           <t>TIPO_INMUEBLE</t>
         </is>
       </c>
-      <c r="M1" s="82" t="inlineStr">
+      <c r="M1" s="84" t="inlineStr">
         <is>
           <t>PROVINCIA</t>
         </is>
       </c>
-      <c r="N1" s="82" t="inlineStr">
+      <c r="N1" s="84" t="inlineStr">
         <is>
           <t>CANTON</t>
         </is>
       </c>
-      <c r="O1" s="82" t="inlineStr">
+      <c r="O1" s="84" t="inlineStr">
         <is>
           <t>TIPO_ACREEDOR</t>
         </is>
       </c>
-      <c r="P1" s="82" t="inlineStr">
+      <c r="P1" s="84" t="inlineStr">
         <is>
           <t>TIPO_IDENTIFICACION</t>
         </is>
       </c>
-      <c r="Q1" s="82" t="inlineStr">
+      <c r="Q1" s="84" t="inlineStr">
         <is>
           <t>REGULARIZACION</t>
         </is>
       </c>
-      <c r="R1" s="82" t="inlineStr">
+      <c r="R1" s="84" t="inlineStr">
         <is>
           <t>JUSTIF_INCREMENTO</t>
         </is>
       </c>
-      <c r="S1" s="82" t="inlineStr">
+      <c r="S1" s="84" t="inlineStr">
         <is>
           <t>JUSTIF_DECREMENTO</t>
         </is>

</xml_diff>

<commit_message>
feat(tools): genera el .xlsm con la macro VBA y el boton embebidos
Agrega _xlsm_builder.py, que arma un vbaProject.bin (contenedor OLE +
compresion MS-OVBA) con la macro GenerarXmlSRI y lo empaqueta en un
.xlsm junto con un boton (forma DrawingML vinculada a la macro) en la
hoja "Generar XML". El generador produce ahora tanto el .xlsx como el
.xlsm listo para usar con un clic.

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -2555,7 +2555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2599,95 +2599,81 @@
     <row r="7">
       <c r="B7" s="78" t="inlineStr">
         <is>
-          <t>Dibuje el boton sobre este recuadro y asignele la macro GenerarXmlSRI</t>
+          <t>En el archivo .xlsm el boton verde ya esta vinculado a la macro GenerarXmlSRI.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="79" t="inlineStr">
         <is>
-          <t>CONFIGURACION POR UNICA VEZ (activa el boton)</t>
+          <t>COMO USAR ESTE ARCHIVO</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="80" t="inlineStr">
         <is>
-          <t>1. Abra el editor de macros con la tecla  Alt + F11.</t>
+          <t>1. Al abrir el archivo .xlsm, pulse 'Habilitar contenido' en la barra de seguridad de Excel.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="80" t="inlineStr">
         <is>
-          <t>2. Menu Archivo &gt; Importar archivo... y seleccione el archivo GenerarXmlSRI.bas.</t>
+          <t>2. Llene las columnas amarillas de cada modulo (Dinero, Vehiculos, etc.) y la hoja Justificacion.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="80" t="inlineStr">
         <is>
-          <t>3. Cierre el editor y guarde este libro como  'Libro de Excel habilitado para macros (*.xlsm)'.</t>
+          <t>3. Pulse el boton verde GENERAR XML, indique el anio y elija donde guardar el archivo.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="80" t="inlineStr">
         <is>
-          <t>4. Active la pestana Programador:  Archivo &gt; Opciones &gt; Personalizar cinta de opciones &gt; marque 'Programador'.</t>
+          <t>4. El archivo .xml queda listo para subir al portal del SRI.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="80" t="inlineStr">
-        <is>
-          <t>5. Programador &gt; Insertar &gt; Boton (control de formulario) y dibujelo sobre el recuadro verde de arriba.</t>
-        </is>
-      </c>
+      <c r="B14" s="80" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="80" t="inlineStr">
-        <is>
-          <t>6. Cuando Excel lo solicite, asigne la macro  GenerarXmlSRI.</t>
+      <c r="B15" s="79" t="inlineStr">
+        <is>
+          <t>SI EXCEL BLOQUEA LAS MACROS</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="80" t="inlineStr"/>
+      <c r="B16" s="80" t="inlineStr">
+        <is>
+          <t>- Cierre Excel. En el Explorador, clic derecho sobre el archivo &gt; Propiedades.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="B17" s="79" t="inlineStr">
-        <is>
-          <t>USO DIARIO</t>
+      <c r="B17" s="80" t="inlineStr">
+        <is>
+          <t>- Al final de la pestana General marque 'Desbloquear' y pulse Aceptar.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="80" t="inlineStr">
         <is>
-          <t>7. Llene las columnas amarillas de cada modulo y la hoja Justificacion.</t>
+          <t>- Vuelva a abrirlo y pulse 'Habilitar contenido'. Conserve siempre la extension .xlsm.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="80" t="inlineStr">
-        <is>
-          <t>8. Pulse el boton GENERAR XML, indique el anio y elija donde guardar.</t>
-        </is>
-      </c>
+      <c r="B19" s="80" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="B20" s="80" t="inlineStr">
-        <is>
-          <t>9. El archivo .xml queda listo para subir al portal del SRI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="80" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="80" t="inlineStr">
         <is>
           <t>Alternativa sin macros:  ejecutar  python tools/generar_xml_sri.py  desde la terminal.</t>
         </is>

</xml_diff>

<commit_message>
fix(tools): desbloquea el proyecto VBA y rehace la hoja Justificacion
Quita CMG/DPB/GC del PROJECT stream para que el proyecto VBA quede
visible y se puedan asignar las macros. Rehace la hoja Justificacion
como lista de seleccion Si/No de los 6 conceptos de la Tabla 14, igual
que el formulario del SRI; el generador de XML y la macro toman los
conceptos marcados con 'Si'.

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -34,7 +34,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="+0.0%;-0.0%;0.0%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -122,10 +122,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
@@ -232,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -423,18 +419,6 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -442,17 +426,14 @@
     <xf numFmtId="164" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -647,144 +628,6 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Distribucion del incremento patrimonial</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <pieChart>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Justificacion'!$B$12:$B$13</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Justificacion'!$E$12:$E$13</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showPercent val="1"/>
-        </dLbls>
-        <firstSliceAng val="0"/>
-      </pieChart>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Monto asignado por concepto</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Justificacion'!E11</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Justificacion'!$B$12:$B$13</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Justificacion'!$E$12:$E$13</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -804,55 +647,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>8</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5400000" cy="3240000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>8</col>
-      <colOff>0</colOff>
-      <row>22</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5400000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2175,16 +1969,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2197,208 +1989,148 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Conceptos declarados en el XML  -  ejercicio 2025  (catalogo Tabla 14 del SRI)</t>
+          <t>Marque 'Si' los conceptos que justifican la variacion patrimonial  -  ejercicio 2025</t>
         </is>
       </c>
     </row>
     <row r="3" ht="5" customHeight="1">
       <c r="A3" s="3" t="n"/>
     </row>
-    <row r="5" ht="6" customHeight="1">
-      <c r="B5" s="9" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="6" t="n"/>
-    </row>
-    <row r="6">
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>INCREMENTO PATRIMONIAL</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="n"/>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL JUSTIFICADO</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>DIFERENCIA</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="n"/>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="18">
-        <f>E15</f>
-        <v/>
-      </c>
-      <c r="C7" s="15" t="n"/>
-      <c r="D7" s="16">
-        <f>E14</f>
-        <v/>
-      </c>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="17">
-        <f>E16</f>
-        <v/>
-      </c>
-      <c r="G7" s="13" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="23" t="inlineStr">
-        <is>
-          <t>Declarado en el XML 2025</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="n"/>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>Suma de montos asignados</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="21" t="inlineStr">
-        <is>
-          <t>Debe quedar en $0.00</t>
-        </is>
-      </c>
-      <c r="G8" s="13" t="n"/>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="70" t="inlineStr">
+        <is>
+          <t>Incremento patrimonial declarado en el XML</t>
+        </is>
+      </c>
+      <c r="C5" s="71" t="n"/>
+      <c r="D5" s="71" t="n"/>
+      <c r="E5" s="72" t="n">
+        <v>81715.59</v>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Concepto (Tabla 14 del SRI)</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Justifica la variacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="73" t="inlineStr">
+        <is>
+          <t>1 - Ingresos locales</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="73" t="inlineStr">
+        <is>
+          <t>2 - Ingresos exterior</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="50" t="inlineStr">
-        <is>
-          <t>DISTRIBUCION DEL INCREMENTO PATRIMONIAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="27" t="inlineStr">
-        <is>
-          <t>Concepto declarado (Tabla del SRI)</t>
-        </is>
-      </c>
-      <c r="E11" s="27" t="inlineStr">
-        <is>
-          <t>Monto asignado</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="inlineStr">
-        <is>
-          <t>% del total</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="70" t="inlineStr">
-        <is>
-          <t>1 - Ingresos locales</t>
-        </is>
-      </c>
-      <c r="E12" s="63" t="n">
-        <v>40857.79</v>
-      </c>
-      <c r="F12" s="64">
-        <f>IF($E$14=0,"",E12/$E$14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="70" t="inlineStr">
+      <c r="B10" s="73" t="inlineStr">
+        <is>
+          <t>3 - Herencias, legados o donaciones</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="73" t="inlineStr">
+        <is>
+          <t>4 - Loterias o rifas</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="73" t="inlineStr">
+        <is>
+          <t>5 - Ganancias de capital</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="73" t="inlineStr">
         <is>
           <t>6 - Otros</t>
         </is>
       </c>
-      <c r="E13" s="63" t="n">
-        <v>40857.79</v>
-      </c>
-      <c r="F13" s="64">
-        <f>IF($E$14=0,"",E13/$E$14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="71" t="inlineStr">
-        <is>
-          <t>TOTAL JUSTIFICADO</t>
-        </is>
-      </c>
-      <c r="E14" s="72">
-        <f>SUM(E12:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="73">
-        <f>IF(E14=0,"",1)</f>
-        <v/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="74" t="inlineStr">
-        <is>
-          <t>Incremento patrimonial declarado (XML)</t>
-        </is>
-      </c>
-      <c r="C15" s="75" t="n"/>
-      <c r="D15" s="75" t="n"/>
-      <c r="E15" s="76" t="n">
-        <v>81715.59</v>
-      </c>
-      <c r="F15" s="75" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="77" t="inlineStr">
-        <is>
-          <t>Diferencia por justificar (debe ser $0.00)</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="78">
-        <f>E15-E14</f>
-        <v/>
-      </c>
-      <c r="F16" s="15" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="60" t="inlineStr">
-        <is>
-          <t>Escoja el concepto en la lista desplegable (catalogo del SRI) y asigne el monto en la columna amarilla.</t>
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>Esta hoja reproduce la seccion Justificacion del formulario del SRI. Marque 'Si' en los conceptos que apliquen; el generador de XML los toma de aqui.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="11">
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
     <mergeCell ref="B13:D13"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="B10:G10"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:E1"/>
     <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B12:B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Catalogos!$R$2:$R$7</formula1>
+    <dataValidation sqref="E8:E13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Si,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2436,7 +2168,7 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="79" t="inlineStr">
+      <c r="B5" s="74" t="inlineStr">
         <is>
           <t>►   GENERAR XML</t>
         </is>
@@ -2450,83 +2182,83 @@
       <c r="D6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="80" t="inlineStr">
+      <c r="B7" s="75" t="inlineStr">
         <is>
           <t>En el archivo .xlsm el boton verde ya esta vinculado a la macro GenerarXmlSRI.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="81" t="inlineStr">
+      <c r="B9" s="76" t="inlineStr">
         <is>
           <t>COMO USAR ESTE ARCHIVO</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="82" t="inlineStr">
+      <c r="B10" s="77" t="inlineStr">
         <is>
           <t>1. Al abrir el archivo .xlsm, pulse 'Habilitar contenido' en la barra de seguridad de Excel.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="82" t="inlineStr">
+      <c r="B11" s="77" t="inlineStr">
         <is>
           <t>2. Llene las columnas amarillas de cada modulo (Dinero, Vehiculos, etc.) y la hoja Justificacion.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="82" t="inlineStr">
+      <c r="B12" s="77" t="inlineStr">
         <is>
           <t>3. Pulse el boton verde GENERAR XML, indique el anio y elija donde guardar el archivo.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="82" t="inlineStr">
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>4. El archivo .xml queda listo para subir al portal del SRI.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="82" t="inlineStr"/>
+      <c r="B14" s="77" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="81" t="inlineStr">
+      <c r="B15" s="76" t="inlineStr">
         <is>
           <t>SI EXCEL BLOQUEA LAS MACROS</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="82" t="inlineStr">
+      <c r="B16" s="77" t="inlineStr">
         <is>
           <t>- Cierre Excel. En el Explorador, clic derecho sobre el archivo &gt; Propiedades.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="82" t="inlineStr">
+      <c r="B17" s="77" t="inlineStr">
         <is>
           <t>- Al final de la pestana General marque 'Desbloquear' y pulse Aceptar.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="82" t="inlineStr">
+      <c r="B18" s="77" t="inlineStr">
         <is>
           <t>- Vuelva a abrirlo y pulse 'Habilitar contenido'. Conserve siempre la extension .xlsm.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="82" t="inlineStr"/>
+      <c r="B19" s="77" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="B20" s="82" t="inlineStr">
+      <c r="B20" s="77" t="inlineStr">
         <is>
           <t>Alternativa sin macros:  ejecutar  python tools/generar_xml_sri.py  desde la terminal.</t>
         </is>
@@ -2567,108 +2299,108 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="83" t="inlineStr">
+      <c r="A5" s="78" t="inlineStr">
         <is>
           <t>IDENTIFICACION</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="84" t="inlineStr">
+      <c r="A6" s="79" t="inlineStr">
         <is>
           <t>Anio de la declaracion</t>
         </is>
       </c>
-      <c r="B6" s="85" t="n">
+      <c r="B6" s="80" t="n">
         <v>2025</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="84" t="inlineStr">
+      <c r="A7" s="79" t="inlineStr">
         <is>
           <t>Tipo de declaracion</t>
         </is>
       </c>
-      <c r="B7" s="85" t="inlineStr">
+      <c r="B7" s="80" t="inlineStr">
         <is>
           <t>SOC - Sociedad conyugal o union de hecho</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="84" t="inlineStr">
+      <c r="A8" s="79" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="B8" s="85" t="inlineStr">
+      <c r="B8" s="80" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="84" t="inlineStr">
+      <c r="A9" s="79" t="inlineStr">
         <is>
           <t>Numero de identificacion</t>
         </is>
       </c>
-      <c r="B9" s="85" t="inlineStr">
+      <c r="B9" s="80" t="inlineStr">
         <is>
           <t>1709164899001</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="84" t="inlineStr">
+      <c r="A10" s="79" t="inlineStr">
         <is>
           <t>Nombre del declarante</t>
         </is>
       </c>
-      <c r="B10" s="85" t="inlineStr">
+      <c r="B10" s="80" t="inlineStr">
         <is>
           <t>GONZALEZ NAVAS MARCO VINICIO</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="84" t="inlineStr">
+      <c r="A11" s="79" t="inlineStr">
         <is>
           <t>Identificacion del conyuge</t>
         </is>
       </c>
-      <c r="B11" s="85" t="inlineStr">
+      <c r="B11" s="80" t="inlineStr">
         <is>
           <t>C - Cedula</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="84" t="inlineStr">
+      <c r="A12" s="79" t="inlineStr">
         <is>
           <t>Numero ident. conyuge</t>
         </is>
       </c>
-      <c r="B12" s="85" t="inlineStr">
+      <c r="B12" s="80" t="inlineStr">
         <is>
           <t>1709784225</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="84" t="inlineStr">
+      <c r="A13" s="79" t="inlineStr">
         <is>
           <t>Nombre del conyuge</t>
         </is>
       </c>
-      <c r="B13" s="85" t="inlineStr">
+      <c r="B13" s="80" t="inlineStr">
         <is>
           <t>HIDALGO LOZA ROSA CONSUELO</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="84" t="inlineStr">
+      <c r="A14" s="79" t="inlineStr">
         <is>
           <t>Total creditos / cuentas por cobrar</t>
         </is>
@@ -2678,14 +2410,14 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="83" t="inlineStr">
+      <c r="A16" s="78" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO (enlazado a la hoja Dashboard)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="84" t="inlineStr">
+      <c r="A17" s="79" t="inlineStr">
         <is>
           <t>Patrimonio neto 2025</t>
         </is>
@@ -2696,7 +2428,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="84" t="inlineStr">
+      <c r="A18" s="79" t="inlineStr">
         <is>
           <t>Patrimonio neto 2026 (proyectado)</t>
         </is>
@@ -2707,7 +2439,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="84" t="inlineStr">
+      <c r="A19" s="79" t="inlineStr">
         <is>
           <t>Variacion proyectada</t>
         </is>
@@ -2718,7 +2450,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="84" t="inlineStr">
+      <c r="A20" s="79" t="inlineStr">
         <is>
           <t>Variacion % proyectada</t>
         </is>
@@ -2729,14 +2461,14 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="83" t="inlineStr">
+      <c r="A22" s="78" t="inlineStr">
         <is>
           <t>PATRIMONIO DECLARADO EN EL XML</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="84" t="inlineStr">
+      <c r="A23" s="79" t="inlineStr">
         <is>
           <t>Patrimonio total declarado</t>
         </is>
@@ -2746,7 +2478,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="84" t="inlineStr">
+      <c r="A24" s="79" t="inlineStr">
         <is>
           <t>Atribuible a hijos no emancipados</t>
         </is>
@@ -2756,7 +2488,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="84" t="inlineStr">
+      <c r="A25" s="79" t="inlineStr">
         <is>
           <t>Patrimonio en la sociedad conyugal</t>
         </is>
@@ -2766,7 +2498,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="84" t="inlineStr">
+      <c r="A26" s="79" t="inlineStr">
         <is>
           <t>Patrimonio individual del declarante</t>
         </is>
@@ -2776,7 +2508,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="84" t="inlineStr">
+      <c r="A27" s="79" t="inlineStr">
         <is>
           <t>Patrimonio del anio anterior</t>
         </is>
@@ -2786,7 +2518,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="84" t="inlineStr">
+      <c r="A28" s="79" t="inlineStr">
         <is>
           <t>Crecimiento / decremento patrimonial</t>
         </is>
@@ -2796,21 +2528,21 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="81" t="inlineStr">
+      <c r="A30" s="76" t="inlineStr">
         <is>
           <t>Justificacion de la variacion (ver hoja Justificacion)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="82" t="inlineStr">
+      <c r="A31" s="77" t="inlineStr">
         <is>
           <t>- 1 - Ingresos locales</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="82" t="inlineStr">
+      <c r="A32" s="77" t="inlineStr">
         <is>
           <t>- 6 - Otros</t>
         </is>
@@ -6088,97 +5820,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="86" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>DINERO_EN</t>
         </is>
       </c>
-      <c r="B1" s="86" t="inlineStr">
+      <c r="B1" s="81" t="inlineStr">
         <is>
           <t>TIPO_INVERSION</t>
         </is>
       </c>
-      <c r="C1" s="86" t="inlineStr">
+      <c r="C1" s="81" t="inlineStr">
         <is>
           <t>UBICACION</t>
         </is>
       </c>
-      <c r="D1" s="86" t="inlineStr">
+      <c r="D1" s="81" t="inlineStr">
         <is>
           <t>PAIS</t>
         </is>
       </c>
-      <c r="E1" s="86" t="inlineStr">
+      <c r="E1" s="81" t="inlineStr">
         <is>
           <t>INSTITUCION_FINANCIERA</t>
         </is>
       </c>
-      <c r="F1" s="86" t="inlineStr">
+      <c r="F1" s="81" t="inlineStr">
         <is>
           <t>PARTES_RELACIONADAS</t>
         </is>
       </c>
-      <c r="G1" s="86" t="inlineStr">
+      <c r="G1" s="81" t="inlineStr">
         <is>
           <t>TIPO_DRC</t>
         </is>
       </c>
-      <c r="H1" s="86" t="inlineStr">
+      <c r="H1" s="81" t="inlineStr">
         <is>
           <t>TIPO_PERSONA</t>
         </is>
       </c>
-      <c r="I1" s="86" t="inlineStr">
+      <c r="I1" s="81" t="inlineStr">
         <is>
           <t>TIPO_BIEN_MUEBLE</t>
         </is>
       </c>
-      <c r="J1" s="86" t="inlineStr">
+      <c r="J1" s="81" t="inlineStr">
         <is>
           <t>TIPO_VEHICULO</t>
         </is>
       </c>
-      <c r="K1" s="86" t="inlineStr">
+      <c r="K1" s="81" t="inlineStr">
         <is>
           <t>TIPO_DERECHO</t>
         </is>
       </c>
-      <c r="L1" s="86" t="inlineStr">
+      <c r="L1" s="81" t="inlineStr">
         <is>
           <t>TIPO_INMUEBLE</t>
         </is>
       </c>
-      <c r="M1" s="86" t="inlineStr">
+      <c r="M1" s="81" t="inlineStr">
         <is>
           <t>PROVINCIA</t>
         </is>
       </c>
-      <c r="N1" s="86" t="inlineStr">
+      <c r="N1" s="81" t="inlineStr">
         <is>
           <t>CANTON</t>
         </is>
       </c>
-      <c r="O1" s="86" t="inlineStr">
+      <c r="O1" s="81" t="inlineStr">
         <is>
           <t>TIPO_ACREEDOR</t>
         </is>
       </c>
-      <c r="P1" s="86" t="inlineStr">
+      <c r="P1" s="81" t="inlineStr">
         <is>
           <t>TIPO_IDENTIFICACION</t>
         </is>
       </c>
-      <c r="Q1" s="86" t="inlineStr">
+      <c r="Q1" s="81" t="inlineStr">
         <is>
           <t>REGULARIZACION</t>
         </is>
       </c>
-      <c r="R1" s="86" t="inlineStr">
+      <c r="R1" s="81" t="inlineStr">
         <is>
           <t>JUSTIF_INCREMENTO</t>
         </is>
       </c>
-      <c r="S1" s="86" t="inlineStr">
+      <c r="S1" s="81" t="inlineStr">
         <is>
           <t>JUSTIF_DECREMENTO</t>
         </is>

</xml_diff>

<commit_message>
fix(tools): Dashboard con dos graficos fijos sin macro
Reemplaza el selector de grafico (que requeria macro) por dos graficos
estaticos en el Dashboard: barras con la concentracion de los activos y
un circular con la composicion de activos, pasivos y patrimonio. Quita
la macro CambiarGrafico y el boton APLICAR GRAFICO.

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -34,7 +34,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="+0.0%;-0.0%;0.0%"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,11 +116,6 @@
     <font>
       <b val="1"/>
       <color rgb="0020507D"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -228,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -237,14 +232,8 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -429,11 +418,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -534,7 +526,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Activos / Pasivos / Patrimonio: 2025 vs 2026</a:t>
+              <a:t>Concentracion de activos: 2025 vs 2026</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -549,7 +541,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!D37</f>
+              <f>'Dashboard'!D11</f>
             </strRef>
           </tx>
           <spPr>
@@ -559,12 +551,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$B$38:$B$40</f>
+              <f>'Dashboard'!$B$12:$B$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$D$38:$D$40</f>
+              <f>'Dashboard'!$D$12:$D$19</f>
             </numRef>
           </val>
         </ser>
@@ -573,7 +565,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!E37</f>
+              <f>'Dashboard'!E11</f>
             </strRef>
           </tx>
           <spPr>
@@ -583,12 +575,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$B$38:$B$40</f>
+              <f>'Dashboard'!$B$12:$B$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$E$38:$E$40</f>
+              <f>'Dashboard'!$E$12:$E$19</f>
             </numRef>
           </val>
         </ser>
@@ -628,16 +620,71 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Composicion: activos, pasivos y patrimonio</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$B$38:$B$40</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$D$38:$D$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showPercent val="1"/>
+        </dLbls>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="4320000"/>
+    <ext cx="6840000" cy="3420000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -647,6 +694,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="3420000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -944,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -955,10 +1024,6 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="3" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -977,676 +1042,663 @@
     </row>
     <row r="3" ht="5" customHeight="1">
       <c r="A3" s="3" t="n"/>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>TIPO DE GRAFICO</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>Columnas</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="n"/>
     </row>
     <row r="5" ht="6" customHeight="1">
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="6" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>TOTAL ACTIVOS</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>TOTAL PASIVOS</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO</t>
         </is>
       </c>
-      <c r="G6" s="15" t="n"/>
+      <c r="G6" s="13" t="n"/>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="16">
+      <c r="B7" s="14">
         <f>D20</f>
         <v/>
       </c>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="17">
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="15">
         <f>D25</f>
         <v/>
       </c>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="18">
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="16">
         <f>D31</f>
         <v/>
       </c>
-      <c r="G7" s="15" t="n"/>
+      <c r="G7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Var. proyectada</t>
         </is>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="18">
         <f>G20</f>
         <v/>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>Var. proyectada</t>
         </is>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="20">
         <f>G25</f>
         <v/>
       </c>
-      <c r="F8" s="23" t="inlineStr">
+      <c r="F8" s="21" t="inlineStr">
         <is>
           <t>Var. proyectada</t>
         </is>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="22">
         <f>G31</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="25" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>ACTIVOS</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C11" s="26" t="n"/>
-      <c r="D11" s="27" t="inlineStr">
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="25" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="E11" s="27" t="inlineStr">
+      <c r="E11" s="25" t="inlineStr">
         <is>
           <t>Total 2026</t>
         </is>
       </c>
-      <c r="F11" s="27" t="inlineStr">
+      <c r="F11" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="G11" s="27" t="inlineStr">
+      <c r="G11" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Dinero e inversiones</t>
         </is>
       </c>
-      <c r="D12" s="29">
+      <c r="D12" s="27">
         <f>'Dinero'!J10</f>
         <v/>
       </c>
-      <c r="E12" s="29">
+      <c r="E12" s="27">
         <f>'Dinero'!K10</f>
         <v/>
       </c>
-      <c r="F12" s="29">
+      <c r="F12" s="27">
         <f>E12-D12</f>
         <v/>
       </c>
-      <c r="G12" s="30">
+      <c r="G12" s="28">
         <f>IF(D12=0,"",(E12-D12)/D12)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>Derechos representativos de capital</t>
         </is>
       </c>
-      <c r="D13" s="29">
+      <c r="D13" s="27">
         <f>'Derechos de Capital'!J14</f>
         <v/>
       </c>
-      <c r="E13" s="29">
+      <c r="E13" s="27">
         <f>'Derechos de Capital'!K14</f>
         <v/>
       </c>
-      <c r="F13" s="29">
+      <c r="F13" s="27">
         <f>E13-D13</f>
         <v/>
       </c>
-      <c r="G13" s="30">
+      <c r="G13" s="28">
         <f>IF(D13=0,"",(E13-D13)/D13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>Cuentas por cobrar</t>
         </is>
       </c>
-      <c r="D14" s="29">
+      <c r="D14" s="27">
         <f>'Cuentas por Cobrar'!J14</f>
         <v/>
       </c>
-      <c r="E14" s="29">
+      <c r="E14" s="27">
         <f>'Cuentas por Cobrar'!K14</f>
         <v/>
       </c>
-      <c r="F14" s="29">
+      <c r="F14" s="27">
         <f>E14-D14</f>
         <v/>
       </c>
-      <c r="G14" s="30">
+      <c r="G14" s="28">
         <f>IF(D14=0,"",(E14-D14)/D14)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>Bienes muebles</t>
         </is>
       </c>
-      <c r="D15" s="29">
+      <c r="D15" s="27">
         <f>'Bienes Muebles'!F14</f>
         <v/>
       </c>
-      <c r="E15" s="29">
+      <c r="E15" s="27">
         <f>'Bienes Muebles'!G14</f>
         <v/>
       </c>
-      <c r="F15" s="29">
+      <c r="F15" s="27">
         <f>E15-D15</f>
         <v/>
       </c>
-      <c r="G15" s="30">
+      <c r="G15" s="28">
         <f>IF(D15=0,"",(E15-D15)/D15)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>Vehiculos, naves y aeronaves</t>
         </is>
       </c>
-      <c r="D16" s="29">
+      <c r="D16" s="27">
         <f>'Vehiculos'!G9</f>
         <v/>
       </c>
-      <c r="E16" s="29">
+      <c r="E16" s="27">
         <f>'Vehiculos'!H9</f>
         <v/>
       </c>
-      <c r="F16" s="29">
+      <c r="F16" s="27">
         <f>E16-D16</f>
         <v/>
       </c>
-      <c r="G16" s="30">
+      <c r="G16" s="28">
         <f>IF(D16=0,"",(E16-D16)/D16)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>Derechos (usufructo, uso, etc.)</t>
         </is>
       </c>
-      <c r="D17" s="29">
+      <c r="D17" s="27">
         <f>'Derechos'!F14</f>
         <v/>
       </c>
-      <c r="E17" s="29">
+      <c r="E17" s="27">
         <f>'Derechos'!G14</f>
         <v/>
       </c>
-      <c r="F17" s="29">
+      <c r="F17" s="27">
         <f>E17-D17</f>
         <v/>
       </c>
-      <c r="G17" s="30">
+      <c r="G17" s="28">
         <f>IF(D17=0,"",(E17-D17)/D17)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="26" t="inlineStr">
         <is>
           <t>Bienes inmuebles</t>
         </is>
       </c>
-      <c r="D18" s="29">
+      <c r="D18" s="27">
         <f>'Bienes Inmuebles'!J10</f>
         <v/>
       </c>
-      <c r="E18" s="29">
+      <c r="E18" s="27">
         <f>'Bienes Inmuebles'!K10</f>
         <v/>
       </c>
-      <c r="F18" s="29">
+      <c r="F18" s="27">
         <f>E18-D18</f>
         <v/>
       </c>
-      <c r="G18" s="30">
+      <c r="G18" s="28">
         <f>IF(D18=0,"",(E18-D18)/D18)</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="28" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>Otros activos</t>
         </is>
       </c>
-      <c r="D19" s="29">
+      <c r="D19" s="27">
         <f>'Otros Activos'!F14</f>
         <v/>
       </c>
-      <c r="E19" s="29">
+      <c r="E19" s="27">
         <f>'Otros Activos'!G14</f>
         <v/>
       </c>
-      <c r="F19" s="29">
+      <c r="F19" s="27">
         <f>E19-D19</f>
         <v/>
       </c>
-      <c r="G19" s="30">
+      <c r="G19" s="28">
         <f>IF(D19=0,"",(E19-D19)/D19)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="31" t="inlineStr">
+      <c r="B20" s="29" t="inlineStr">
         <is>
           <t>TOTAL ACTIVOS</t>
         </is>
       </c>
-      <c r="D20" s="32">
+      <c r="D20" s="30">
         <f>SUM(D12:D19)</f>
         <v/>
       </c>
-      <c r="E20" s="32">
+      <c r="E20" s="30">
         <f>SUM(E12:E19)</f>
         <v/>
       </c>
-      <c r="F20" s="32">
+      <c r="F20" s="30">
         <f>E20-D20</f>
         <v/>
       </c>
-      <c r="G20" s="33">
+      <c r="G20" s="31">
         <f>IF(D20=0,"",(E20-D20)/D20)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="34" t="inlineStr">
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>PASIVOS</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="B23" s="26" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C23" s="26" t="n"/>
-      <c r="D23" s="27" t="inlineStr">
+      <c r="C23" s="24" t="n"/>
+      <c r="D23" s="25" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="E23" s="27" t="inlineStr">
+      <c r="E23" s="25" t="inlineStr">
         <is>
           <t>Total 2026</t>
         </is>
       </c>
-      <c r="F23" s="27" t="inlineStr">
+      <c r="F23" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="G23" s="27" t="inlineStr">
+      <c r="G23" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="35" t="inlineStr">
+      <c r="B24" s="33" t="inlineStr">
         <is>
           <t>Deudas y obligaciones</t>
         </is>
       </c>
-      <c r="D24" s="36">
+      <c r="D24" s="34">
         <f>'Pasivos'!I8</f>
         <v/>
       </c>
-      <c r="E24" s="36">
+      <c r="E24" s="34">
         <f>'Pasivos'!J8</f>
         <v/>
       </c>
-      <c r="F24" s="36">
+      <c r="F24" s="34">
         <f>E24-D24</f>
         <v/>
       </c>
-      <c r="G24" s="37">
+      <c r="G24" s="35">
         <f>IF(D24=0,"",(E24-D24)/D24)</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="38" t="inlineStr">
+      <c r="B25" s="36" t="inlineStr">
         <is>
           <t>TOTAL PASIVOS</t>
         </is>
       </c>
-      <c r="D25" s="39">
+      <c r="D25" s="37">
         <f>SUM(D24:D24)</f>
         <v/>
       </c>
-      <c r="E25" s="39">
+      <c r="E25" s="37">
         <f>SUM(E24:E24)</f>
         <v/>
       </c>
-      <c r="F25" s="39">
+      <c r="F25" s="37">
         <f>E25-D25</f>
         <v/>
       </c>
-      <c r="G25" s="40">
+      <c r="G25" s="38">
         <f>IF(D25=0,"",(E25-D25)/D25)</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="41" t="inlineStr">
+      <c r="B27" s="39" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
-      <c r="B28" s="26" t="inlineStr">
+      <c r="B28" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C28" s="26" t="n"/>
-      <c r="D28" s="27" t="inlineStr">
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="25" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="E28" s="27" t="inlineStr">
+      <c r="E28" s="25" t="inlineStr">
         <is>
           <t>Total 2026</t>
         </is>
       </c>
-      <c r="F28" s="27" t="inlineStr">
+      <c r="F28" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="G28" s="27" t="inlineStr">
+      <c r="G28" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="42" t="inlineStr">
+      <c r="B29" s="40" t="inlineStr">
         <is>
           <t>(+) Total activos</t>
         </is>
       </c>
-      <c r="D29" s="43">
+      <c r="D29" s="41">
         <f>D20</f>
         <v/>
       </c>
-      <c r="E29" s="43">
+      <c r="E29" s="41">
         <f>E20</f>
         <v/>
       </c>
-      <c r="F29" s="43">
+      <c r="F29" s="41">
         <f>E29-D29</f>
         <v/>
       </c>
-      <c r="G29" s="44">
+      <c r="G29" s="42">
         <f>IF(D29=0,"",(E29-D29)/D29)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="42" t="inlineStr">
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>(-) Total pasivos</t>
         </is>
       </c>
-      <c r="D30" s="43">
+      <c r="D30" s="41">
         <f>D25</f>
         <v/>
       </c>
-      <c r="E30" s="43">
+      <c r="E30" s="41">
         <f>E25</f>
         <v/>
       </c>
-      <c r="F30" s="43">
+      <c r="F30" s="41">
         <f>E30-D30</f>
         <v/>
       </c>
-      <c r="G30" s="44">
+      <c r="G30" s="42">
         <f>IF(D30=0,"",(E30-D30)/D30)</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="45" t="inlineStr">
+      <c r="B31" s="43" t="inlineStr">
         <is>
           <t>(=) PATRIMONIO NETO</t>
         </is>
       </c>
-      <c r="D31" s="46">
+      <c r="D31" s="44">
         <f>D29-D30</f>
         <v/>
       </c>
-      <c r="E31" s="46">
+      <c r="E31" s="44">
         <f>E29-E30</f>
         <v/>
       </c>
-      <c r="F31" s="46">
+      <c r="F31" s="44">
         <f>E31-D31</f>
         <v/>
       </c>
-      <c r="G31" s="47">
+      <c r="G31" s="45">
         <f>IF(D31=0,"",(E31-D31)/D31)</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="48" t="inlineStr">
+      <c r="B32" s="46" t="inlineStr">
         <is>
           <t>Patrimonio declarado en el XML (2025)</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="49" t="n">
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="47" t="n">
         <v>883285.5600000001</v>
       </c>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="B33" s="48" t="inlineStr">
+      <c r="B33" s="46" t="inlineStr">
         <is>
           <t>Patrimonio neto del anio anterior</t>
         </is>
       </c>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="49" t="n">
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="47" t="n">
         <v>801569.97</v>
       </c>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="6" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="B34" s="48" t="inlineStr">
+      <c r="B34" s="46" t="inlineStr">
         <is>
           <t>Crecimiento / decremento patrimonial (XML)</t>
         </is>
       </c>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="49" t="n">
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="47" t="n">
         <v>81715.59</v>
       </c>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="5" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="50" t="inlineStr">
+      <c r="B36" s="48" t="inlineStr">
         <is>
           <t>CONSOLIDADO</t>
         </is>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1">
-      <c r="B37" s="26" t="inlineStr">
+      <c r="B37" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C37" s="26" t="n"/>
-      <c r="D37" s="27" t="inlineStr">
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="25" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="E37" s="27" t="inlineStr">
+      <c r="E37" s="25" t="inlineStr">
         <is>
           <t>Total 2026</t>
         </is>
       </c>
-      <c r="F37" s="27" t="inlineStr">
+      <c r="F37" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="G37" s="27" t="inlineStr">
+      <c r="G37" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="51" t="inlineStr">
+      <c r="B38" s="49" t="inlineStr">
         <is>
           <t>Activos</t>
         </is>
       </c>
-      <c r="D38" s="52">
+      <c r="D38" s="50">
         <f>D20</f>
         <v/>
       </c>
-      <c r="E38" s="52">
+      <c r="E38" s="50">
         <f>E20</f>
         <v/>
       </c>
-      <c r="F38" s="52">
+      <c r="F38" s="50">
         <f>E38-D38</f>
         <v/>
       </c>
-      <c r="G38" s="53">
+      <c r="G38" s="51">
         <f>IF(D38=0,"",(E38-D38)/D38)</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="54" t="inlineStr">
+      <c r="B39" s="52" t="inlineStr">
         <is>
           <t>Pasivos</t>
         </is>
       </c>
-      <c r="D39" s="55">
+      <c r="D39" s="53">
         <f>D25</f>
         <v/>
       </c>
-      <c r="E39" s="55">
+      <c r="E39" s="53">
         <f>E25</f>
         <v/>
       </c>
-      <c r="F39" s="55">
+      <c r="F39" s="53">
         <f>E39-D39</f>
         <v/>
       </c>
-      <c r="G39" s="56">
+      <c r="G39" s="54">
         <f>IF(D39=0,"",(E39-D39)/D39)</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="B40" s="57" t="inlineStr">
+      <c r="B40" s="55" t="inlineStr">
         <is>
           <t>Patrimonio neto</t>
         </is>
       </c>
-      <c r="D40" s="58">
+      <c r="D40" s="56">
         <f>D31</f>
         <v/>
       </c>
-      <c r="E40" s="58">
+      <c r="E40" s="56">
         <f>E31</f>
         <v/>
       </c>
-      <c r="F40" s="58">
+      <c r="F40" s="56">
         <f>E40-D40</f>
         <v/>
       </c>
-      <c r="G40" s="59">
+      <c r="G40" s="57">
         <f>IF(D40=0,"",(E40-D40)/D40)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="60" t="inlineStr">
+      <c r="B42" s="58" t="inlineStr">
         <is>
           <t>Edite las columnas amarillas en las hojas de cada modulo; las tarjetas, secciones y graficos se recalculan solos.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="40">
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B25:C25"/>
@@ -1679,22 +1731,15 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="I4:J4"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B22:G22"/>
-    <mergeCell ref="I3:L3"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B27:G27"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="B32:C32"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="I4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Columnas,Barras,Pastel,Anillo,Lineas,Area"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1741,197 +1786,197 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Tipo de acreedor</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Domicilio del acreedor</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Nombre del acreedor</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>N. de identificacion</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>N. registro Banco Central</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Partes relacionadas</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="J5" s="27" t="inlineStr">
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="K5" s="27" t="inlineStr">
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="L5" s="27" t="inlineStr">
+      <c r="L5" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr">
+      <c r="A6" s="59" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B6" s="61" t="inlineStr">
+      <c r="B6" s="59" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C6" s="61" t="inlineStr">
+      <c r="C6" s="59" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D6" s="61" t="inlineStr">
+      <c r="D6" s="59" t="inlineStr">
         <is>
           <t>DINERS CLUB DEL ECUADOR</t>
         </is>
       </c>
-      <c r="E6" s="61" t="inlineStr">
+      <c r="E6" s="59" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
-      <c r="F6" s="61" t="inlineStr">
+      <c r="F6" s="59" t="inlineStr">
         <is>
           <t>1792260957001</t>
         </is>
       </c>
-      <c r="G6" s="61" t="inlineStr"/>
-      <c r="H6" s="61" t="inlineStr">
+      <c r="G6" s="59" t="inlineStr"/>
+      <c r="H6" s="59" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="I6" s="62" t="n">
+      <c r="I6" s="60" t="n">
         <v>4891.88</v>
       </c>
-      <c r="J6" s="63" t="n">
+      <c r="J6" s="61" t="n">
         <v>4891.88</v>
       </c>
-      <c r="K6" s="62">
+      <c r="K6" s="60">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="64">
+      <c r="L6" s="62">
         <f>IF(I6=0,"",(J6-I6)/I6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="65" t="inlineStr">
+      <c r="A7" s="63" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B7" s="65" t="inlineStr">
+      <c r="B7" s="63" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C7" s="65" t="inlineStr">
+      <c r="C7" s="63" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D7" s="65" t="inlineStr">
+      <c r="D7" s="63" t="inlineStr">
         <is>
           <t>BANCO DEL PICHINCHA</t>
         </is>
       </c>
-      <c r="E7" s="65" t="inlineStr">
+      <c r="E7" s="63" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
-      <c r="F7" s="65" t="inlineStr">
+      <c r="F7" s="63" t="inlineStr">
         <is>
           <t>1790010937001</t>
         </is>
       </c>
-      <c r="G7" s="65" t="inlineStr"/>
-      <c r="H7" s="65" t="inlineStr">
+      <c r="G7" s="63" t="inlineStr"/>
+      <c r="H7" s="63" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="I7" s="66" t="n">
+      <c r="I7" s="64" t="n">
         <v>5547.31</v>
       </c>
-      <c r="J7" s="63" t="n">
+      <c r="J7" s="61" t="n">
         <v>5547.31</v>
       </c>
-      <c r="K7" s="66">
+      <c r="K7" s="64">
         <f>J7-I7</f>
         <v/>
       </c>
-      <c r="L7" s="67">
+      <c r="L7" s="65">
         <f>IF(I7=0,"",(J7-I7)/I7)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="69" t="inlineStr">
+      <c r="A8" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="69" t="n"/>
-      <c r="C8" s="69" t="n"/>
-      <c r="D8" s="69" t="n"/>
-      <c r="E8" s="69" t="n"/>
-      <c r="F8" s="69" t="n"/>
-      <c r="G8" s="69" t="n"/>
-      <c r="H8" s="69" t="n"/>
-      <c r="I8" s="39">
+      <c r="B8" s="67" t="n"/>
+      <c r="C8" s="67" t="n"/>
+      <c r="D8" s="67" t="n"/>
+      <c r="E8" s="67" t="n"/>
+      <c r="F8" s="67" t="n"/>
+      <c r="G8" s="67" t="n"/>
+      <c r="H8" s="67" t="n"/>
+      <c r="I8" s="37">
         <f>SUM(I6:I7)</f>
         <v/>
       </c>
-      <c r="J8" s="39">
+      <c r="J8" s="37">
         <f>SUM(J6:J7)</f>
         <v/>
       </c>
-      <c r="K8" s="39">
+      <c r="K8" s="37">
         <f>J8-I8</f>
         <v/>
       </c>
-      <c r="L8" s="40">
+      <c r="L8" s="38">
         <f>IF(I8=0,"",(J8-I8)/I8)</f>
         <v/>
       </c>
@@ -1997,115 +2042,115 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="70" t="inlineStr">
+      <c r="B5" s="68" t="inlineStr">
         <is>
           <t>Incremento patrimonial declarado en el XML</t>
         </is>
       </c>
-      <c r="C5" s="71" t="n"/>
-      <c r="D5" s="71" t="n"/>
-      <c r="E5" s="72" t="n">
+      <c r="C5" s="69" t="n"/>
+      <c r="D5" s="69" t="n"/>
+      <c r="E5" s="70" t="n">
         <v>81715.59</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>Concepto (Tabla 14 del SRI)</t>
         </is>
       </c>
-      <c r="E7" s="27" t="inlineStr">
+      <c r="E7" s="25" t="inlineStr">
         <is>
           <t>Justifica la variacion</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="73" t="inlineStr">
+      <c r="B8" s="71" t="inlineStr">
         <is>
           <t>1 - Ingresos locales</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="72" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="73" t="inlineStr">
+      <c r="B9" s="71" t="inlineStr">
         <is>
           <t>2 - Ingresos exterior</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="72" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="73" t="inlineStr">
+      <c r="B10" s="71" t="inlineStr">
         <is>
           <t>3 - Herencias, legados o donaciones</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="72" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="73" t="inlineStr">
+      <c r="B11" s="71" t="inlineStr">
         <is>
           <t>4 - Loterias o rifas</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="72" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="73" t="inlineStr">
+      <c r="B12" s="71" t="inlineStr">
         <is>
           <t>5 - Ganancias de capital</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="72" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="73" t="inlineStr">
+      <c r="B13" s="71" t="inlineStr">
         <is>
           <t>6 - Otros</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="72" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="60" t="inlineStr">
+      <c r="B15" s="58" t="inlineStr">
         <is>
           <t>Esta hoja reproduce la seccion Justificacion del formulario del SRI. Marque 'Si' en los conceptos que apliquen; el generador de XML los toma de aqui.</t>
         </is>
@@ -2168,97 +2213,97 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="74" t="inlineStr">
+      <c r="B5" s="73" t="inlineStr">
         <is>
           <t>►   GENERAR XML</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="75" t="inlineStr">
+      <c r="B7" s="74" t="inlineStr">
         <is>
           <t>En el archivo .xlsm el boton verde ya esta vinculado a la macro GenerarXmlSRI.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="76" t="inlineStr">
+      <c r="B9" s="75" t="inlineStr">
         <is>
           <t>COMO USAR ESTE ARCHIVO</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="77" t="inlineStr">
+      <c r="B10" s="76" t="inlineStr">
         <is>
           <t>1. Al abrir el archivo .xlsm, pulse 'Habilitar contenido' en la barra de seguridad de Excel.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="77" t="inlineStr">
+      <c r="B11" s="76" t="inlineStr">
         <is>
           <t>2. Llene las columnas amarillas de cada modulo (Dinero, Vehiculos, etc.) y la hoja Justificacion.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="77" t="inlineStr">
+      <c r="B12" s="76" t="inlineStr">
         <is>
           <t>3. Pulse el boton verde GENERAR XML, indique el anio y elija donde guardar el archivo.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="77" t="inlineStr">
+      <c r="B13" s="76" t="inlineStr">
         <is>
           <t>4. El archivo .xml queda listo para subir al portal del SRI.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="77" t="inlineStr"/>
+      <c r="B14" s="76" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="76" t="inlineStr">
+      <c r="B15" s="75" t="inlineStr">
         <is>
           <t>SI EXCEL BLOQUEA LAS MACROS</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="77" t="inlineStr">
+      <c r="B16" s="76" t="inlineStr">
         <is>
           <t>- Cierre Excel. En el Explorador, clic derecho sobre el archivo &gt; Propiedades.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="77" t="inlineStr">
+      <c r="B17" s="76" t="inlineStr">
         <is>
           <t>- Al final de la pestana General marque 'Desbloquear' y pulse Aceptar.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="77" t="inlineStr">
+      <c r="B18" s="76" t="inlineStr">
         <is>
           <t>- Vuelva a abrirlo y pulse 'Habilitar contenido'. Conserve siempre la extension .xlsm.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="77" t="inlineStr"/>
+      <c r="B19" s="76" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="B20" s="77" t="inlineStr">
+      <c r="B20" s="76" t="inlineStr">
         <is>
           <t>Alternativa sin macros:  ejecutar  python tools/generar_xml_sri.py  desde la terminal.</t>
         </is>
@@ -2299,257 +2344,257 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="78" t="inlineStr">
+      <c r="A5" s="77" t="inlineStr">
         <is>
           <t>IDENTIFICACION</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="79" t="inlineStr">
+      <c r="A6" s="78" t="inlineStr">
         <is>
           <t>Anio de la declaracion</t>
         </is>
       </c>
-      <c r="B6" s="80" t="n">
+      <c r="B6" s="79" t="n">
         <v>2025</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="79" t="inlineStr">
+      <c r="A7" s="78" t="inlineStr">
         <is>
           <t>Tipo de declaracion</t>
         </is>
       </c>
-      <c r="B7" s="80" t="inlineStr">
+      <c r="B7" s="79" t="inlineStr">
         <is>
           <t>SOC - Sociedad conyugal o union de hecho</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="79" t="inlineStr">
+      <c r="A8" s="78" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="B8" s="80" t="inlineStr">
+      <c r="B8" s="79" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="79" t="inlineStr">
+      <c r="A9" s="78" t="inlineStr">
         <is>
           <t>Numero de identificacion</t>
         </is>
       </c>
-      <c r="B9" s="80" t="inlineStr">
+      <c r="B9" s="79" t="inlineStr">
         <is>
           <t>1709164899001</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="79" t="inlineStr">
+      <c r="A10" s="78" t="inlineStr">
         <is>
           <t>Nombre del declarante</t>
         </is>
       </c>
-      <c r="B10" s="80" t="inlineStr">
+      <c r="B10" s="79" t="inlineStr">
         <is>
           <t>GONZALEZ NAVAS MARCO VINICIO</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="79" t="inlineStr">
+      <c r="A11" s="78" t="inlineStr">
         <is>
           <t>Identificacion del conyuge</t>
         </is>
       </c>
-      <c r="B11" s="80" t="inlineStr">
+      <c r="B11" s="79" t="inlineStr">
         <is>
           <t>C - Cedula</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="79" t="inlineStr">
+      <c r="A12" s="78" t="inlineStr">
         <is>
           <t>Numero ident. conyuge</t>
         </is>
       </c>
-      <c r="B12" s="80" t="inlineStr">
+      <c r="B12" s="79" t="inlineStr">
         <is>
           <t>1709784225</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="79" t="inlineStr">
+      <c r="A13" s="78" t="inlineStr">
         <is>
           <t>Nombre del conyuge</t>
         </is>
       </c>
-      <c r="B13" s="80" t="inlineStr">
+      <c r="B13" s="79" t="inlineStr">
         <is>
           <t>HIDALGO LOZA ROSA CONSUELO</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="79" t="inlineStr">
+      <c r="A14" s="78" t="inlineStr">
         <is>
           <t>Total creditos / cuentas por cobrar</t>
         </is>
       </c>
-      <c r="B14" s="62" t="n">
+      <c r="B14" s="60" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="78" t="inlineStr">
+      <c r="A16" s="77" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO (enlazado a la hoja Dashboard)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="79" t="inlineStr">
+      <c r="A17" s="78" t="inlineStr">
         <is>
           <t>Patrimonio neto 2025</t>
         </is>
       </c>
-      <c r="B17" s="62">
+      <c r="B17" s="60">
         <f>Dashboard!D31</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="79" t="inlineStr">
+      <c r="A18" s="78" t="inlineStr">
         <is>
           <t>Patrimonio neto 2026 (proyectado)</t>
         </is>
       </c>
-      <c r="B18" s="62">
+      <c r="B18" s="60">
         <f>Dashboard!E31</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="79" t="inlineStr">
+      <c r="A19" s="78" t="inlineStr">
         <is>
           <t>Variacion proyectada</t>
         </is>
       </c>
-      <c r="B19" s="62">
+      <c r="B19" s="60">
         <f>Dashboard!F31</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="79" t="inlineStr">
+      <c r="A20" s="78" t="inlineStr">
         <is>
           <t>Variacion % proyectada</t>
         </is>
       </c>
-      <c r="B20" s="64">
+      <c r="B20" s="62">
         <f>Dashboard!G31</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="78" t="inlineStr">
+      <c r="A22" s="77" t="inlineStr">
         <is>
           <t>PATRIMONIO DECLARADO EN EL XML</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="79" t="inlineStr">
+      <c r="A23" s="78" t="inlineStr">
         <is>
           <t>Patrimonio total declarado</t>
         </is>
       </c>
-      <c r="B23" s="62" t="n">
+      <c r="B23" s="60" t="n">
         <v>883285.5600000001</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="79" t="inlineStr">
+      <c r="A24" s="78" t="inlineStr">
         <is>
           <t>Atribuible a hijos no emancipados</t>
         </is>
       </c>
-      <c r="B24" s="62" t="n">
+      <c r="B24" s="60" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="79" t="inlineStr">
+      <c r="A25" s="78" t="inlineStr">
         <is>
           <t>Patrimonio en la sociedad conyugal</t>
         </is>
       </c>
-      <c r="B25" s="62" t="n">
+      <c r="B25" s="60" t="n">
         <v>883285.5600000001</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="79" t="inlineStr">
+      <c r="A26" s="78" t="inlineStr">
         <is>
           <t>Patrimonio individual del declarante</t>
         </is>
       </c>
-      <c r="B26" s="62" t="n">
+      <c r="B26" s="60" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="79" t="inlineStr">
+      <c r="A27" s="78" t="inlineStr">
         <is>
           <t>Patrimonio del anio anterior</t>
         </is>
       </c>
-      <c r="B27" s="62" t="n">
+      <c r="B27" s="60" t="n">
         <v>801569.97</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="79" t="inlineStr">
+      <c r="A28" s="78" t="inlineStr">
         <is>
           <t>Crecimiento / decremento patrimonial</t>
         </is>
       </c>
-      <c r="B28" s="62" t="n">
+      <c r="B28" s="60" t="n">
         <v>81715.59</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="76" t="inlineStr">
+      <c r="A30" s="75" t="inlineStr">
         <is>
           <t>Justificacion de la variacion (ver hoja Justificacion)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="77" t="inlineStr">
+      <c r="A31" s="76" t="inlineStr">
         <is>
           <t>- 1 - Ingresos locales</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="77" t="inlineStr">
+      <c r="A32" s="76" t="inlineStr">
         <is>
           <t>- 6 - Otros</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="60" t="inlineStr">
+      <c r="A34" s="58" t="inlineStr">
         <is>
           <t>Catalogos del SRI integrados (Tablas 1-19 del archivo CATALOGO.xls). El XML se genera con generar_xml_sri.py.</t>
         </is>
@@ -5820,97 +5865,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="81" t="inlineStr">
+      <c r="A1" s="80" t="inlineStr">
         <is>
           <t>DINERO_EN</t>
         </is>
       </c>
-      <c r="B1" s="81" t="inlineStr">
+      <c r="B1" s="80" t="inlineStr">
         <is>
           <t>TIPO_INVERSION</t>
         </is>
       </c>
-      <c r="C1" s="81" t="inlineStr">
+      <c r="C1" s="80" t="inlineStr">
         <is>
           <t>UBICACION</t>
         </is>
       </c>
-      <c r="D1" s="81" t="inlineStr">
+      <c r="D1" s="80" t="inlineStr">
         <is>
           <t>PAIS</t>
         </is>
       </c>
-      <c r="E1" s="81" t="inlineStr">
+      <c r="E1" s="80" t="inlineStr">
         <is>
           <t>INSTITUCION_FINANCIERA</t>
         </is>
       </c>
-      <c r="F1" s="81" t="inlineStr">
+      <c r="F1" s="80" t="inlineStr">
         <is>
           <t>PARTES_RELACIONADAS</t>
         </is>
       </c>
-      <c r="G1" s="81" t="inlineStr">
+      <c r="G1" s="80" t="inlineStr">
         <is>
           <t>TIPO_DRC</t>
         </is>
       </c>
-      <c r="H1" s="81" t="inlineStr">
+      <c r="H1" s="80" t="inlineStr">
         <is>
           <t>TIPO_PERSONA</t>
         </is>
       </c>
-      <c r="I1" s="81" t="inlineStr">
+      <c r="I1" s="80" t="inlineStr">
         <is>
           <t>TIPO_BIEN_MUEBLE</t>
         </is>
       </c>
-      <c r="J1" s="81" t="inlineStr">
+      <c r="J1" s="80" t="inlineStr">
         <is>
           <t>TIPO_VEHICULO</t>
         </is>
       </c>
-      <c r="K1" s="81" t="inlineStr">
+      <c r="K1" s="80" t="inlineStr">
         <is>
           <t>TIPO_DERECHO</t>
         </is>
       </c>
-      <c r="L1" s="81" t="inlineStr">
+      <c r="L1" s="80" t="inlineStr">
         <is>
           <t>TIPO_INMUEBLE</t>
         </is>
       </c>
-      <c r="M1" s="81" t="inlineStr">
+      <c r="M1" s="80" t="inlineStr">
         <is>
           <t>PROVINCIA</t>
         </is>
       </c>
-      <c r="N1" s="81" t="inlineStr">
+      <c r="N1" s="80" t="inlineStr">
         <is>
           <t>CANTON</t>
         </is>
       </c>
-      <c r="O1" s="81" t="inlineStr">
+      <c r="O1" s="80" t="inlineStr">
         <is>
           <t>TIPO_ACREEDOR</t>
         </is>
       </c>
-      <c r="P1" s="81" t="inlineStr">
+      <c r="P1" s="80" t="inlineStr">
         <is>
           <t>TIPO_IDENTIFICACION</t>
         </is>
       </c>
-      <c r="Q1" s="81" t="inlineStr">
+      <c r="Q1" s="80" t="inlineStr">
         <is>
           <t>REGULARIZACION</t>
         </is>
       </c>
-      <c r="R1" s="81" t="inlineStr">
+      <c r="R1" s="80" t="inlineStr">
         <is>
           <t>JUSTIF_INCREMENTO</t>
         </is>
       </c>
-      <c r="S1" s="81" t="inlineStr">
+      <c r="S1" s="80" t="inlineStr">
         <is>
           <t>JUSTIF_DECREMENTO</t>
         </is>
@@ -12444,311 +12489,311 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Dinero en</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Tipo de inversion</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Institucion financiera</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Tipo de moneda</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Partes relacionadas</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="J5" s="27" t="inlineStr">
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="K5" s="27" t="inlineStr">
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="L5" s="27" t="inlineStr">
+      <c r="L5" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="M5" s="27" t="inlineStr">
+      <c r="M5" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr">
+      <c r="A6" s="59" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B6" s="61" t="inlineStr">
+      <c r="B6" s="59" t="inlineStr">
         <is>
           <t>3 - Cuenta de ahorros</t>
         </is>
       </c>
-      <c r="C6" s="61" t="inlineStr">
+      <c r="C6" s="59" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D6" s="61" t="inlineStr">
+      <c r="D6" s="59" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E6" s="61" t="inlineStr">
+      <c r="E6" s="59" t="inlineStr">
         <is>
           <t>1029 - BANCO PICHINCHA C.A.</t>
         </is>
       </c>
-      <c r="F6" s="61" t="inlineStr">
+      <c r="F6" s="59" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G6" s="61" t="inlineStr">
+      <c r="G6" s="59" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H6" s="61" t="inlineStr"/>
-      <c r="I6" s="61" t="inlineStr"/>
-      <c r="J6" s="62" t="n">
+      <c r="H6" s="59" t="inlineStr"/>
+      <c r="I6" s="59" t="inlineStr"/>
+      <c r="J6" s="60" t="n">
         <v>130.2</v>
       </c>
-      <c r="K6" s="63" t="n">
+      <c r="K6" s="61" t="n">
         <v>130.2</v>
       </c>
-      <c r="L6" s="62">
+      <c r="L6" s="60">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="64">
+      <c r="M6" s="62">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="65" t="inlineStr">
+      <c r="A7" s="63" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B7" s="65" t="inlineStr">
+      <c r="B7" s="63" t="inlineStr">
         <is>
           <t>4 - Cuenta corriente</t>
         </is>
       </c>
-      <c r="C7" s="65" t="inlineStr">
+      <c r="C7" s="63" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D7" s="65" t="inlineStr">
+      <c r="D7" s="63" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E7" s="65" t="inlineStr">
+      <c r="E7" s="63" t="inlineStr">
         <is>
           <t>1029 - BANCO PICHINCHA C.A.</t>
         </is>
       </c>
-      <c r="F7" s="65" t="inlineStr">
+      <c r="F7" s="63" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G7" s="65" t="inlineStr">
+      <c r="G7" s="63" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H7" s="65" t="inlineStr"/>
-      <c r="I7" s="65" t="inlineStr"/>
-      <c r="J7" s="66" t="n">
+      <c r="H7" s="63" t="inlineStr"/>
+      <c r="I7" s="63" t="inlineStr"/>
+      <c r="J7" s="64" t="n">
         <v>5590.32</v>
       </c>
-      <c r="K7" s="63" t="n">
+      <c r="K7" s="61" t="n">
         <v>5590.32</v>
       </c>
-      <c r="L7" s="66">
+      <c r="L7" s="64">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="67">
+      <c r="M7" s="65">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="59" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B8" s="61" t="inlineStr">
+      <c r="B8" s="59" t="inlineStr">
         <is>
           <t>3 - Cuenta de ahorros</t>
         </is>
       </c>
-      <c r="C8" s="61" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D8" s="61" t="inlineStr">
+      <c r="D8" s="59" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E8" s="61" t="inlineStr">
+      <c r="E8" s="59" t="inlineStr">
         <is>
           <t>1418 - BANCO PROMERICA S.A.</t>
         </is>
       </c>
-      <c r="F8" s="61" t="inlineStr">
+      <c r="F8" s="59" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G8" s="61" t="inlineStr">
+      <c r="G8" s="59" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H8" s="61" t="inlineStr"/>
-      <c r="I8" s="61" t="inlineStr"/>
-      <c r="J8" s="62" t="n">
+      <c r="H8" s="59" t="inlineStr"/>
+      <c r="I8" s="59" t="inlineStr"/>
+      <c r="J8" s="60" t="n">
         <v>53237.31</v>
       </c>
-      <c r="K8" s="63" t="n">
+      <c r="K8" s="61" t="n">
         <v>53237.31</v>
       </c>
-      <c r="L8" s="62">
+      <c r="L8" s="60">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="64">
+      <c r="M8" s="62">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="65" t="inlineStr">
+      <c r="A9" s="63" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B9" s="65" t="inlineStr">
+      <c r="B9" s="63" t="inlineStr">
         <is>
           <t>2 - Inversiones financieras</t>
         </is>
       </c>
-      <c r="C9" s="65" t="inlineStr">
+      <c r="C9" s="63" t="inlineStr">
         <is>
           <t>EXT - En el exterior</t>
         </is>
       </c>
-      <c r="D9" s="65" t="inlineStr">
+      <c r="D9" s="63" t="inlineStr">
         <is>
           <t>118 - PANAMA</t>
         </is>
       </c>
-      <c r="E9" s="65" t="inlineStr">
+      <c r="E9" s="63" t="inlineStr">
         <is>
           <t>BANCO PICHINCHA CA</t>
         </is>
       </c>
-      <c r="F9" s="65" t="inlineStr">
+      <c r="F9" s="63" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G9" s="65" t="inlineStr">
+      <c r="G9" s="63" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H9" s="65" t="inlineStr"/>
-      <c r="I9" s="65" t="inlineStr"/>
-      <c r="J9" s="66" t="n">
+      <c r="H9" s="63" t="inlineStr"/>
+      <c r="I9" s="63" t="inlineStr"/>
+      <c r="J9" s="64" t="n">
         <v>189049.31</v>
       </c>
-      <c r="K9" s="63" t="n">
+      <c r="K9" s="61" t="n">
         <v>189049.31</v>
       </c>
-      <c r="L9" s="66">
+      <c r="L9" s="64">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="67">
+      <c r="M9" s="65">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="68" t="inlineStr">
+      <c r="A10" s="66" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B10" s="68" t="n"/>
-      <c r="C10" s="68" t="n"/>
-      <c r="D10" s="68" t="n"/>
-      <c r="E10" s="68" t="n"/>
-      <c r="F10" s="68" t="n"/>
-      <c r="G10" s="68" t="n"/>
-      <c r="H10" s="68" t="n"/>
-      <c r="I10" s="68" t="n"/>
-      <c r="J10" s="32">
+      <c r="B10" s="66" t="n"/>
+      <c r="C10" s="66" t="n"/>
+      <c r="D10" s="66" t="n"/>
+      <c r="E10" s="66" t="n"/>
+      <c r="F10" s="66" t="n"/>
+      <c r="G10" s="66" t="n"/>
+      <c r="H10" s="66" t="n"/>
+      <c r="I10" s="66" t="n"/>
+      <c r="J10" s="30">
         <f>SUM(J6:J9)</f>
         <v/>
       </c>
-      <c r="K10" s="32">
+      <c r="K10" s="30">
         <f>SUM(K6:K9)</f>
         <v/>
       </c>
-      <c r="L10" s="32">
+      <c r="L10" s="30">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="33">
+      <c r="M10" s="31">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
@@ -12828,299 +12873,299 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Tipo de inversion</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Empresa / Administradora / Fideicomiso</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>% de participacion</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>N. de acciones / participaciones</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Partes relacionadas</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="J5" s="27" t="inlineStr">
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="K5" s="27" t="inlineStr">
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="L5" s="27" t="inlineStr">
+      <c r="L5" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="M5" s="27" t="inlineStr">
+      <c r="M5" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr"/>
-      <c r="B6" s="61" t="inlineStr"/>
-      <c r="C6" s="61" t="inlineStr"/>
-      <c r="D6" s="61" t="inlineStr"/>
-      <c r="E6" s="61" t="inlineStr"/>
-      <c r="F6" s="61" t="inlineStr"/>
-      <c r="G6" s="61" t="inlineStr"/>
-      <c r="H6" s="61" t="inlineStr"/>
-      <c r="I6" s="61" t="inlineStr"/>
-      <c r="J6" s="63" t="n">
+      <c r="A6" s="59" t="inlineStr"/>
+      <c r="B6" s="59" t="inlineStr"/>
+      <c r="C6" s="59" t="inlineStr"/>
+      <c r="D6" s="59" t="inlineStr"/>
+      <c r="E6" s="59" t="inlineStr"/>
+      <c r="F6" s="59" t="inlineStr"/>
+      <c r="G6" s="59" t="inlineStr"/>
+      <c r="H6" s="59" t="inlineStr"/>
+      <c r="I6" s="59" t="inlineStr"/>
+      <c r="J6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="63" t="n">
+      <c r="K6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="62">
+      <c r="L6" s="60">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="64">
+      <c r="M6" s="62">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="65" t="inlineStr"/>
-      <c r="B7" s="65" t="inlineStr"/>
-      <c r="C7" s="65" t="inlineStr"/>
-      <c r="D7" s="65" t="inlineStr"/>
-      <c r="E7" s="65" t="inlineStr"/>
-      <c r="F7" s="65" t="inlineStr"/>
-      <c r="G7" s="65" t="inlineStr"/>
-      <c r="H7" s="65" t="inlineStr"/>
-      <c r="I7" s="65" t="inlineStr"/>
-      <c r="J7" s="63" t="n">
+      <c r="A7" s="63" t="inlineStr"/>
+      <c r="B7" s="63" t="inlineStr"/>
+      <c r="C7" s="63" t="inlineStr"/>
+      <c r="D7" s="63" t="inlineStr"/>
+      <c r="E7" s="63" t="inlineStr"/>
+      <c r="F7" s="63" t="inlineStr"/>
+      <c r="G7" s="63" t="inlineStr"/>
+      <c r="H7" s="63" t="inlineStr"/>
+      <c r="I7" s="63" t="inlineStr"/>
+      <c r="J7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="63" t="n">
+      <c r="K7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="66">
+      <c r="L7" s="64">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="67">
+      <c r="M7" s="65">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr"/>
-      <c r="B8" s="61" t="inlineStr"/>
-      <c r="C8" s="61" t="inlineStr"/>
-      <c r="D8" s="61" t="inlineStr"/>
-      <c r="E8" s="61" t="inlineStr"/>
-      <c r="F8" s="61" t="inlineStr"/>
-      <c r="G8" s="61" t="inlineStr"/>
-      <c r="H8" s="61" t="inlineStr"/>
-      <c r="I8" s="61" t="inlineStr"/>
-      <c r="J8" s="63" t="n">
+      <c r="A8" s="59" t="inlineStr"/>
+      <c r="B8" s="59" t="inlineStr"/>
+      <c r="C8" s="59" t="inlineStr"/>
+      <c r="D8" s="59" t="inlineStr"/>
+      <c r="E8" s="59" t="inlineStr"/>
+      <c r="F8" s="59" t="inlineStr"/>
+      <c r="G8" s="59" t="inlineStr"/>
+      <c r="H8" s="59" t="inlineStr"/>
+      <c r="I8" s="59" t="inlineStr"/>
+      <c r="J8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="63" t="n">
+      <c r="K8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="62">
+      <c r="L8" s="60">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="64">
+      <c r="M8" s="62">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="65" t="inlineStr"/>
-      <c r="B9" s="65" t="inlineStr"/>
-      <c r="C9" s="65" t="inlineStr"/>
-      <c r="D9" s="65" t="inlineStr"/>
-      <c r="E9" s="65" t="inlineStr"/>
-      <c r="F9" s="65" t="inlineStr"/>
-      <c r="G9" s="65" t="inlineStr"/>
-      <c r="H9" s="65" t="inlineStr"/>
-      <c r="I9" s="65" t="inlineStr"/>
-      <c r="J9" s="63" t="n">
+      <c r="A9" s="63" t="inlineStr"/>
+      <c r="B9" s="63" t="inlineStr"/>
+      <c r="C9" s="63" t="inlineStr"/>
+      <c r="D9" s="63" t="inlineStr"/>
+      <c r="E9" s="63" t="inlineStr"/>
+      <c r="F9" s="63" t="inlineStr"/>
+      <c r="G9" s="63" t="inlineStr"/>
+      <c r="H9" s="63" t="inlineStr"/>
+      <c r="I9" s="63" t="inlineStr"/>
+      <c r="J9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="63" t="n">
+      <c r="K9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="66">
+      <c r="L9" s="64">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="67">
+      <c r="M9" s="65">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr"/>
-      <c r="B10" s="61" t="inlineStr"/>
-      <c r="C10" s="61" t="inlineStr"/>
-      <c r="D10" s="61" t="inlineStr"/>
-      <c r="E10" s="61" t="inlineStr"/>
-      <c r="F10" s="61" t="inlineStr"/>
-      <c r="G10" s="61" t="inlineStr"/>
-      <c r="H10" s="61" t="inlineStr"/>
-      <c r="I10" s="61" t="inlineStr"/>
-      <c r="J10" s="63" t="n">
+      <c r="A10" s="59" t="inlineStr"/>
+      <c r="B10" s="59" t="inlineStr"/>
+      <c r="C10" s="59" t="inlineStr"/>
+      <c r="D10" s="59" t="inlineStr"/>
+      <c r="E10" s="59" t="inlineStr"/>
+      <c r="F10" s="59" t="inlineStr"/>
+      <c r="G10" s="59" t="inlineStr"/>
+      <c r="H10" s="59" t="inlineStr"/>
+      <c r="I10" s="59" t="inlineStr"/>
+      <c r="J10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="63" t="n">
+      <c r="K10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="62">
+      <c r="L10" s="60">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="64">
+      <c r="M10" s="62">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="65" t="inlineStr"/>
-      <c r="B11" s="65" t="inlineStr"/>
-      <c r="C11" s="65" t="inlineStr"/>
-      <c r="D11" s="65" t="inlineStr"/>
-      <c r="E11" s="65" t="inlineStr"/>
-      <c r="F11" s="65" t="inlineStr"/>
-      <c r="G11" s="65" t="inlineStr"/>
-      <c r="H11" s="65" t="inlineStr"/>
-      <c r="I11" s="65" t="inlineStr"/>
-      <c r="J11" s="63" t="n">
+      <c r="A11" s="63" t="inlineStr"/>
+      <c r="B11" s="63" t="inlineStr"/>
+      <c r="C11" s="63" t="inlineStr"/>
+      <c r="D11" s="63" t="inlineStr"/>
+      <c r="E11" s="63" t="inlineStr"/>
+      <c r="F11" s="63" t="inlineStr"/>
+      <c r="G11" s="63" t="inlineStr"/>
+      <c r="H11" s="63" t="inlineStr"/>
+      <c r="I11" s="63" t="inlineStr"/>
+      <c r="J11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="63" t="n">
+      <c r="K11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="66">
+      <c r="L11" s="64">
         <f>K11-J11</f>
         <v/>
       </c>
-      <c r="M11" s="67">
+      <c r="M11" s="65">
         <f>IF(J11=0,"",(K11-J11)/J11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr"/>
-      <c r="B12" s="61" t="inlineStr"/>
-      <c r="C12" s="61" t="inlineStr"/>
-      <c r="D12" s="61" t="inlineStr"/>
-      <c r="E12" s="61" t="inlineStr"/>
-      <c r="F12" s="61" t="inlineStr"/>
-      <c r="G12" s="61" t="inlineStr"/>
-      <c r="H12" s="61" t="inlineStr"/>
-      <c r="I12" s="61" t="inlineStr"/>
-      <c r="J12" s="63" t="n">
+      <c r="A12" s="59" t="inlineStr"/>
+      <c r="B12" s="59" t="inlineStr"/>
+      <c r="C12" s="59" t="inlineStr"/>
+      <c r="D12" s="59" t="inlineStr"/>
+      <c r="E12" s="59" t="inlineStr"/>
+      <c r="F12" s="59" t="inlineStr"/>
+      <c r="G12" s="59" t="inlineStr"/>
+      <c r="H12" s="59" t="inlineStr"/>
+      <c r="I12" s="59" t="inlineStr"/>
+      <c r="J12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="63" t="n">
+      <c r="K12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="62">
+      <c r="L12" s="60">
         <f>K12-J12</f>
         <v/>
       </c>
-      <c r="M12" s="64">
+      <c r="M12" s="62">
         <f>IF(J12=0,"",(K12-J12)/J12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="65" t="inlineStr"/>
-      <c r="B13" s="65" t="inlineStr"/>
-      <c r="C13" s="65" t="inlineStr"/>
-      <c r="D13" s="65" t="inlineStr"/>
-      <c r="E13" s="65" t="inlineStr"/>
-      <c r="F13" s="65" t="inlineStr"/>
-      <c r="G13" s="65" t="inlineStr"/>
-      <c r="H13" s="65" t="inlineStr"/>
-      <c r="I13" s="65" t="inlineStr"/>
-      <c r="J13" s="63" t="n">
+      <c r="A13" s="63" t="inlineStr"/>
+      <c r="B13" s="63" t="inlineStr"/>
+      <c r="C13" s="63" t="inlineStr"/>
+      <c r="D13" s="63" t="inlineStr"/>
+      <c r="E13" s="63" t="inlineStr"/>
+      <c r="F13" s="63" t="inlineStr"/>
+      <c r="G13" s="63" t="inlineStr"/>
+      <c r="H13" s="63" t="inlineStr"/>
+      <c r="I13" s="63" t="inlineStr"/>
+      <c r="J13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="63" t="n">
+      <c r="K13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="66">
+      <c r="L13" s="64">
         <f>K13-J13</f>
         <v/>
       </c>
-      <c r="M13" s="67">
+      <c r="M13" s="65">
         <f>IF(J13=0,"",(K13-J13)/J13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="68" t="inlineStr">
+      <c r="A14" s="66" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="68" t="n"/>
-      <c r="C14" s="68" t="n"/>
-      <c r="D14" s="68" t="n"/>
-      <c r="E14" s="68" t="n"/>
-      <c r="F14" s="68" t="n"/>
-      <c r="G14" s="68" t="n"/>
-      <c r="H14" s="68" t="n"/>
-      <c r="I14" s="68" t="n"/>
-      <c r="J14" s="32">
+      <c r="B14" s="66" t="n"/>
+      <c r="C14" s="66" t="n"/>
+      <c r="D14" s="66" t="n"/>
+      <c r="E14" s="66" t="n"/>
+      <c r="F14" s="66" t="n"/>
+      <c r="G14" s="66" t="n"/>
+      <c r="H14" s="66" t="n"/>
+      <c r="I14" s="66" t="n"/>
+      <c r="J14" s="30">
         <f>SUM(J6:J13)</f>
         <v/>
       </c>
-      <c r="K14" s="32">
+      <c r="K14" s="30">
         <f>SUM(K6:K13)</f>
         <v/>
       </c>
-      <c r="L14" s="32">
+      <c r="L14" s="30">
         <f>K14-J14</f>
         <v/>
       </c>
-      <c r="M14" s="33">
+      <c r="M14" s="31">
         <f>IF(J14=0,"",(K14-J14)/J14)</f>
         <v/>
       </c>
@@ -13194,299 +13239,299 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Nombre del deudor</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Tipo de deudor</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>N. de identificacion</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Partes relacionadas</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="J5" s="27" t="inlineStr">
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="K5" s="27" t="inlineStr">
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="L5" s="27" t="inlineStr">
+      <c r="L5" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="M5" s="27" t="inlineStr">
+      <c r="M5" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr"/>
-      <c r="B6" s="61" t="inlineStr"/>
-      <c r="C6" s="61" t="inlineStr"/>
-      <c r="D6" s="61" t="inlineStr"/>
-      <c r="E6" s="61" t="inlineStr"/>
-      <c r="F6" s="61" t="inlineStr"/>
-      <c r="G6" s="61" t="inlineStr"/>
-      <c r="H6" s="61" t="inlineStr"/>
-      <c r="I6" s="61" t="inlineStr"/>
-      <c r="J6" s="63" t="n">
+      <c r="A6" s="59" t="inlineStr"/>
+      <c r="B6" s="59" t="inlineStr"/>
+      <c r="C6" s="59" t="inlineStr"/>
+      <c r="D6" s="59" t="inlineStr"/>
+      <c r="E6" s="59" t="inlineStr"/>
+      <c r="F6" s="59" t="inlineStr"/>
+      <c r="G6" s="59" t="inlineStr"/>
+      <c r="H6" s="59" t="inlineStr"/>
+      <c r="I6" s="59" t="inlineStr"/>
+      <c r="J6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="63" t="n">
+      <c r="K6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="62">
+      <c r="L6" s="60">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="64">
+      <c r="M6" s="62">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="65" t="inlineStr"/>
-      <c r="B7" s="65" t="inlineStr"/>
-      <c r="C7" s="65" t="inlineStr"/>
-      <c r="D7" s="65" t="inlineStr"/>
-      <c r="E7" s="65" t="inlineStr"/>
-      <c r="F7" s="65" t="inlineStr"/>
-      <c r="G7" s="65" t="inlineStr"/>
-      <c r="H7" s="65" t="inlineStr"/>
-      <c r="I7" s="65" t="inlineStr"/>
-      <c r="J7" s="63" t="n">
+      <c r="A7" s="63" t="inlineStr"/>
+      <c r="B7" s="63" t="inlineStr"/>
+      <c r="C7" s="63" t="inlineStr"/>
+      <c r="D7" s="63" t="inlineStr"/>
+      <c r="E7" s="63" t="inlineStr"/>
+      <c r="F7" s="63" t="inlineStr"/>
+      <c r="G7" s="63" t="inlineStr"/>
+      <c r="H7" s="63" t="inlineStr"/>
+      <c r="I7" s="63" t="inlineStr"/>
+      <c r="J7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="63" t="n">
+      <c r="K7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="66">
+      <c r="L7" s="64">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="67">
+      <c r="M7" s="65">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr"/>
-      <c r="B8" s="61" t="inlineStr"/>
-      <c r="C8" s="61" t="inlineStr"/>
-      <c r="D8" s="61" t="inlineStr"/>
-      <c r="E8" s="61" t="inlineStr"/>
-      <c r="F8" s="61" t="inlineStr"/>
-      <c r="G8" s="61" t="inlineStr"/>
-      <c r="H8" s="61" t="inlineStr"/>
-      <c r="I8" s="61" t="inlineStr"/>
-      <c r="J8" s="63" t="n">
+      <c r="A8" s="59" t="inlineStr"/>
+      <c r="B8" s="59" t="inlineStr"/>
+      <c r="C8" s="59" t="inlineStr"/>
+      <c r="D8" s="59" t="inlineStr"/>
+      <c r="E8" s="59" t="inlineStr"/>
+      <c r="F8" s="59" t="inlineStr"/>
+      <c r="G8" s="59" t="inlineStr"/>
+      <c r="H8" s="59" t="inlineStr"/>
+      <c r="I8" s="59" t="inlineStr"/>
+      <c r="J8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="63" t="n">
+      <c r="K8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="62">
+      <c r="L8" s="60">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="64">
+      <c r="M8" s="62">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="65" t="inlineStr"/>
-      <c r="B9" s="65" t="inlineStr"/>
-      <c r="C9" s="65" t="inlineStr"/>
-      <c r="D9" s="65" t="inlineStr"/>
-      <c r="E9" s="65" t="inlineStr"/>
-      <c r="F9" s="65" t="inlineStr"/>
-      <c r="G9" s="65" t="inlineStr"/>
-      <c r="H9" s="65" t="inlineStr"/>
-      <c r="I9" s="65" t="inlineStr"/>
-      <c r="J9" s="63" t="n">
+      <c r="A9" s="63" t="inlineStr"/>
+      <c r="B9" s="63" t="inlineStr"/>
+      <c r="C9" s="63" t="inlineStr"/>
+      <c r="D9" s="63" t="inlineStr"/>
+      <c r="E9" s="63" t="inlineStr"/>
+      <c r="F9" s="63" t="inlineStr"/>
+      <c r="G9" s="63" t="inlineStr"/>
+      <c r="H9" s="63" t="inlineStr"/>
+      <c r="I9" s="63" t="inlineStr"/>
+      <c r="J9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="63" t="n">
+      <c r="K9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="66">
+      <c r="L9" s="64">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="67">
+      <c r="M9" s="65">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr"/>
-      <c r="B10" s="61" t="inlineStr"/>
-      <c r="C10" s="61" t="inlineStr"/>
-      <c r="D10" s="61" t="inlineStr"/>
-      <c r="E10" s="61" t="inlineStr"/>
-      <c r="F10" s="61" t="inlineStr"/>
-      <c r="G10" s="61" t="inlineStr"/>
-      <c r="H10" s="61" t="inlineStr"/>
-      <c r="I10" s="61" t="inlineStr"/>
-      <c r="J10" s="63" t="n">
+      <c r="A10" s="59" t="inlineStr"/>
+      <c r="B10" s="59" t="inlineStr"/>
+      <c r="C10" s="59" t="inlineStr"/>
+      <c r="D10" s="59" t="inlineStr"/>
+      <c r="E10" s="59" t="inlineStr"/>
+      <c r="F10" s="59" t="inlineStr"/>
+      <c r="G10" s="59" t="inlineStr"/>
+      <c r="H10" s="59" t="inlineStr"/>
+      <c r="I10" s="59" t="inlineStr"/>
+      <c r="J10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="63" t="n">
+      <c r="K10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="62">
+      <c r="L10" s="60">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="64">
+      <c r="M10" s="62">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="65" t="inlineStr"/>
-      <c r="B11" s="65" t="inlineStr"/>
-      <c r="C11" s="65" t="inlineStr"/>
-      <c r="D11" s="65" t="inlineStr"/>
-      <c r="E11" s="65" t="inlineStr"/>
-      <c r="F11" s="65" t="inlineStr"/>
-      <c r="G11" s="65" t="inlineStr"/>
-      <c r="H11" s="65" t="inlineStr"/>
-      <c r="I11" s="65" t="inlineStr"/>
-      <c r="J11" s="63" t="n">
+      <c r="A11" s="63" t="inlineStr"/>
+      <c r="B11" s="63" t="inlineStr"/>
+      <c r="C11" s="63" t="inlineStr"/>
+      <c r="D11" s="63" t="inlineStr"/>
+      <c r="E11" s="63" t="inlineStr"/>
+      <c r="F11" s="63" t="inlineStr"/>
+      <c r="G11" s="63" t="inlineStr"/>
+      <c r="H11" s="63" t="inlineStr"/>
+      <c r="I11" s="63" t="inlineStr"/>
+      <c r="J11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="63" t="n">
+      <c r="K11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="66">
+      <c r="L11" s="64">
         <f>K11-J11</f>
         <v/>
       </c>
-      <c r="M11" s="67">
+      <c r="M11" s="65">
         <f>IF(J11=0,"",(K11-J11)/J11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr"/>
-      <c r="B12" s="61" t="inlineStr"/>
-      <c r="C12" s="61" t="inlineStr"/>
-      <c r="D12" s="61" t="inlineStr"/>
-      <c r="E12" s="61" t="inlineStr"/>
-      <c r="F12" s="61" t="inlineStr"/>
-      <c r="G12" s="61" t="inlineStr"/>
-      <c r="H12" s="61" t="inlineStr"/>
-      <c r="I12" s="61" t="inlineStr"/>
-      <c r="J12" s="63" t="n">
+      <c r="A12" s="59" t="inlineStr"/>
+      <c r="B12" s="59" t="inlineStr"/>
+      <c r="C12" s="59" t="inlineStr"/>
+      <c r="D12" s="59" t="inlineStr"/>
+      <c r="E12" s="59" t="inlineStr"/>
+      <c r="F12" s="59" t="inlineStr"/>
+      <c r="G12" s="59" t="inlineStr"/>
+      <c r="H12" s="59" t="inlineStr"/>
+      <c r="I12" s="59" t="inlineStr"/>
+      <c r="J12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="63" t="n">
+      <c r="K12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="62">
+      <c r="L12" s="60">
         <f>K12-J12</f>
         <v/>
       </c>
-      <c r="M12" s="64">
+      <c r="M12" s="62">
         <f>IF(J12=0,"",(K12-J12)/J12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="65" t="inlineStr"/>
-      <c r="B13" s="65" t="inlineStr"/>
-      <c r="C13" s="65" t="inlineStr"/>
-      <c r="D13" s="65" t="inlineStr"/>
-      <c r="E13" s="65" t="inlineStr"/>
-      <c r="F13" s="65" t="inlineStr"/>
-      <c r="G13" s="65" t="inlineStr"/>
-      <c r="H13" s="65" t="inlineStr"/>
-      <c r="I13" s="65" t="inlineStr"/>
-      <c r="J13" s="63" t="n">
+      <c r="A13" s="63" t="inlineStr"/>
+      <c r="B13" s="63" t="inlineStr"/>
+      <c r="C13" s="63" t="inlineStr"/>
+      <c r="D13" s="63" t="inlineStr"/>
+      <c r="E13" s="63" t="inlineStr"/>
+      <c r="F13" s="63" t="inlineStr"/>
+      <c r="G13" s="63" t="inlineStr"/>
+      <c r="H13" s="63" t="inlineStr"/>
+      <c r="I13" s="63" t="inlineStr"/>
+      <c r="J13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="63" t="n">
+      <c r="K13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="66">
+      <c r="L13" s="64">
         <f>K13-J13</f>
         <v/>
       </c>
-      <c r="M13" s="67">
+      <c r="M13" s="65">
         <f>IF(J13=0,"",(K13-J13)/J13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="68" t="inlineStr">
+      <c r="A14" s="66" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="68" t="n"/>
-      <c r="C14" s="68" t="n"/>
-      <c r="D14" s="68" t="n"/>
-      <c r="E14" s="68" t="n"/>
-      <c r="F14" s="68" t="n"/>
-      <c r="G14" s="68" t="n"/>
-      <c r="H14" s="68" t="n"/>
-      <c r="I14" s="68" t="n"/>
-      <c r="J14" s="32">
+      <c r="B14" s="66" t="n"/>
+      <c r="C14" s="66" t="n"/>
+      <c r="D14" s="66" t="n"/>
+      <c r="E14" s="66" t="n"/>
+      <c r="F14" s="66" t="n"/>
+      <c r="G14" s="66" t="n"/>
+      <c r="H14" s="66" t="n"/>
+      <c r="I14" s="66" t="n"/>
+      <c r="J14" s="30">
         <f>SUM(J6:J13)</f>
         <v/>
       </c>
-      <c r="K14" s="32">
+      <c r="K14" s="30">
         <f>SUM(K6:K13)</f>
         <v/>
       </c>
-      <c r="L14" s="32">
+      <c r="L14" s="30">
         <f>K14-J14</f>
         <v/>
       </c>
-      <c r="M14" s="33">
+      <c r="M14" s="31">
         <f>IF(J14=0,"",(K14-J14)/J14)</f>
         <v/>
       </c>
@@ -13559,243 +13604,243 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Tipo de bien</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr"/>
-      <c r="B6" s="61" t="inlineStr"/>
-      <c r="C6" s="61" t="inlineStr"/>
-      <c r="D6" s="61" t="inlineStr"/>
-      <c r="E6" s="61" t="inlineStr"/>
-      <c r="F6" s="63" t="n">
+      <c r="A6" s="59" t="inlineStr"/>
+      <c r="B6" s="59" t="inlineStr"/>
+      <c r="C6" s="59" t="inlineStr"/>
+      <c r="D6" s="59" t="inlineStr"/>
+      <c r="E6" s="59" t="inlineStr"/>
+      <c r="F6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="63" t="n">
+      <c r="G6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="62">
+      <c r="H6" s="60">
         <f>G6-F6</f>
         <v/>
       </c>
-      <c r="I6" s="64">
+      <c r="I6" s="62">
         <f>IF(F6=0,"",(G6-F6)/F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="65" t="inlineStr"/>
-      <c r="B7" s="65" t="inlineStr"/>
-      <c r="C7" s="65" t="inlineStr"/>
-      <c r="D7" s="65" t="inlineStr"/>
-      <c r="E7" s="65" t="inlineStr"/>
-      <c r="F7" s="63" t="n">
+      <c r="A7" s="63" t="inlineStr"/>
+      <c r="B7" s="63" t="inlineStr"/>
+      <c r="C7" s="63" t="inlineStr"/>
+      <c r="D7" s="63" t="inlineStr"/>
+      <c r="E7" s="63" t="inlineStr"/>
+      <c r="F7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="63" t="n">
+      <c r="G7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="66">
+      <c r="H7" s="64">
         <f>G7-F7</f>
         <v/>
       </c>
-      <c r="I7" s="67">
+      <c r="I7" s="65">
         <f>IF(F7=0,"",(G7-F7)/F7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr"/>
-      <c r="B8" s="61" t="inlineStr"/>
-      <c r="C8" s="61" t="inlineStr"/>
-      <c r="D8" s="61" t="inlineStr"/>
-      <c r="E8" s="61" t="inlineStr"/>
-      <c r="F8" s="63" t="n">
+      <c r="A8" s="59" t="inlineStr"/>
+      <c r="B8" s="59" t="inlineStr"/>
+      <c r="C8" s="59" t="inlineStr"/>
+      <c r="D8" s="59" t="inlineStr"/>
+      <c r="E8" s="59" t="inlineStr"/>
+      <c r="F8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="63" t="n">
+      <c r="G8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="62">
+      <c r="H8" s="60">
         <f>G8-F8</f>
         <v/>
       </c>
-      <c r="I8" s="64">
+      <c r="I8" s="62">
         <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="65" t="inlineStr"/>
-      <c r="B9" s="65" t="inlineStr"/>
-      <c r="C9" s="65" t="inlineStr"/>
-      <c r="D9" s="65" t="inlineStr"/>
-      <c r="E9" s="65" t="inlineStr"/>
-      <c r="F9" s="63" t="n">
+      <c r="A9" s="63" t="inlineStr"/>
+      <c r="B9" s="63" t="inlineStr"/>
+      <c r="C9" s="63" t="inlineStr"/>
+      <c r="D9" s="63" t="inlineStr"/>
+      <c r="E9" s="63" t="inlineStr"/>
+      <c r="F9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="63" t="n">
+      <c r="G9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="66">
+      <c r="H9" s="64">
         <f>G9-F9</f>
         <v/>
       </c>
-      <c r="I9" s="67">
+      <c r="I9" s="65">
         <f>IF(F9=0,"",(G9-F9)/F9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr"/>
-      <c r="B10" s="61" t="inlineStr"/>
-      <c r="C10" s="61" t="inlineStr"/>
-      <c r="D10" s="61" t="inlineStr"/>
-      <c r="E10" s="61" t="inlineStr"/>
-      <c r="F10" s="63" t="n">
+      <c r="A10" s="59" t="inlineStr"/>
+      <c r="B10" s="59" t="inlineStr"/>
+      <c r="C10" s="59" t="inlineStr"/>
+      <c r="D10" s="59" t="inlineStr"/>
+      <c r="E10" s="59" t="inlineStr"/>
+      <c r="F10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="63" t="n">
+      <c r="G10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="62">
+      <c r="H10" s="60">
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="64">
+      <c r="I10" s="62">
         <f>IF(F10=0,"",(G10-F10)/F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="65" t="inlineStr"/>
-      <c r="B11" s="65" t="inlineStr"/>
-      <c r="C11" s="65" t="inlineStr"/>
-      <c r="D11" s="65" t="inlineStr"/>
-      <c r="E11" s="65" t="inlineStr"/>
-      <c r="F11" s="63" t="n">
+      <c r="A11" s="63" t="inlineStr"/>
+      <c r="B11" s="63" t="inlineStr"/>
+      <c r="C11" s="63" t="inlineStr"/>
+      <c r="D11" s="63" t="inlineStr"/>
+      <c r="E11" s="63" t="inlineStr"/>
+      <c r="F11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="63" t="n">
+      <c r="G11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="66">
+      <c r="H11" s="64">
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="67">
+      <c r="I11" s="65">
         <f>IF(F11=0,"",(G11-F11)/F11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr"/>
-      <c r="B12" s="61" t="inlineStr"/>
-      <c r="C12" s="61" t="inlineStr"/>
-      <c r="D12" s="61" t="inlineStr"/>
-      <c r="E12" s="61" t="inlineStr"/>
-      <c r="F12" s="63" t="n">
+      <c r="A12" s="59" t="inlineStr"/>
+      <c r="B12" s="59" t="inlineStr"/>
+      <c r="C12" s="59" t="inlineStr"/>
+      <c r="D12" s="59" t="inlineStr"/>
+      <c r="E12" s="59" t="inlineStr"/>
+      <c r="F12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="63" t="n">
+      <c r="G12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="62">
+      <c r="H12" s="60">
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="64">
+      <c r="I12" s="62">
         <f>IF(F12=0,"",(G12-F12)/F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="65" t="inlineStr"/>
-      <c r="B13" s="65" t="inlineStr"/>
-      <c r="C13" s="65" t="inlineStr"/>
-      <c r="D13" s="65" t="inlineStr"/>
-      <c r="E13" s="65" t="inlineStr"/>
-      <c r="F13" s="63" t="n">
+      <c r="A13" s="63" t="inlineStr"/>
+      <c r="B13" s="63" t="inlineStr"/>
+      <c r="C13" s="63" t="inlineStr"/>
+      <c r="D13" s="63" t="inlineStr"/>
+      <c r="E13" s="63" t="inlineStr"/>
+      <c r="F13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="63" t="n">
+      <c r="G13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="66">
+      <c r="H13" s="64">
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="67">
+      <c r="I13" s="65">
         <f>IF(F13=0,"",(G13-F13)/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="68" t="inlineStr">
+      <c r="A14" s="66" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="68" t="n"/>
-      <c r="C14" s="68" t="n"/>
-      <c r="D14" s="68" t="n"/>
-      <c r="E14" s="68" t="n"/>
-      <c r="F14" s="32">
+      <c r="B14" s="66" t="n"/>
+      <c r="C14" s="66" t="n"/>
+      <c r="D14" s="66" t="n"/>
+      <c r="E14" s="66" t="n"/>
+      <c r="F14" s="30">
         <f>SUM(F6:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="32">
+      <c r="G14" s="30">
         <f>SUM(G6:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="32">
+      <c r="H14" s="30">
         <f>G14-F14</f>
         <v/>
       </c>
-      <c r="I14" s="33">
+      <c r="I14" s="31">
         <f>IF(F14=0,"",(G14-F14)/F14)</f>
         <v/>
       </c>
@@ -13863,195 +13908,195 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Tipo de vehiculo</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Registro / placa / chasis</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="J5" s="27" t="inlineStr">
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr">
+      <c r="A6" s="59" t="inlineStr">
         <is>
           <t>1 - Vehiculos motorizados terrestres</t>
         </is>
       </c>
-      <c r="B6" s="61" t="inlineStr">
+      <c r="B6" s="59" t="inlineStr">
         <is>
           <t>PBO7092</t>
         </is>
       </c>
-      <c r="C6" s="61" t="inlineStr">
+      <c r="C6" s="59" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D6" s="61" t="inlineStr">
+      <c r="D6" s="59" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E6" s="61" t="inlineStr"/>
-      <c r="F6" s="61" t="inlineStr"/>
-      <c r="G6" s="62" t="n">
+      <c r="E6" s="59" t="inlineStr"/>
+      <c r="F6" s="59" t="inlineStr"/>
+      <c r="G6" s="60" t="n">
         <v>12000</v>
       </c>
-      <c r="H6" s="63" t="n">
+      <c r="H6" s="61" t="n">
         <v>12000</v>
       </c>
-      <c r="I6" s="62">
+      <c r="I6" s="60">
         <f>H6-G6</f>
         <v/>
       </c>
-      <c r="J6" s="64">
+      <c r="J6" s="62">
         <f>IF(G6=0,"",(H6-G6)/G6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="65" t="inlineStr">
+      <c r="A7" s="63" t="inlineStr">
         <is>
           <t>1 - Vehiculos motorizados terrestres</t>
         </is>
       </c>
-      <c r="B7" s="65" t="inlineStr">
+      <c r="B7" s="63" t="inlineStr">
         <is>
           <t>PBF9690</t>
         </is>
       </c>
-      <c r="C7" s="65" t="inlineStr">
+      <c r="C7" s="63" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D7" s="65" t="inlineStr">
+      <c r="D7" s="63" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E7" s="65" t="inlineStr"/>
-      <c r="F7" s="65" t="inlineStr"/>
-      <c r="G7" s="66" t="n">
+      <c r="E7" s="63" t="inlineStr"/>
+      <c r="F7" s="63" t="inlineStr"/>
+      <c r="G7" s="64" t="n">
         <v>20000</v>
       </c>
-      <c r="H7" s="63" t="n">
+      <c r="H7" s="61" t="n">
         <v>20000</v>
       </c>
-      <c r="I7" s="66">
+      <c r="I7" s="64">
         <f>H7-G7</f>
         <v/>
       </c>
-      <c r="J7" s="67">
+      <c r="J7" s="65">
         <f>IF(G7=0,"",(H7-G7)/G7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="59" t="inlineStr">
         <is>
           <t>1 - Vehiculos motorizados terrestres</t>
         </is>
       </c>
-      <c r="B8" s="61" t="inlineStr">
+      <c r="B8" s="59" t="inlineStr">
         <is>
           <t>PFC8683</t>
         </is>
       </c>
-      <c r="C8" s="61" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D8" s="61" t="inlineStr">
+      <c r="D8" s="59" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E8" s="61" t="inlineStr"/>
-      <c r="F8" s="61" t="inlineStr"/>
-      <c r="G8" s="62" t="n">
+      <c r="E8" s="59" t="inlineStr"/>
+      <c r="F8" s="59" t="inlineStr"/>
+      <c r="G8" s="60" t="n">
         <v>32000</v>
       </c>
-      <c r="H8" s="63" t="n">
+      <c r="H8" s="61" t="n">
         <v>32000</v>
       </c>
-      <c r="I8" s="62">
+      <c r="I8" s="60">
         <f>H8-G8</f>
         <v/>
       </c>
-      <c r="J8" s="64">
+      <c r="J8" s="62">
         <f>IF(G8=0,"",(H8-G8)/G8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="68" t="inlineStr">
+      <c r="A9" s="66" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="68" t="n"/>
-      <c r="C9" s="68" t="n"/>
-      <c r="D9" s="68" t="n"/>
-      <c r="E9" s="68" t="n"/>
-      <c r="F9" s="68" t="n"/>
-      <c r="G9" s="32">
+      <c r="B9" s="66" t="n"/>
+      <c r="C9" s="66" t="n"/>
+      <c r="D9" s="66" t="n"/>
+      <c r="E9" s="66" t="n"/>
+      <c r="F9" s="66" t="n"/>
+      <c r="G9" s="30">
         <f>SUM(G6:G8)</f>
         <v/>
       </c>
-      <c r="H9" s="32">
+      <c r="H9" s="30">
         <f>SUM(H6:H8)</f>
         <v/>
       </c>
-      <c r="I9" s="32">
+      <c r="I9" s="30">
         <f>H9-G9</f>
         <v/>
       </c>
-      <c r="J9" s="33">
+      <c r="J9" s="31">
         <f>IF(G9=0,"",(H9-G9)/G9)</f>
         <v/>
       </c>
@@ -14118,243 +14163,243 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Tipo de derecho</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr"/>
-      <c r="B6" s="61" t="inlineStr"/>
-      <c r="C6" s="61" t="inlineStr"/>
-      <c r="D6" s="61" t="inlineStr"/>
-      <c r="E6" s="61" t="inlineStr"/>
-      <c r="F6" s="63" t="n">
+      <c r="A6" s="59" t="inlineStr"/>
+      <c r="B6" s="59" t="inlineStr"/>
+      <c r="C6" s="59" t="inlineStr"/>
+      <c r="D6" s="59" t="inlineStr"/>
+      <c r="E6" s="59" t="inlineStr"/>
+      <c r="F6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="63" t="n">
+      <c r="G6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="62">
+      <c r="H6" s="60">
         <f>G6-F6</f>
         <v/>
       </c>
-      <c r="I6" s="64">
+      <c r="I6" s="62">
         <f>IF(F6=0,"",(G6-F6)/F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="65" t="inlineStr"/>
-      <c r="B7" s="65" t="inlineStr"/>
-      <c r="C7" s="65" t="inlineStr"/>
-      <c r="D7" s="65" t="inlineStr"/>
-      <c r="E7" s="65" t="inlineStr"/>
-      <c r="F7" s="63" t="n">
+      <c r="A7" s="63" t="inlineStr"/>
+      <c r="B7" s="63" t="inlineStr"/>
+      <c r="C7" s="63" t="inlineStr"/>
+      <c r="D7" s="63" t="inlineStr"/>
+      <c r="E7" s="63" t="inlineStr"/>
+      <c r="F7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="63" t="n">
+      <c r="G7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="66">
+      <c r="H7" s="64">
         <f>G7-F7</f>
         <v/>
       </c>
-      <c r="I7" s="67">
+      <c r="I7" s="65">
         <f>IF(F7=0,"",(G7-F7)/F7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr"/>
-      <c r="B8" s="61" t="inlineStr"/>
-      <c r="C8" s="61" t="inlineStr"/>
-      <c r="D8" s="61" t="inlineStr"/>
-      <c r="E8" s="61" t="inlineStr"/>
-      <c r="F8" s="63" t="n">
+      <c r="A8" s="59" t="inlineStr"/>
+      <c r="B8" s="59" t="inlineStr"/>
+      <c r="C8" s="59" t="inlineStr"/>
+      <c r="D8" s="59" t="inlineStr"/>
+      <c r="E8" s="59" t="inlineStr"/>
+      <c r="F8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="63" t="n">
+      <c r="G8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="62">
+      <c r="H8" s="60">
         <f>G8-F8</f>
         <v/>
       </c>
-      <c r="I8" s="64">
+      <c r="I8" s="62">
         <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="65" t="inlineStr"/>
-      <c r="B9" s="65" t="inlineStr"/>
-      <c r="C9" s="65" t="inlineStr"/>
-      <c r="D9" s="65" t="inlineStr"/>
-      <c r="E9" s="65" t="inlineStr"/>
-      <c r="F9" s="63" t="n">
+      <c r="A9" s="63" t="inlineStr"/>
+      <c r="B9" s="63" t="inlineStr"/>
+      <c r="C9" s="63" t="inlineStr"/>
+      <c r="D9" s="63" t="inlineStr"/>
+      <c r="E9" s="63" t="inlineStr"/>
+      <c r="F9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="63" t="n">
+      <c r="G9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="66">
+      <c r="H9" s="64">
         <f>G9-F9</f>
         <v/>
       </c>
-      <c r="I9" s="67">
+      <c r="I9" s="65">
         <f>IF(F9=0,"",(G9-F9)/F9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr"/>
-      <c r="B10" s="61" t="inlineStr"/>
-      <c r="C10" s="61" t="inlineStr"/>
-      <c r="D10" s="61" t="inlineStr"/>
-      <c r="E10" s="61" t="inlineStr"/>
-      <c r="F10" s="63" t="n">
+      <c r="A10" s="59" t="inlineStr"/>
+      <c r="B10" s="59" t="inlineStr"/>
+      <c r="C10" s="59" t="inlineStr"/>
+      <c r="D10" s="59" t="inlineStr"/>
+      <c r="E10" s="59" t="inlineStr"/>
+      <c r="F10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="63" t="n">
+      <c r="G10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="62">
+      <c r="H10" s="60">
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="64">
+      <c r="I10" s="62">
         <f>IF(F10=0,"",(G10-F10)/F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="65" t="inlineStr"/>
-      <c r="B11" s="65" t="inlineStr"/>
-      <c r="C11" s="65" t="inlineStr"/>
-      <c r="D11" s="65" t="inlineStr"/>
-      <c r="E11" s="65" t="inlineStr"/>
-      <c r="F11" s="63" t="n">
+      <c r="A11" s="63" t="inlineStr"/>
+      <c r="B11" s="63" t="inlineStr"/>
+      <c r="C11" s="63" t="inlineStr"/>
+      <c r="D11" s="63" t="inlineStr"/>
+      <c r="E11" s="63" t="inlineStr"/>
+      <c r="F11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="63" t="n">
+      <c r="G11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="66">
+      <c r="H11" s="64">
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="67">
+      <c r="I11" s="65">
         <f>IF(F11=0,"",(G11-F11)/F11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr"/>
-      <c r="B12" s="61" t="inlineStr"/>
-      <c r="C12" s="61" t="inlineStr"/>
-      <c r="D12" s="61" t="inlineStr"/>
-      <c r="E12" s="61" t="inlineStr"/>
-      <c r="F12" s="63" t="n">
+      <c r="A12" s="59" t="inlineStr"/>
+      <c r="B12" s="59" t="inlineStr"/>
+      <c r="C12" s="59" t="inlineStr"/>
+      <c r="D12" s="59" t="inlineStr"/>
+      <c r="E12" s="59" t="inlineStr"/>
+      <c r="F12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="63" t="n">
+      <c r="G12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="62">
+      <c r="H12" s="60">
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="64">
+      <c r="I12" s="62">
         <f>IF(F12=0,"",(G12-F12)/F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="65" t="inlineStr"/>
-      <c r="B13" s="65" t="inlineStr"/>
-      <c r="C13" s="65" t="inlineStr"/>
-      <c r="D13" s="65" t="inlineStr"/>
-      <c r="E13" s="65" t="inlineStr"/>
-      <c r="F13" s="63" t="n">
+      <c r="A13" s="63" t="inlineStr"/>
+      <c r="B13" s="63" t="inlineStr"/>
+      <c r="C13" s="63" t="inlineStr"/>
+      <c r="D13" s="63" t="inlineStr"/>
+      <c r="E13" s="63" t="inlineStr"/>
+      <c r="F13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="63" t="n">
+      <c r="G13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="66">
+      <c r="H13" s="64">
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="67">
+      <c r="I13" s="65">
         <f>IF(F13=0,"",(G13-F13)/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="68" t="inlineStr">
+      <c r="A14" s="66" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="68" t="n"/>
-      <c r="C14" s="68" t="n"/>
-      <c r="D14" s="68" t="n"/>
-      <c r="E14" s="68" t="n"/>
-      <c r="F14" s="32">
+      <c r="B14" s="66" t="n"/>
+      <c r="C14" s="66" t="n"/>
+      <c r="D14" s="66" t="n"/>
+      <c r="E14" s="66" t="n"/>
+      <c r="F14" s="30">
         <f>SUM(F6:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="32">
+      <c r="G14" s="30">
         <f>SUM(G6:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="32">
+      <c r="H14" s="30">
         <f>G14-F14</f>
         <v/>
       </c>
-      <c r="I14" s="33">
+      <c r="I14" s="31">
         <f>IF(F14=0,"",(G14-F14)/F14)</f>
         <v/>
       </c>
@@ -14425,303 +14470,303 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Tipo de inmueble</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Provincia</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Canton</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Fecha de inscripcion</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Clave catastral</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="J5" s="27" t="inlineStr">
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="K5" s="27" t="inlineStr">
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="L5" s="27" t="inlineStr">
+      <c r="L5" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="M5" s="27" t="inlineStr">
+      <c r="M5" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr">
+      <c r="A6" s="59" t="inlineStr">
         <is>
           <t>3 - Terreno</t>
         </is>
       </c>
-      <c r="B6" s="61" t="inlineStr">
+      <c r="B6" s="59" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C6" s="61" t="inlineStr">
+      <c r="C6" s="59" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D6" s="61" t="inlineStr">
+      <c r="D6" s="59" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E6" s="61" t="inlineStr">
+      <c r="E6" s="59" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F6" s="61" t="inlineStr">
+      <c r="F6" s="59" t="inlineStr">
         <is>
           <t>22/10/2008</t>
         </is>
       </c>
-      <c r="G6" s="61" t="inlineStr">
+      <c r="G6" s="59" t="inlineStr">
         <is>
           <t>1042203018</t>
         </is>
       </c>
-      <c r="H6" s="61" t="inlineStr"/>
-      <c r="I6" s="61" t="inlineStr"/>
-      <c r="J6" s="62" t="n">
+      <c r="H6" s="59" t="inlineStr"/>
+      <c r="I6" s="59" t="inlineStr"/>
+      <c r="J6" s="60" t="n">
         <v>267340.8</v>
       </c>
-      <c r="K6" s="63" t="n">
+      <c r="K6" s="61" t="n">
         <v>267340.8</v>
       </c>
-      <c r="L6" s="62">
+      <c r="L6" s="60">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="64">
+      <c r="M6" s="62">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="65" t="inlineStr">
+      <c r="A7" s="63" t="inlineStr">
         <is>
           <t>1 - Casa</t>
         </is>
       </c>
-      <c r="B7" s="65" t="inlineStr">
+      <c r="B7" s="63" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C7" s="65" t="inlineStr">
+      <c r="C7" s="63" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D7" s="65" t="inlineStr">
+      <c r="D7" s="63" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E7" s="65" t="inlineStr">
+      <c r="E7" s="63" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F7" s="65" t="inlineStr">
+      <c r="F7" s="63" t="inlineStr">
         <is>
           <t>13/03/1997</t>
         </is>
       </c>
-      <c r="G7" s="65" t="inlineStr">
+      <c r="G7" s="63" t="inlineStr">
         <is>
           <t>1012005008000000000</t>
         </is>
       </c>
-      <c r="H7" s="65" t="inlineStr"/>
-      <c r="I7" s="65" t="inlineStr"/>
-      <c r="J7" s="66" t="n">
+      <c r="H7" s="63" t="inlineStr"/>
+      <c r="I7" s="63" t="inlineStr"/>
+      <c r="J7" s="64" t="n">
         <v>198118.55</v>
       </c>
-      <c r="K7" s="63" t="n">
+      <c r="K7" s="61" t="n">
         <v>198118.55</v>
       </c>
-      <c r="L7" s="66">
+      <c r="L7" s="64">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="67">
+      <c r="M7" s="65">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="59" t="inlineStr">
         <is>
           <t>1 - Casa</t>
         </is>
       </c>
-      <c r="B8" s="61" t="inlineStr">
+      <c r="B8" s="59" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C8" s="61" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D8" s="61" t="inlineStr">
+      <c r="D8" s="59" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E8" s="61" t="inlineStr">
+      <c r="E8" s="59" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F8" s="61" t="inlineStr"/>
-      <c r="G8" s="61" t="inlineStr">
+      <c r="F8" s="59" t="inlineStr"/>
+      <c r="G8" s="59" t="inlineStr">
         <is>
           <t>1042203018</t>
         </is>
       </c>
-      <c r="H8" s="61" t="inlineStr"/>
-      <c r="I8" s="61" t="inlineStr"/>
-      <c r="J8" s="62" t="n">
+      <c r="H8" s="59" t="inlineStr"/>
+      <c r="I8" s="59" t="inlineStr"/>
+      <c r="J8" s="60" t="n">
         <v>33634.04</v>
       </c>
-      <c r="K8" s="63" t="n">
+      <c r="K8" s="61" t="n">
         <v>33634.04</v>
       </c>
-      <c r="L8" s="62">
+      <c r="L8" s="60">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="64">
+      <c r="M8" s="62">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="65" t="inlineStr">
+      <c r="A9" s="63" t="inlineStr">
         <is>
           <t>3 - Terreno</t>
         </is>
       </c>
-      <c r="B9" s="65" t="inlineStr">
+      <c r="B9" s="63" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C9" s="65" t="inlineStr">
+      <c r="C9" s="63" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D9" s="65" t="inlineStr">
+      <c r="D9" s="63" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E9" s="65" t="inlineStr">
+      <c r="E9" s="63" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F9" s="65" t="inlineStr"/>
-      <c r="G9" s="65" t="inlineStr">
+      <c r="F9" s="63" t="inlineStr"/>
+      <c r="G9" s="63" t="inlineStr">
         <is>
           <t>1012005008000000000</t>
         </is>
       </c>
-      <c r="H9" s="65" t="inlineStr"/>
-      <c r="I9" s="65" t="inlineStr"/>
-      <c r="J9" s="66" t="n">
+      <c r="H9" s="63" t="inlineStr"/>
+      <c r="I9" s="63" t="inlineStr"/>
+      <c r="J9" s="64" t="n">
         <v>82624.22</v>
       </c>
-      <c r="K9" s="63" t="n">
+      <c r="K9" s="61" t="n">
         <v>82624.22</v>
       </c>
-      <c r="L9" s="66">
+      <c r="L9" s="64">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="67">
+      <c r="M9" s="65">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="68" t="inlineStr">
+      <c r="A10" s="66" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B10" s="68" t="n"/>
-      <c r="C10" s="68" t="n"/>
-      <c r="D10" s="68" t="n"/>
-      <c r="E10" s="68" t="n"/>
-      <c r="F10" s="68" t="n"/>
-      <c r="G10" s="68" t="n"/>
-      <c r="H10" s="68" t="n"/>
-      <c r="I10" s="68" t="n"/>
-      <c r="J10" s="32">
+      <c r="B10" s="66" t="n"/>
+      <c r="C10" s="66" t="n"/>
+      <c r="D10" s="66" t="n"/>
+      <c r="E10" s="66" t="n"/>
+      <c r="F10" s="66" t="n"/>
+      <c r="G10" s="66" t="n"/>
+      <c r="H10" s="66" t="n"/>
+      <c r="I10" s="66" t="n"/>
+      <c r="J10" s="30">
         <f>SUM(J6:J9)</f>
         <v/>
       </c>
-      <c r="K10" s="32">
+      <c r="K10" s="30">
         <f>SUM(K6:K9)</f>
         <v/>
       </c>
-      <c r="L10" s="32">
+      <c r="L10" s="30">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="33">
+      <c r="M10" s="31">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
@@ -14794,243 +14839,243 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Descripcion</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr"/>
-      <c r="B6" s="61" t="inlineStr"/>
-      <c r="C6" s="61" t="inlineStr"/>
-      <c r="D6" s="61" t="inlineStr"/>
-      <c r="E6" s="61" t="inlineStr"/>
-      <c r="F6" s="63" t="n">
+      <c r="A6" s="59" t="inlineStr"/>
+      <c r="B6" s="59" t="inlineStr"/>
+      <c r="C6" s="59" t="inlineStr"/>
+      <c r="D6" s="59" t="inlineStr"/>
+      <c r="E6" s="59" t="inlineStr"/>
+      <c r="F6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="63" t="n">
+      <c r="G6" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="62">
+      <c r="H6" s="60">
         <f>G6-F6</f>
         <v/>
       </c>
-      <c r="I6" s="64">
+      <c r="I6" s="62">
         <f>IF(F6=0,"",(G6-F6)/F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="65" t="inlineStr"/>
-      <c r="B7" s="65" t="inlineStr"/>
-      <c r="C7" s="65" t="inlineStr"/>
-      <c r="D7" s="65" t="inlineStr"/>
-      <c r="E7" s="65" t="inlineStr"/>
-      <c r="F7" s="63" t="n">
+      <c r="A7" s="63" t="inlineStr"/>
+      <c r="B7" s="63" t="inlineStr"/>
+      <c r="C7" s="63" t="inlineStr"/>
+      <c r="D7" s="63" t="inlineStr"/>
+      <c r="E7" s="63" t="inlineStr"/>
+      <c r="F7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="63" t="n">
+      <c r="G7" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="66">
+      <c r="H7" s="64">
         <f>G7-F7</f>
         <v/>
       </c>
-      <c r="I7" s="67">
+      <c r="I7" s="65">
         <f>IF(F7=0,"",(G7-F7)/F7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr"/>
-      <c r="B8" s="61" t="inlineStr"/>
-      <c r="C8" s="61" t="inlineStr"/>
-      <c r="D8" s="61" t="inlineStr"/>
-      <c r="E8" s="61" t="inlineStr"/>
-      <c r="F8" s="63" t="n">
+      <c r="A8" s="59" t="inlineStr"/>
+      <c r="B8" s="59" t="inlineStr"/>
+      <c r="C8" s="59" t="inlineStr"/>
+      <c r="D8" s="59" t="inlineStr"/>
+      <c r="E8" s="59" t="inlineStr"/>
+      <c r="F8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="63" t="n">
+      <c r="G8" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="62">
+      <c r="H8" s="60">
         <f>G8-F8</f>
         <v/>
       </c>
-      <c r="I8" s="64">
+      <c r="I8" s="62">
         <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="65" t="inlineStr"/>
-      <c r="B9" s="65" t="inlineStr"/>
-      <c r="C9" s="65" t="inlineStr"/>
-      <c r="D9" s="65" t="inlineStr"/>
-      <c r="E9" s="65" t="inlineStr"/>
-      <c r="F9" s="63" t="n">
+      <c r="A9" s="63" t="inlineStr"/>
+      <c r="B9" s="63" t="inlineStr"/>
+      <c r="C9" s="63" t="inlineStr"/>
+      <c r="D9" s="63" t="inlineStr"/>
+      <c r="E9" s="63" t="inlineStr"/>
+      <c r="F9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="63" t="n">
+      <c r="G9" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="66">
+      <c r="H9" s="64">
         <f>G9-F9</f>
         <v/>
       </c>
-      <c r="I9" s="67">
+      <c r="I9" s="65">
         <f>IF(F9=0,"",(G9-F9)/F9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr"/>
-      <c r="B10" s="61" t="inlineStr"/>
-      <c r="C10" s="61" t="inlineStr"/>
-      <c r="D10" s="61" t="inlineStr"/>
-      <c r="E10" s="61" t="inlineStr"/>
-      <c r="F10" s="63" t="n">
+      <c r="A10" s="59" t="inlineStr"/>
+      <c r="B10" s="59" t="inlineStr"/>
+      <c r="C10" s="59" t="inlineStr"/>
+      <c r="D10" s="59" t="inlineStr"/>
+      <c r="E10" s="59" t="inlineStr"/>
+      <c r="F10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="63" t="n">
+      <c r="G10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="62">
+      <c r="H10" s="60">
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="64">
+      <c r="I10" s="62">
         <f>IF(F10=0,"",(G10-F10)/F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="65" t="inlineStr"/>
-      <c r="B11" s="65" t="inlineStr"/>
-      <c r="C11" s="65" t="inlineStr"/>
-      <c r="D11" s="65" t="inlineStr"/>
-      <c r="E11" s="65" t="inlineStr"/>
-      <c r="F11" s="63" t="n">
+      <c r="A11" s="63" t="inlineStr"/>
+      <c r="B11" s="63" t="inlineStr"/>
+      <c r="C11" s="63" t="inlineStr"/>
+      <c r="D11" s="63" t="inlineStr"/>
+      <c r="E11" s="63" t="inlineStr"/>
+      <c r="F11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="63" t="n">
+      <c r="G11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="66">
+      <c r="H11" s="64">
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="67">
+      <c r="I11" s="65">
         <f>IF(F11=0,"",(G11-F11)/F11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr"/>
-      <c r="B12" s="61" t="inlineStr"/>
-      <c r="C12" s="61" t="inlineStr"/>
-      <c r="D12" s="61" t="inlineStr"/>
-      <c r="E12" s="61" t="inlineStr"/>
-      <c r="F12" s="63" t="n">
+      <c r="A12" s="59" t="inlineStr"/>
+      <c r="B12" s="59" t="inlineStr"/>
+      <c r="C12" s="59" t="inlineStr"/>
+      <c r="D12" s="59" t="inlineStr"/>
+      <c r="E12" s="59" t="inlineStr"/>
+      <c r="F12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="63" t="n">
+      <c r="G12" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="62">
+      <c r="H12" s="60">
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="64">
+      <c r="I12" s="62">
         <f>IF(F12=0,"",(G12-F12)/F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="65" t="inlineStr"/>
-      <c r="B13" s="65" t="inlineStr"/>
-      <c r="C13" s="65" t="inlineStr"/>
-      <c r="D13" s="65" t="inlineStr"/>
-      <c r="E13" s="65" t="inlineStr"/>
-      <c r="F13" s="63" t="n">
+      <c r="A13" s="63" t="inlineStr"/>
+      <c r="B13" s="63" t="inlineStr"/>
+      <c r="C13" s="63" t="inlineStr"/>
+      <c r="D13" s="63" t="inlineStr"/>
+      <c r="E13" s="63" t="inlineStr"/>
+      <c r="F13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="63" t="n">
+      <c r="G13" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="66">
+      <c r="H13" s="64">
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="67">
+      <c r="I13" s="65">
         <f>IF(F13=0,"",(G13-F13)/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="68" t="inlineStr">
+      <c r="A14" s="66" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="68" t="n"/>
-      <c r="C14" s="68" t="n"/>
-      <c r="D14" s="68" t="n"/>
-      <c r="E14" s="68" t="n"/>
-      <c r="F14" s="32">
+      <c r="B14" s="66" t="n"/>
+      <c r="C14" s="66" t="n"/>
+      <c r="D14" s="66" t="n"/>
+      <c r="E14" s="66" t="n"/>
+      <c r="F14" s="30">
         <f>SUM(F6:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="32">
+      <c r="G14" s="30">
         <f>SUM(G6:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="32">
+      <c r="H14" s="30">
         <f>G14-F14</f>
         <v/>
       </c>
-      <c r="I14" s="33">
+      <c r="I14" s="31">
         <f>IF(F14=0,"",(G14-F14)/F14)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
fix(tools): corrige etiquetas de los graficos del Dashboard
Las categorias de los graficos se escriben como strRef (no numRef), por
lo que el grafico de barras muestra los nombres de los 8 tipos de activo
y el circular las etiquetas de activos/pasivos/patrimonio. El grafico de
barras pasa a una sola serie con etiquetas de valor; el circular muestra
nombre y porcentaje, sin el prefijo "Series1".

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -526,7 +526,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Concentracion de activos: 2025 vs 2026</a:t>
+              <a:t>Concentracion de activos 2025 (por tipo)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -550,9 +550,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Dashboard'!$B$12:$B$19</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -560,30 +560,9 @@
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!E11</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$B$12:$B$19</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$E$12:$E$19</f>
-            </numRef>
-          </val>
-        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -611,9 +590,6 @@
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -650,9 +626,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Dashboard'!$B$38:$B$40</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -661,6 +637,10 @@
           </val>
         </ser>
         <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="1"/>
+          <showSerName val="0"/>
           <showPercent val="1"/>
         </dLbls>
         <firstSliceAng val="0"/>
@@ -684,7 +664,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3420000"/>
+    <ext cx="7560000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -703,10 +683,10 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>23</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5040000" cy="3420000"/>
+    <ext cx="5400000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>

</xml_diff>

<commit_message>
fix(tools): grafico de concentracion limpio, solo activos con valor
El grafico de barras del Dashboard usa un area auxiliar oculta con los
activos que tienen valor (omite los que estan en cero) y muestra
etiquetas de dato solo con el monto, sin el prefijo de serie/categoria.

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -223,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -232,6 +232,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -526,7 +527,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Concentracion de activos 2025 (por tipo)</a:t>
+              <a:t>Concentracion de activos 2025</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -539,11 +540,6 @@
         <ser>
           <idx val="0"/>
           <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!D11</f>
-            </strRef>
-          </tx>
           <spPr>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -551,17 +547,21 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'Dashboard'!$B$12:$B$19</f>
+              <f>'Dashboard'!$AA$3:$AA$5</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$D$12:$D$19</f>
+              <f>'Dashboard'!$AB$3:$AB$5</f>
             </numRef>
           </val>
         </ser>
         <dLbls>
+          <numFmt formatCode="&quot;$&quot;#,##0"/>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
         </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
@@ -664,7 +664,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7560000" cy="3600000"/>
+    <ext cx="7560000" cy="3780000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -683,10 +683,10 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>24</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="3600000"/>
+    <ext cx="5760000" cy="3780000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -993,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:AB42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1004,6 +1004,8 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="3" customWidth="1" min="8" max="8"/>
+    <col hidden="1" width="13" customWidth="1" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1022,656 +1024,685 @@
     </row>
     <row r="3" ht="5" customHeight="1">
       <c r="A3" s="3" t="n"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Dinero e inversiones</t>
+        </is>
+      </c>
+      <c r="AB3" s="4">
+        <f>D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Vehiculos, naves y aeronaves</t>
+        </is>
+      </c>
+      <c r="AB4" s="4">
+        <f>D16</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="6" customHeight="1">
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="5" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Bienes inmuebles</t>
+        </is>
+      </c>
+      <c r="AB5" s="4">
+        <f>D18</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>TOTAL ACTIVOS</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>TOTAL PASIVOS</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="E6" s="12" t="n"/>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO</t>
         </is>
       </c>
-      <c r="G6" s="13" t="n"/>
+      <c r="G6" s="14" t="n"/>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="14">
+      <c r="B7" s="15">
         <f>D20</f>
         <v/>
       </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="15">
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="16">
         <f>D25</f>
         <v/>
       </c>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="16">
+      <c r="E7" s="12" t="n"/>
+      <c r="F7" s="17">
         <f>D31</f>
         <v/>
       </c>
-      <c r="G7" s="13" t="n"/>
+      <c r="G7" s="14" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Var. proyectada</t>
         </is>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="19">
         <f>G20</f>
         <v/>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>Var. proyectada</t>
         </is>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="21">
         <f>G25</f>
         <v/>
       </c>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>Var. proyectada</t>
         </is>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="23">
         <f>G31</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>ACTIVOS</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C11" s="24" t="n"/>
-      <c r="D11" s="25" t="inlineStr">
+      <c r="C11" s="25" t="n"/>
+      <c r="D11" s="26" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="E11" s="25" t="inlineStr">
+      <c r="E11" s="26" t="inlineStr">
         <is>
           <t>Total 2026</t>
         </is>
       </c>
-      <c r="F11" s="25" t="inlineStr">
+      <c r="F11" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="G11" s="25" t="inlineStr">
+      <c r="G11" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>Dinero e inversiones</t>
         </is>
       </c>
-      <c r="D12" s="27">
+      <c r="D12" s="28">
         <f>'Dinero'!J10</f>
         <v/>
       </c>
-      <c r="E12" s="27">
+      <c r="E12" s="28">
         <f>'Dinero'!K10</f>
         <v/>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="28">
         <f>E12-D12</f>
         <v/>
       </c>
-      <c r="G12" s="28">
+      <c r="G12" s="29">
         <f>IF(D12=0,"",(E12-D12)/D12)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="26" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>Derechos representativos de capital</t>
         </is>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="28">
         <f>'Derechos de Capital'!J14</f>
         <v/>
       </c>
-      <c r="E13" s="27">
+      <c r="E13" s="28">
         <f>'Derechos de Capital'!K14</f>
         <v/>
       </c>
-      <c r="F13" s="27">
+      <c r="F13" s="28">
         <f>E13-D13</f>
         <v/>
       </c>
-      <c r="G13" s="28">
+      <c r="G13" s="29">
         <f>IF(D13=0,"",(E13-D13)/D13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="26" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>Cuentas por cobrar</t>
         </is>
       </c>
-      <c r="D14" s="27">
+      <c r="D14" s="28">
         <f>'Cuentas por Cobrar'!J14</f>
         <v/>
       </c>
-      <c r="E14" s="27">
+      <c r="E14" s="28">
         <f>'Cuentas por Cobrar'!K14</f>
         <v/>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="28">
         <f>E14-D14</f>
         <v/>
       </c>
-      <c r="G14" s="28">
+      <c r="G14" s="29">
         <f>IF(D14=0,"",(E14-D14)/D14)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>Bienes muebles</t>
         </is>
       </c>
-      <c r="D15" s="27">
+      <c r="D15" s="28">
         <f>'Bienes Muebles'!F14</f>
         <v/>
       </c>
-      <c r="E15" s="27">
+      <c r="E15" s="28">
         <f>'Bienes Muebles'!G14</f>
         <v/>
       </c>
-      <c r="F15" s="27">
+      <c r="F15" s="28">
         <f>E15-D15</f>
         <v/>
       </c>
-      <c r="G15" s="28">
+      <c r="G15" s="29">
         <f>IF(D15=0,"",(E15-D15)/D15)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>Vehiculos, naves y aeronaves</t>
         </is>
       </c>
-      <c r="D16" s="27">
+      <c r="D16" s="28">
         <f>'Vehiculos'!G9</f>
         <v/>
       </c>
-      <c r="E16" s="27">
+      <c r="E16" s="28">
         <f>'Vehiculos'!H9</f>
         <v/>
       </c>
-      <c r="F16" s="27">
+      <c r="F16" s="28">
         <f>E16-D16</f>
         <v/>
       </c>
-      <c r="G16" s="28">
+      <c r="G16" s="29">
         <f>IF(D16=0,"",(E16-D16)/D16)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>Derechos (usufructo, uso, etc.)</t>
         </is>
       </c>
-      <c r="D17" s="27">
+      <c r="D17" s="28">
         <f>'Derechos'!F14</f>
         <v/>
       </c>
-      <c r="E17" s="27">
+      <c r="E17" s="28">
         <f>'Derechos'!G14</f>
         <v/>
       </c>
-      <c r="F17" s="27">
+      <c r="F17" s="28">
         <f>E17-D17</f>
         <v/>
       </c>
-      <c r="G17" s="28">
+      <c r="G17" s="29">
         <f>IF(D17=0,"",(E17-D17)/D17)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="26" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>Bienes inmuebles</t>
         </is>
       </c>
-      <c r="D18" s="27">
+      <c r="D18" s="28">
         <f>'Bienes Inmuebles'!J10</f>
         <v/>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="28">
         <f>'Bienes Inmuebles'!K10</f>
         <v/>
       </c>
-      <c r="F18" s="27">
+      <c r="F18" s="28">
         <f>E18-D18</f>
         <v/>
       </c>
-      <c r="G18" s="28">
+      <c r="G18" s="29">
         <f>IF(D18=0,"",(E18-D18)/D18)</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>Otros activos</t>
         </is>
       </c>
-      <c r="D19" s="27">
+      <c r="D19" s="28">
         <f>'Otros Activos'!F14</f>
         <v/>
       </c>
-      <c r="E19" s="27">
+      <c r="E19" s="28">
         <f>'Otros Activos'!G14</f>
         <v/>
       </c>
-      <c r="F19" s="27">
+      <c r="F19" s="28">
         <f>E19-D19</f>
         <v/>
       </c>
-      <c r="G19" s="28">
+      <c r="G19" s="29">
         <f>IF(D19=0,"",(E19-D19)/D19)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="30" t="inlineStr">
         <is>
           <t>TOTAL ACTIVOS</t>
         </is>
       </c>
-      <c r="D20" s="30">
+      <c r="D20" s="31">
         <f>SUM(D12:D19)</f>
         <v/>
       </c>
-      <c r="E20" s="30">
+      <c r="E20" s="31">
         <f>SUM(E12:E19)</f>
         <v/>
       </c>
-      <c r="F20" s="30">
+      <c r="F20" s="31">
         <f>E20-D20</f>
         <v/>
       </c>
-      <c r="G20" s="31">
+      <c r="G20" s="32">
         <f>IF(D20=0,"",(E20-D20)/D20)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="32" t="inlineStr">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>PASIVOS</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B23" s="25" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="25" t="inlineStr">
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="26" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="E23" s="25" t="inlineStr">
+      <c r="E23" s="26" t="inlineStr">
         <is>
           <t>Total 2026</t>
         </is>
       </c>
-      <c r="F23" s="25" t="inlineStr">
+      <c r="F23" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="G23" s="25" t="inlineStr">
+      <c r="G23" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="33" t="inlineStr">
+      <c r="B24" s="34" t="inlineStr">
         <is>
           <t>Deudas y obligaciones</t>
         </is>
       </c>
-      <c r="D24" s="34">
+      <c r="D24" s="35">
         <f>'Pasivos'!I8</f>
         <v/>
       </c>
-      <c r="E24" s="34">
+      <c r="E24" s="35">
         <f>'Pasivos'!J8</f>
         <v/>
       </c>
-      <c r="F24" s="34">
+      <c r="F24" s="35">
         <f>E24-D24</f>
         <v/>
       </c>
-      <c r="G24" s="35">
+      <c r="G24" s="36">
         <f>IF(D24=0,"",(E24-D24)/D24)</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="36" t="inlineStr">
+      <c r="B25" s="37" t="inlineStr">
         <is>
           <t>TOTAL PASIVOS</t>
         </is>
       </c>
-      <c r="D25" s="37">
+      <c r="D25" s="38">
         <f>SUM(D24:D24)</f>
         <v/>
       </c>
-      <c r="E25" s="37">
+      <c r="E25" s="38">
         <f>SUM(E24:E24)</f>
         <v/>
       </c>
-      <c r="F25" s="37">
+      <c r="F25" s="38">
         <f>E25-D25</f>
         <v/>
       </c>
-      <c r="G25" s="38">
+      <c r="G25" s="39">
         <f>IF(D25=0,"",(E25-D25)/D25)</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="39" t="inlineStr">
+      <c r="B27" s="40" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C28" s="24" t="n"/>
-      <c r="D28" s="25" t="inlineStr">
+      <c r="C28" s="25" t="n"/>
+      <c r="D28" s="26" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="E28" s="25" t="inlineStr">
+      <c r="E28" s="26" t="inlineStr">
         <is>
           <t>Total 2026</t>
         </is>
       </c>
-      <c r="F28" s="25" t="inlineStr">
+      <c r="F28" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="G28" s="25" t="inlineStr">
+      <c r="G28" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="40" t="inlineStr">
+      <c r="B29" s="41" t="inlineStr">
         <is>
           <t>(+) Total activos</t>
         </is>
       </c>
-      <c r="D29" s="41">
+      <c r="D29" s="42">
         <f>D20</f>
         <v/>
       </c>
-      <c r="E29" s="41">
+      <c r="E29" s="42">
         <f>E20</f>
         <v/>
       </c>
-      <c r="F29" s="41">
+      <c r="F29" s="42">
         <f>E29-D29</f>
         <v/>
       </c>
-      <c r="G29" s="42">
+      <c r="G29" s="43">
         <f>IF(D29=0,"",(E29-D29)/D29)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="40" t="inlineStr">
+      <c r="B30" s="41" t="inlineStr">
         <is>
           <t>(-) Total pasivos</t>
         </is>
       </c>
-      <c r="D30" s="41">
+      <c r="D30" s="42">
         <f>D25</f>
         <v/>
       </c>
-      <c r="E30" s="41">
+      <c r="E30" s="42">
         <f>E25</f>
         <v/>
       </c>
-      <c r="F30" s="41">
+      <c r="F30" s="42">
         <f>E30-D30</f>
         <v/>
       </c>
-      <c r="G30" s="42">
+      <c r="G30" s="43">
         <f>IF(D30=0,"",(E30-D30)/D30)</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="43" t="inlineStr">
+      <c r="B31" s="44" t="inlineStr">
         <is>
           <t>(=) PATRIMONIO NETO</t>
         </is>
       </c>
-      <c r="D31" s="44">
+      <c r="D31" s="45">
         <f>D29-D30</f>
         <v/>
       </c>
-      <c r="E31" s="44">
+      <c r="E31" s="45">
         <f>E29-E30</f>
         <v/>
       </c>
-      <c r="F31" s="44">
+      <c r="F31" s="45">
         <f>E31-D31</f>
         <v/>
       </c>
-      <c r="G31" s="45">
+      <c r="G31" s="46">
         <f>IF(D31=0,"",(E31-D31)/D31)</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="46" t="inlineStr">
+      <c r="B32" s="47" t="inlineStr">
         <is>
           <t>Patrimonio declarado en el XML (2025)</t>
         </is>
       </c>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="47" t="n">
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="48" t="n">
         <v>883285.5600000001</v>
       </c>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="6" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="B33" s="46" t="inlineStr">
+      <c r="B33" s="47" t="inlineStr">
         <is>
           <t>Patrimonio neto del anio anterior</t>
         </is>
       </c>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="47" t="n">
+      <c r="C33" s="6" t="n"/>
+      <c r="D33" s="48" t="n">
         <v>801569.97</v>
       </c>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="6" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="B34" s="46" t="inlineStr">
+      <c r="B34" s="47" t="inlineStr">
         <is>
           <t>Crecimiento / decremento patrimonial (XML)</t>
         </is>
       </c>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="47" t="n">
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="48" t="n">
         <v>81715.59</v>
       </c>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="6" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="48" t="inlineStr">
+      <c r="B36" s="49" t="inlineStr">
         <is>
           <t>CONSOLIDADO</t>
         </is>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1">
-      <c r="B37" s="24" t="inlineStr">
+      <c r="B37" s="25" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C37" s="24" t="n"/>
-      <c r="D37" s="25" t="inlineStr">
+      <c r="C37" s="25" t="n"/>
+      <c r="D37" s="26" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="E37" s="25" t="inlineStr">
+      <c r="E37" s="26" t="inlineStr">
         <is>
           <t>Total 2026</t>
         </is>
       </c>
-      <c r="F37" s="25" t="inlineStr">
+      <c r="F37" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="G37" s="25" t="inlineStr">
+      <c r="G37" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="49" t="inlineStr">
+      <c r="B38" s="50" t="inlineStr">
         <is>
           <t>Activos</t>
         </is>
       </c>
-      <c r="D38" s="50">
+      <c r="D38" s="51">
         <f>D20</f>
         <v/>
       </c>
-      <c r="E38" s="50">
+      <c r="E38" s="51">
         <f>E20</f>
         <v/>
       </c>
-      <c r="F38" s="50">
+      <c r="F38" s="51">
         <f>E38-D38</f>
         <v/>
       </c>
-      <c r="G38" s="51">
+      <c r="G38" s="52">
         <f>IF(D38=0,"",(E38-D38)/D38)</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="52" t="inlineStr">
+      <c r="B39" s="53" t="inlineStr">
         <is>
           <t>Pasivos</t>
         </is>
       </c>
-      <c r="D39" s="53">
+      <c r="D39" s="54">
         <f>D25</f>
         <v/>
       </c>
-      <c r="E39" s="53">
+      <c r="E39" s="54">
         <f>E25</f>
         <v/>
       </c>
-      <c r="F39" s="53">
+      <c r="F39" s="54">
         <f>E39-D39</f>
         <v/>
       </c>
-      <c r="G39" s="54">
+      <c r="G39" s="55">
         <f>IF(D39=0,"",(E39-D39)/D39)</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="B40" s="55" t="inlineStr">
+      <c r="B40" s="56" t="inlineStr">
         <is>
           <t>Patrimonio neto</t>
         </is>
       </c>
-      <c r="D40" s="56">
+      <c r="D40" s="57">
         <f>D31</f>
         <v/>
       </c>
-      <c r="E40" s="56">
+      <c r="E40" s="57">
         <f>E31</f>
         <v/>
       </c>
-      <c r="F40" s="56">
+      <c r="F40" s="57">
         <f>E40-D40</f>
         <v/>
       </c>
-      <c r="G40" s="57">
+      <c r="G40" s="58">
         <f>IF(D40=0,"",(E40-D40)/D40)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="58" t="inlineStr">
+      <c r="B42" s="59" t="inlineStr">
         <is>
           <t>Edite las columnas amarillas en las hojas de cada modulo; las tarjetas, secciones y graficos se recalculan solos.</t>
         </is>
@@ -1766,197 +1797,197 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Tipo de acreedor</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Domicilio del acreedor</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Nombre del acreedor</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>N. de identificacion</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>N. registro Banco Central</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Partes relacionadas</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="26" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr">
+      <c r="K5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="L5" s="25" t="inlineStr">
+      <c r="L5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C6" s="59" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>DINERS CLUB DEL ECUADOR</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr">
+      <c r="E6" s="60" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
-      <c r="F6" s="59" t="inlineStr">
+      <c r="F6" s="60" t="inlineStr">
         <is>
           <t>1792260957001</t>
         </is>
       </c>
-      <c r="G6" s="59" t="inlineStr"/>
-      <c r="H6" s="59" t="inlineStr">
+      <c r="G6" s="60" t="inlineStr"/>
+      <c r="H6" s="60" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="I6" s="60" t="n">
+      <c r="I6" s="61" t="n">
         <v>4891.88</v>
       </c>
-      <c r="J6" s="61" t="n">
+      <c r="J6" s="62" t="n">
         <v>4891.88</v>
       </c>
-      <c r="K6" s="60">
+      <c r="K6" s="61">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="62">
+      <c r="L6" s="63">
         <f>IF(I6=0,"",(J6-I6)/I6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="63" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B7" s="63" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C7" s="63" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D7" s="63" t="inlineStr">
+      <c r="D7" s="64" t="inlineStr">
         <is>
           <t>BANCO DEL PICHINCHA</t>
         </is>
       </c>
-      <c r="E7" s="63" t="inlineStr">
+      <c r="E7" s="64" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
-      <c r="F7" s="63" t="inlineStr">
+      <c r="F7" s="64" t="inlineStr">
         <is>
           <t>1790010937001</t>
         </is>
       </c>
-      <c r="G7" s="63" t="inlineStr"/>
-      <c r="H7" s="63" t="inlineStr">
+      <c r="G7" s="64" t="inlineStr"/>
+      <c r="H7" s="64" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="I7" s="64" t="n">
+      <c r="I7" s="65" t="n">
         <v>5547.31</v>
       </c>
-      <c r="J7" s="61" t="n">
+      <c r="J7" s="62" t="n">
         <v>5547.31</v>
       </c>
-      <c r="K7" s="64">
+      <c r="K7" s="65">
         <f>J7-I7</f>
         <v/>
       </c>
-      <c r="L7" s="65">
+      <c r="L7" s="66">
         <f>IF(I7=0,"",(J7-I7)/I7)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="67" t="inlineStr">
+      <c r="A8" s="68" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="67" t="n"/>
-      <c r="C8" s="67" t="n"/>
-      <c r="D8" s="67" t="n"/>
-      <c r="E8" s="67" t="n"/>
-      <c r="F8" s="67" t="n"/>
-      <c r="G8" s="67" t="n"/>
-      <c r="H8" s="67" t="n"/>
-      <c r="I8" s="37">
+      <c r="B8" s="68" t="n"/>
+      <c r="C8" s="68" t="n"/>
+      <c r="D8" s="68" t="n"/>
+      <c r="E8" s="68" t="n"/>
+      <c r="F8" s="68" t="n"/>
+      <c r="G8" s="68" t="n"/>
+      <c r="H8" s="68" t="n"/>
+      <c r="I8" s="38">
         <f>SUM(I6:I7)</f>
         <v/>
       </c>
-      <c r="J8" s="37">
+      <c r="J8" s="38">
         <f>SUM(J6:J7)</f>
         <v/>
       </c>
-      <c r="K8" s="37">
+      <c r="K8" s="38">
         <f>J8-I8</f>
         <v/>
       </c>
-      <c r="L8" s="38">
+      <c r="L8" s="39">
         <f>IF(I8=0,"",(J8-I8)/I8)</f>
         <v/>
       </c>
@@ -2022,115 +2053,115 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="68" t="inlineStr">
+      <c r="B5" s="69" t="inlineStr">
         <is>
           <t>Incremento patrimonial declarado en el XML</t>
         </is>
       </c>
-      <c r="C5" s="69" t="n"/>
-      <c r="D5" s="69" t="n"/>
-      <c r="E5" s="70" t="n">
+      <c r="C5" s="70" t="n"/>
+      <c r="D5" s="70" t="n"/>
+      <c r="E5" s="71" t="n">
         <v>81715.59</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>Concepto (Tabla 14 del SRI)</t>
         </is>
       </c>
-      <c r="E7" s="25" t="inlineStr">
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>Justifica la variacion</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="71" t="inlineStr">
+      <c r="B8" s="72" t="inlineStr">
         <is>
           <t>1 - Ingresos locales</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="72" t="inlineStr">
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="73" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="71" t="inlineStr">
+      <c r="B9" s="72" t="inlineStr">
         <is>
           <t>2 - Ingresos exterior</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="72" t="inlineStr">
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="73" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="71" t="inlineStr">
+      <c r="B10" s="72" t="inlineStr">
         <is>
           <t>3 - Herencias, legados o donaciones</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="72" t="inlineStr">
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="73" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="71" t="inlineStr">
+      <c r="B11" s="72" t="inlineStr">
         <is>
           <t>4 - Loterias o rifas</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="72" t="inlineStr">
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="73" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="71" t="inlineStr">
+      <c r="B12" s="72" t="inlineStr">
         <is>
           <t>5 - Ganancias de capital</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="72" t="inlineStr">
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="73" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="71" t="inlineStr">
+      <c r="B13" s="72" t="inlineStr">
         <is>
           <t>6 - Otros</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="72" t="inlineStr">
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="73" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="58" t="inlineStr">
+      <c r="B15" s="59" t="inlineStr">
         <is>
           <t>Esta hoja reproduce la seccion Justificacion del formulario del SRI. Marque 'Si' en los conceptos que apliquen; el generador de XML los toma de aqui.</t>
         </is>
@@ -2193,97 +2224,97 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="73" t="inlineStr">
+      <c r="B5" s="74" t="inlineStr">
         <is>
           <t>►   GENERAR XML</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="74" t="inlineStr">
+      <c r="B7" s="75" t="inlineStr">
         <is>
           <t>En el archivo .xlsm el boton verde ya esta vinculado a la macro GenerarXmlSRI.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="75" t="inlineStr">
+      <c r="B9" s="76" t="inlineStr">
         <is>
           <t>COMO USAR ESTE ARCHIVO</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="76" t="inlineStr">
+      <c r="B10" s="77" t="inlineStr">
         <is>
           <t>1. Al abrir el archivo .xlsm, pulse 'Habilitar contenido' en la barra de seguridad de Excel.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="76" t="inlineStr">
+      <c r="B11" s="77" t="inlineStr">
         <is>
           <t>2. Llene las columnas amarillas de cada modulo (Dinero, Vehiculos, etc.) y la hoja Justificacion.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="76" t="inlineStr">
+      <c r="B12" s="77" t="inlineStr">
         <is>
           <t>3. Pulse el boton verde GENERAR XML, indique el anio y elija donde guardar el archivo.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="76" t="inlineStr">
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>4. El archivo .xml queda listo para subir al portal del SRI.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="76" t="inlineStr"/>
+      <c r="B14" s="77" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="75" t="inlineStr">
+      <c r="B15" s="76" t="inlineStr">
         <is>
           <t>SI EXCEL BLOQUEA LAS MACROS</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="76" t="inlineStr">
+      <c r="B16" s="77" t="inlineStr">
         <is>
           <t>- Cierre Excel. En el Explorador, clic derecho sobre el archivo &gt; Propiedades.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="76" t="inlineStr">
+      <c r="B17" s="77" t="inlineStr">
         <is>
           <t>- Al final de la pestana General marque 'Desbloquear' y pulse Aceptar.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="76" t="inlineStr">
+      <c r="B18" s="77" t="inlineStr">
         <is>
           <t>- Vuelva a abrirlo y pulse 'Habilitar contenido'. Conserve siempre la extension .xlsm.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="76" t="inlineStr"/>
+      <c r="B19" s="77" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="B20" s="76" t="inlineStr">
+      <c r="B20" s="77" t="inlineStr">
         <is>
           <t>Alternativa sin macros:  ejecutar  python tools/generar_xml_sri.py  desde la terminal.</t>
         </is>
@@ -2324,257 +2355,257 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="77" t="inlineStr">
+      <c r="A5" s="78" t="inlineStr">
         <is>
           <t>IDENTIFICACION</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="78" t="inlineStr">
+      <c r="A6" s="79" t="inlineStr">
         <is>
           <t>Anio de la declaracion</t>
         </is>
       </c>
-      <c r="B6" s="79" t="n">
+      <c r="B6" s="80" t="n">
         <v>2025</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="78" t="inlineStr">
+      <c r="A7" s="79" t="inlineStr">
         <is>
           <t>Tipo de declaracion</t>
         </is>
       </c>
-      <c r="B7" s="79" t="inlineStr">
+      <c r="B7" s="80" t="inlineStr">
         <is>
           <t>SOC - Sociedad conyugal o union de hecho</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="78" t="inlineStr">
+      <c r="A8" s="79" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="B8" s="79" t="inlineStr">
+      <c r="B8" s="80" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="78" t="inlineStr">
+      <c r="A9" s="79" t="inlineStr">
         <is>
           <t>Numero de identificacion</t>
         </is>
       </c>
-      <c r="B9" s="79" t="inlineStr">
+      <c r="B9" s="80" t="inlineStr">
         <is>
           <t>1709164899001</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="78" t="inlineStr">
+      <c r="A10" s="79" t="inlineStr">
         <is>
           <t>Nombre del declarante</t>
         </is>
       </c>
-      <c r="B10" s="79" t="inlineStr">
+      <c r="B10" s="80" t="inlineStr">
         <is>
           <t>GONZALEZ NAVAS MARCO VINICIO</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="78" t="inlineStr">
+      <c r="A11" s="79" t="inlineStr">
         <is>
           <t>Identificacion del conyuge</t>
         </is>
       </c>
-      <c r="B11" s="79" t="inlineStr">
+      <c r="B11" s="80" t="inlineStr">
         <is>
           <t>C - Cedula</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="78" t="inlineStr">
+      <c r="A12" s="79" t="inlineStr">
         <is>
           <t>Numero ident. conyuge</t>
         </is>
       </c>
-      <c r="B12" s="79" t="inlineStr">
+      <c r="B12" s="80" t="inlineStr">
         <is>
           <t>1709784225</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="78" t="inlineStr">
+      <c r="A13" s="79" t="inlineStr">
         <is>
           <t>Nombre del conyuge</t>
         </is>
       </c>
-      <c r="B13" s="79" t="inlineStr">
+      <c r="B13" s="80" t="inlineStr">
         <is>
           <t>HIDALGO LOZA ROSA CONSUELO</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="78" t="inlineStr">
+      <c r="A14" s="79" t="inlineStr">
         <is>
           <t>Total creditos / cuentas por cobrar</t>
         </is>
       </c>
-      <c r="B14" s="60" t="n">
+      <c r="B14" s="61" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="77" t="inlineStr">
+      <c r="A16" s="78" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO (enlazado a la hoja Dashboard)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="78" t="inlineStr">
+      <c r="A17" s="79" t="inlineStr">
         <is>
           <t>Patrimonio neto 2025</t>
         </is>
       </c>
-      <c r="B17" s="60">
+      <c r="B17" s="61">
         <f>Dashboard!D31</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="78" t="inlineStr">
+      <c r="A18" s="79" t="inlineStr">
         <is>
           <t>Patrimonio neto 2026 (proyectado)</t>
         </is>
       </c>
-      <c r="B18" s="60">
+      <c r="B18" s="61">
         <f>Dashboard!E31</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="78" t="inlineStr">
+      <c r="A19" s="79" t="inlineStr">
         <is>
           <t>Variacion proyectada</t>
         </is>
       </c>
-      <c r="B19" s="60">
+      <c r="B19" s="61">
         <f>Dashboard!F31</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="78" t="inlineStr">
+      <c r="A20" s="79" t="inlineStr">
         <is>
           <t>Variacion % proyectada</t>
         </is>
       </c>
-      <c r="B20" s="62">
+      <c r="B20" s="63">
         <f>Dashboard!G31</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="77" t="inlineStr">
+      <c r="A22" s="78" t="inlineStr">
         <is>
           <t>PATRIMONIO DECLARADO EN EL XML</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="78" t="inlineStr">
+      <c r="A23" s="79" t="inlineStr">
         <is>
           <t>Patrimonio total declarado</t>
         </is>
       </c>
-      <c r="B23" s="60" t="n">
+      <c r="B23" s="61" t="n">
         <v>883285.5600000001</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="78" t="inlineStr">
+      <c r="A24" s="79" t="inlineStr">
         <is>
           <t>Atribuible a hijos no emancipados</t>
         </is>
       </c>
-      <c r="B24" s="60" t="n">
+      <c r="B24" s="61" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="78" t="inlineStr">
+      <c r="A25" s="79" t="inlineStr">
         <is>
           <t>Patrimonio en la sociedad conyugal</t>
         </is>
       </c>
-      <c r="B25" s="60" t="n">
+      <c r="B25" s="61" t="n">
         <v>883285.5600000001</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="78" t="inlineStr">
+      <c r="A26" s="79" t="inlineStr">
         <is>
           <t>Patrimonio individual del declarante</t>
         </is>
       </c>
-      <c r="B26" s="60" t="n">
+      <c r="B26" s="61" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="78" t="inlineStr">
+      <c r="A27" s="79" t="inlineStr">
         <is>
           <t>Patrimonio del anio anterior</t>
         </is>
       </c>
-      <c r="B27" s="60" t="n">
+      <c r="B27" s="61" t="n">
         <v>801569.97</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="78" t="inlineStr">
+      <c r="A28" s="79" t="inlineStr">
         <is>
           <t>Crecimiento / decremento patrimonial</t>
         </is>
       </c>
-      <c r="B28" s="60" t="n">
+      <c r="B28" s="61" t="n">
         <v>81715.59</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="75" t="inlineStr">
+      <c r="A30" s="76" t="inlineStr">
         <is>
           <t>Justificacion de la variacion (ver hoja Justificacion)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="76" t="inlineStr">
+      <c r="A31" s="77" t="inlineStr">
         <is>
           <t>- 1 - Ingresos locales</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="76" t="inlineStr">
+      <c r="A32" s="77" t="inlineStr">
         <is>
           <t>- 6 - Otros</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="58" t="inlineStr">
+      <c r="A34" s="59" t="inlineStr">
         <is>
           <t>Catalogos del SRI integrados (Tablas 1-19 del archivo CATALOGO.xls). El XML se genera con generar_xml_sri.py.</t>
         </is>
@@ -5845,97 +5876,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="80" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>DINERO_EN</t>
         </is>
       </c>
-      <c r="B1" s="80" t="inlineStr">
+      <c r="B1" s="81" t="inlineStr">
         <is>
           <t>TIPO_INVERSION</t>
         </is>
       </c>
-      <c r="C1" s="80" t="inlineStr">
+      <c r="C1" s="81" t="inlineStr">
         <is>
           <t>UBICACION</t>
         </is>
       </c>
-      <c r="D1" s="80" t="inlineStr">
+      <c r="D1" s="81" t="inlineStr">
         <is>
           <t>PAIS</t>
         </is>
       </c>
-      <c r="E1" s="80" t="inlineStr">
+      <c r="E1" s="81" t="inlineStr">
         <is>
           <t>INSTITUCION_FINANCIERA</t>
         </is>
       </c>
-      <c r="F1" s="80" t="inlineStr">
+      <c r="F1" s="81" t="inlineStr">
         <is>
           <t>PARTES_RELACIONADAS</t>
         </is>
       </c>
-      <c r="G1" s="80" t="inlineStr">
+      <c r="G1" s="81" t="inlineStr">
         <is>
           <t>TIPO_DRC</t>
         </is>
       </c>
-      <c r="H1" s="80" t="inlineStr">
+      <c r="H1" s="81" t="inlineStr">
         <is>
           <t>TIPO_PERSONA</t>
         </is>
       </c>
-      <c r="I1" s="80" t="inlineStr">
+      <c r="I1" s="81" t="inlineStr">
         <is>
           <t>TIPO_BIEN_MUEBLE</t>
         </is>
       </c>
-      <c r="J1" s="80" t="inlineStr">
+      <c r="J1" s="81" t="inlineStr">
         <is>
           <t>TIPO_VEHICULO</t>
         </is>
       </c>
-      <c r="K1" s="80" t="inlineStr">
+      <c r="K1" s="81" t="inlineStr">
         <is>
           <t>TIPO_DERECHO</t>
         </is>
       </c>
-      <c r="L1" s="80" t="inlineStr">
+      <c r="L1" s="81" t="inlineStr">
         <is>
           <t>TIPO_INMUEBLE</t>
         </is>
       </c>
-      <c r="M1" s="80" t="inlineStr">
+      <c r="M1" s="81" t="inlineStr">
         <is>
           <t>PROVINCIA</t>
         </is>
       </c>
-      <c r="N1" s="80" t="inlineStr">
+      <c r="N1" s="81" t="inlineStr">
         <is>
           <t>CANTON</t>
         </is>
       </c>
-      <c r="O1" s="80" t="inlineStr">
+      <c r="O1" s="81" t="inlineStr">
         <is>
           <t>TIPO_ACREEDOR</t>
         </is>
       </c>
-      <c r="P1" s="80" t="inlineStr">
+      <c r="P1" s="81" t="inlineStr">
         <is>
           <t>TIPO_IDENTIFICACION</t>
         </is>
       </c>
-      <c r="Q1" s="80" t="inlineStr">
+      <c r="Q1" s="81" t="inlineStr">
         <is>
           <t>REGULARIZACION</t>
         </is>
       </c>
-      <c r="R1" s="80" t="inlineStr">
+      <c r="R1" s="81" t="inlineStr">
         <is>
           <t>JUSTIF_INCREMENTO</t>
         </is>
       </c>
-      <c r="S1" s="80" t="inlineStr">
+      <c r="S1" s="81" t="inlineStr">
         <is>
           <t>JUSTIF_DECREMENTO</t>
         </is>
@@ -12469,311 +12500,311 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Dinero en</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Tipo de inversion</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Institucion financiera</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Tipo de moneda</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Partes relacionadas</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr">
+      <c r="K5" s="26" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="L5" s="25" t="inlineStr">
+      <c r="L5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="M5" s="25" t="inlineStr">
+      <c r="M5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>3 - Cuenta de ahorros</t>
         </is>
       </c>
-      <c r="C6" s="59" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr">
+      <c r="E6" s="60" t="inlineStr">
         <is>
           <t>1029 - BANCO PICHINCHA C.A.</t>
         </is>
       </c>
-      <c r="F6" s="59" t="inlineStr">
+      <c r="F6" s="60" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G6" s="59" t="inlineStr">
+      <c r="G6" s="60" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H6" s="59" t="inlineStr"/>
-      <c r="I6" s="59" t="inlineStr"/>
-      <c r="J6" s="60" t="n">
+      <c r="H6" s="60" t="inlineStr"/>
+      <c r="I6" s="60" t="inlineStr"/>
+      <c r="J6" s="61" t="n">
         <v>130.2</v>
       </c>
-      <c r="K6" s="61" t="n">
+      <c r="K6" s="62" t="n">
         <v>130.2</v>
       </c>
-      <c r="L6" s="60">
+      <c r="L6" s="61">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="62">
+      <c r="M6" s="63">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="63" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B7" s="63" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>4 - Cuenta corriente</t>
         </is>
       </c>
-      <c r="C7" s="63" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D7" s="63" t="inlineStr">
+      <c r="D7" s="64" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E7" s="63" t="inlineStr">
+      <c r="E7" s="64" t="inlineStr">
         <is>
           <t>1029 - BANCO PICHINCHA C.A.</t>
         </is>
       </c>
-      <c r="F7" s="63" t="inlineStr">
+      <c r="F7" s="64" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G7" s="63" t="inlineStr">
+      <c r="G7" s="64" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H7" s="63" t="inlineStr"/>
-      <c r="I7" s="63" t="inlineStr"/>
-      <c r="J7" s="64" t="n">
+      <c r="H7" s="64" t="inlineStr"/>
+      <c r="I7" s="64" t="inlineStr"/>
+      <c r="J7" s="65" t="n">
         <v>5590.32</v>
       </c>
-      <c r="K7" s="61" t="n">
+      <c r="K7" s="62" t="n">
         <v>5590.32</v>
       </c>
-      <c r="L7" s="64">
+      <c r="L7" s="65">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="65">
+      <c r="M7" s="66">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>3 - Cuenta de ahorros</t>
         </is>
       </c>
-      <c r="C8" s="59" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D8" s="59" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E8" s="59" t="inlineStr">
+      <c r="E8" s="60" t="inlineStr">
         <is>
           <t>1418 - BANCO PROMERICA S.A.</t>
         </is>
       </c>
-      <c r="F8" s="59" t="inlineStr">
+      <c r="F8" s="60" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G8" s="59" t="inlineStr">
+      <c r="G8" s="60" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H8" s="59" t="inlineStr"/>
-      <c r="I8" s="59" t="inlineStr"/>
-      <c r="J8" s="60" t="n">
+      <c r="H8" s="60" t="inlineStr"/>
+      <c r="I8" s="60" t="inlineStr"/>
+      <c r="J8" s="61" t="n">
         <v>53237.31</v>
       </c>
-      <c r="K8" s="61" t="n">
+      <c r="K8" s="62" t="n">
         <v>53237.31</v>
       </c>
-      <c r="L8" s="60">
+      <c r="L8" s="61">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="62">
+      <c r="M8" s="63">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="63" t="inlineStr">
+      <c r="A9" s="64" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B9" s="63" t="inlineStr">
+      <c r="B9" s="64" t="inlineStr">
         <is>
           <t>2 - Inversiones financieras</t>
         </is>
       </c>
-      <c r="C9" s="63" t="inlineStr">
+      <c r="C9" s="64" t="inlineStr">
         <is>
           <t>EXT - En el exterior</t>
         </is>
       </c>
-      <c r="D9" s="63" t="inlineStr">
+      <c r="D9" s="64" t="inlineStr">
         <is>
           <t>118 - PANAMA</t>
         </is>
       </c>
-      <c r="E9" s="63" t="inlineStr">
+      <c r="E9" s="64" t="inlineStr">
         <is>
           <t>BANCO PICHINCHA CA</t>
         </is>
       </c>
-      <c r="F9" s="63" t="inlineStr">
+      <c r="F9" s="64" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G9" s="63" t="inlineStr">
+      <c r="G9" s="64" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H9" s="63" t="inlineStr"/>
-      <c r="I9" s="63" t="inlineStr"/>
-      <c r="J9" s="64" t="n">
+      <c r="H9" s="64" t="inlineStr"/>
+      <c r="I9" s="64" t="inlineStr"/>
+      <c r="J9" s="65" t="n">
         <v>189049.31</v>
       </c>
-      <c r="K9" s="61" t="n">
+      <c r="K9" s="62" t="n">
         <v>189049.31</v>
       </c>
-      <c r="L9" s="64">
+      <c r="L9" s="65">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="65">
+      <c r="M9" s="66">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="66" t="inlineStr">
+      <c r="A10" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B10" s="66" t="n"/>
-      <c r="C10" s="66" t="n"/>
-      <c r="D10" s="66" t="n"/>
-      <c r="E10" s="66" t="n"/>
-      <c r="F10" s="66" t="n"/>
-      <c r="G10" s="66" t="n"/>
-      <c r="H10" s="66" t="n"/>
-      <c r="I10" s="66" t="n"/>
-      <c r="J10" s="30">
+      <c r="B10" s="67" t="n"/>
+      <c r="C10" s="67" t="n"/>
+      <c r="D10" s="67" t="n"/>
+      <c r="E10" s="67" t="n"/>
+      <c r="F10" s="67" t="n"/>
+      <c r="G10" s="67" t="n"/>
+      <c r="H10" s="67" t="n"/>
+      <c r="I10" s="67" t="n"/>
+      <c r="J10" s="31">
         <f>SUM(J6:J9)</f>
         <v/>
       </c>
-      <c r="K10" s="30">
+      <c r="K10" s="31">
         <f>SUM(K6:K9)</f>
         <v/>
       </c>
-      <c r="L10" s="30">
+      <c r="L10" s="31">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="31">
+      <c r="M10" s="32">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
@@ -12853,299 +12884,299 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Tipo de inversion</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Empresa / Administradora / Fideicomiso</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>% de participacion</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>N. de acciones / participaciones</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Partes relacionadas</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr">
+      <c r="K5" s="26" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="L5" s="25" t="inlineStr">
+      <c r="L5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="M5" s="25" t="inlineStr">
+      <c r="M5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr"/>
-      <c r="B6" s="59" t="inlineStr"/>
-      <c r="C6" s="59" t="inlineStr"/>
-      <c r="D6" s="59" t="inlineStr"/>
-      <c r="E6" s="59" t="inlineStr"/>
-      <c r="F6" s="59" t="inlineStr"/>
-      <c r="G6" s="59" t="inlineStr"/>
-      <c r="H6" s="59" t="inlineStr"/>
-      <c r="I6" s="59" t="inlineStr"/>
-      <c r="J6" s="61" t="n">
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="60" t="inlineStr"/>
+      <c r="C6" s="60" t="inlineStr"/>
+      <c r="D6" s="60" t="inlineStr"/>
+      <c r="E6" s="60" t="inlineStr"/>
+      <c r="F6" s="60" t="inlineStr"/>
+      <c r="G6" s="60" t="inlineStr"/>
+      <c r="H6" s="60" t="inlineStr"/>
+      <c r="I6" s="60" t="inlineStr"/>
+      <c r="J6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="61" t="n">
+      <c r="K6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="60">
+      <c r="L6" s="61">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="62">
+      <c r="M6" s="63">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="63" t="inlineStr"/>
-      <c r="B7" s="63" t="inlineStr"/>
-      <c r="C7" s="63" t="inlineStr"/>
-      <c r="D7" s="63" t="inlineStr"/>
-      <c r="E7" s="63" t="inlineStr"/>
-      <c r="F7" s="63" t="inlineStr"/>
-      <c r="G7" s="63" t="inlineStr"/>
-      <c r="H7" s="63" t="inlineStr"/>
-      <c r="I7" s="63" t="inlineStr"/>
-      <c r="J7" s="61" t="n">
+      <c r="A7" s="64" t="inlineStr"/>
+      <c r="B7" s="64" t="inlineStr"/>
+      <c r="C7" s="64" t="inlineStr"/>
+      <c r="D7" s="64" t="inlineStr"/>
+      <c r="E7" s="64" t="inlineStr"/>
+      <c r="F7" s="64" t="inlineStr"/>
+      <c r="G7" s="64" t="inlineStr"/>
+      <c r="H7" s="64" t="inlineStr"/>
+      <c r="I7" s="64" t="inlineStr"/>
+      <c r="J7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="61" t="n">
+      <c r="K7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="64">
+      <c r="L7" s="65">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="65">
+      <c r="M7" s="66">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr"/>
-      <c r="B8" s="59" t="inlineStr"/>
-      <c r="C8" s="59" t="inlineStr"/>
-      <c r="D8" s="59" t="inlineStr"/>
-      <c r="E8" s="59" t="inlineStr"/>
-      <c r="F8" s="59" t="inlineStr"/>
-      <c r="G8" s="59" t="inlineStr"/>
-      <c r="H8" s="59" t="inlineStr"/>
-      <c r="I8" s="59" t="inlineStr"/>
-      <c r="J8" s="61" t="n">
+      <c r="A8" s="60" t="inlineStr"/>
+      <c r="B8" s="60" t="inlineStr"/>
+      <c r="C8" s="60" t="inlineStr"/>
+      <c r="D8" s="60" t="inlineStr"/>
+      <c r="E8" s="60" t="inlineStr"/>
+      <c r="F8" s="60" t="inlineStr"/>
+      <c r="G8" s="60" t="inlineStr"/>
+      <c r="H8" s="60" t="inlineStr"/>
+      <c r="I8" s="60" t="inlineStr"/>
+      <c r="J8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="61" t="n">
+      <c r="K8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="60">
+      <c r="L8" s="61">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="62">
+      <c r="M8" s="63">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="63" t="inlineStr"/>
-      <c r="B9" s="63" t="inlineStr"/>
-      <c r="C9" s="63" t="inlineStr"/>
-      <c r="D9" s="63" t="inlineStr"/>
-      <c r="E9" s="63" t="inlineStr"/>
-      <c r="F9" s="63" t="inlineStr"/>
-      <c r="G9" s="63" t="inlineStr"/>
-      <c r="H9" s="63" t="inlineStr"/>
-      <c r="I9" s="63" t="inlineStr"/>
-      <c r="J9" s="61" t="n">
+      <c r="A9" s="64" t="inlineStr"/>
+      <c r="B9" s="64" t="inlineStr"/>
+      <c r="C9" s="64" t="inlineStr"/>
+      <c r="D9" s="64" t="inlineStr"/>
+      <c r="E9" s="64" t="inlineStr"/>
+      <c r="F9" s="64" t="inlineStr"/>
+      <c r="G9" s="64" t="inlineStr"/>
+      <c r="H9" s="64" t="inlineStr"/>
+      <c r="I9" s="64" t="inlineStr"/>
+      <c r="J9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="61" t="n">
+      <c r="K9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="64">
+      <c r="L9" s="65">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="65">
+      <c r="M9" s="66">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr"/>
-      <c r="B10" s="59" t="inlineStr"/>
-      <c r="C10" s="59" t="inlineStr"/>
-      <c r="D10" s="59" t="inlineStr"/>
-      <c r="E10" s="59" t="inlineStr"/>
-      <c r="F10" s="59" t="inlineStr"/>
-      <c r="G10" s="59" t="inlineStr"/>
-      <c r="H10" s="59" t="inlineStr"/>
-      <c r="I10" s="59" t="inlineStr"/>
-      <c r="J10" s="61" t="n">
+      <c r="A10" s="60" t="inlineStr"/>
+      <c r="B10" s="60" t="inlineStr"/>
+      <c r="C10" s="60" t="inlineStr"/>
+      <c r="D10" s="60" t="inlineStr"/>
+      <c r="E10" s="60" t="inlineStr"/>
+      <c r="F10" s="60" t="inlineStr"/>
+      <c r="G10" s="60" t="inlineStr"/>
+      <c r="H10" s="60" t="inlineStr"/>
+      <c r="I10" s="60" t="inlineStr"/>
+      <c r="J10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="61" t="n">
+      <c r="K10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="60">
+      <c r="L10" s="61">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="62">
+      <c r="M10" s="63">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="63" t="inlineStr"/>
-      <c r="B11" s="63" t="inlineStr"/>
-      <c r="C11" s="63" t="inlineStr"/>
-      <c r="D11" s="63" t="inlineStr"/>
-      <c r="E11" s="63" t="inlineStr"/>
-      <c r="F11" s="63" t="inlineStr"/>
-      <c r="G11" s="63" t="inlineStr"/>
-      <c r="H11" s="63" t="inlineStr"/>
-      <c r="I11" s="63" t="inlineStr"/>
-      <c r="J11" s="61" t="n">
+      <c r="A11" s="64" t="inlineStr"/>
+      <c r="B11" s="64" t="inlineStr"/>
+      <c r="C11" s="64" t="inlineStr"/>
+      <c r="D11" s="64" t="inlineStr"/>
+      <c r="E11" s="64" t="inlineStr"/>
+      <c r="F11" s="64" t="inlineStr"/>
+      <c r="G11" s="64" t="inlineStr"/>
+      <c r="H11" s="64" t="inlineStr"/>
+      <c r="I11" s="64" t="inlineStr"/>
+      <c r="J11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="61" t="n">
+      <c r="K11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="64">
+      <c r="L11" s="65">
         <f>K11-J11</f>
         <v/>
       </c>
-      <c r="M11" s="65">
+      <c r="M11" s="66">
         <f>IF(J11=0,"",(K11-J11)/J11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr"/>
-      <c r="B12" s="59" t="inlineStr"/>
-      <c r="C12" s="59" t="inlineStr"/>
-      <c r="D12" s="59" t="inlineStr"/>
-      <c r="E12" s="59" t="inlineStr"/>
-      <c r="F12" s="59" t="inlineStr"/>
-      <c r="G12" s="59" t="inlineStr"/>
-      <c r="H12" s="59" t="inlineStr"/>
-      <c r="I12" s="59" t="inlineStr"/>
-      <c r="J12" s="61" t="n">
+      <c r="A12" s="60" t="inlineStr"/>
+      <c r="B12" s="60" t="inlineStr"/>
+      <c r="C12" s="60" t="inlineStr"/>
+      <c r="D12" s="60" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr"/>
+      <c r="F12" s="60" t="inlineStr"/>
+      <c r="G12" s="60" t="inlineStr"/>
+      <c r="H12" s="60" t="inlineStr"/>
+      <c r="I12" s="60" t="inlineStr"/>
+      <c r="J12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="61" t="n">
+      <c r="K12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="60">
+      <c r="L12" s="61">
         <f>K12-J12</f>
         <v/>
       </c>
-      <c r="M12" s="62">
+      <c r="M12" s="63">
         <f>IF(J12=0,"",(K12-J12)/J12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="63" t="inlineStr"/>
-      <c r="B13" s="63" t="inlineStr"/>
-      <c r="C13" s="63" t="inlineStr"/>
-      <c r="D13" s="63" t="inlineStr"/>
-      <c r="E13" s="63" t="inlineStr"/>
-      <c r="F13" s="63" t="inlineStr"/>
-      <c r="G13" s="63" t="inlineStr"/>
-      <c r="H13" s="63" t="inlineStr"/>
-      <c r="I13" s="63" t="inlineStr"/>
-      <c r="J13" s="61" t="n">
+      <c r="A13" s="64" t="inlineStr"/>
+      <c r="B13" s="64" t="inlineStr"/>
+      <c r="C13" s="64" t="inlineStr"/>
+      <c r="D13" s="64" t="inlineStr"/>
+      <c r="E13" s="64" t="inlineStr"/>
+      <c r="F13" s="64" t="inlineStr"/>
+      <c r="G13" s="64" t="inlineStr"/>
+      <c r="H13" s="64" t="inlineStr"/>
+      <c r="I13" s="64" t="inlineStr"/>
+      <c r="J13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="61" t="n">
+      <c r="K13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="64">
+      <c r="L13" s="65">
         <f>K13-J13</f>
         <v/>
       </c>
-      <c r="M13" s="65">
+      <c r="M13" s="66">
         <f>IF(J13=0,"",(K13-J13)/J13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="66" t="inlineStr">
+      <c r="A14" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="66" t="n"/>
-      <c r="C14" s="66" t="n"/>
-      <c r="D14" s="66" t="n"/>
-      <c r="E14" s="66" t="n"/>
-      <c r="F14" s="66" t="n"/>
-      <c r="G14" s="66" t="n"/>
-      <c r="H14" s="66" t="n"/>
-      <c r="I14" s="66" t="n"/>
-      <c r="J14" s="30">
+      <c r="B14" s="67" t="n"/>
+      <c r="C14" s="67" t="n"/>
+      <c r="D14" s="67" t="n"/>
+      <c r="E14" s="67" t="n"/>
+      <c r="F14" s="67" t="n"/>
+      <c r="G14" s="67" t="n"/>
+      <c r="H14" s="67" t="n"/>
+      <c r="I14" s="67" t="n"/>
+      <c r="J14" s="31">
         <f>SUM(J6:J13)</f>
         <v/>
       </c>
-      <c r="K14" s="30">
+      <c r="K14" s="31">
         <f>SUM(K6:K13)</f>
         <v/>
       </c>
-      <c r="L14" s="30">
+      <c r="L14" s="31">
         <f>K14-J14</f>
         <v/>
       </c>
-      <c r="M14" s="31">
+      <c r="M14" s="32">
         <f>IF(J14=0,"",(K14-J14)/J14)</f>
         <v/>
       </c>
@@ -13219,299 +13250,299 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Nombre del deudor</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Tipo de deudor</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>N. de identificacion</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Partes relacionadas</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr">
+      <c r="K5" s="26" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="L5" s="25" t="inlineStr">
+      <c r="L5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="M5" s="25" t="inlineStr">
+      <c r="M5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr"/>
-      <c r="B6" s="59" t="inlineStr"/>
-      <c r="C6" s="59" t="inlineStr"/>
-      <c r="D6" s="59" t="inlineStr"/>
-      <c r="E6" s="59" t="inlineStr"/>
-      <c r="F6" s="59" t="inlineStr"/>
-      <c r="G6" s="59" t="inlineStr"/>
-      <c r="H6" s="59" t="inlineStr"/>
-      <c r="I6" s="59" t="inlineStr"/>
-      <c r="J6" s="61" t="n">
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="60" t="inlineStr"/>
+      <c r="C6" s="60" t="inlineStr"/>
+      <c r="D6" s="60" t="inlineStr"/>
+      <c r="E6" s="60" t="inlineStr"/>
+      <c r="F6" s="60" t="inlineStr"/>
+      <c r="G6" s="60" t="inlineStr"/>
+      <c r="H6" s="60" t="inlineStr"/>
+      <c r="I6" s="60" t="inlineStr"/>
+      <c r="J6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="61" t="n">
+      <c r="K6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="60">
+      <c r="L6" s="61">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="62">
+      <c r="M6" s="63">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="63" t="inlineStr"/>
-      <c r="B7" s="63" t="inlineStr"/>
-      <c r="C7" s="63" t="inlineStr"/>
-      <c r="D7" s="63" t="inlineStr"/>
-      <c r="E7" s="63" t="inlineStr"/>
-      <c r="F7" s="63" t="inlineStr"/>
-      <c r="G7" s="63" t="inlineStr"/>
-      <c r="H7" s="63" t="inlineStr"/>
-      <c r="I7" s="63" t="inlineStr"/>
-      <c r="J7" s="61" t="n">
+      <c r="A7" s="64" t="inlineStr"/>
+      <c r="B7" s="64" t="inlineStr"/>
+      <c r="C7" s="64" t="inlineStr"/>
+      <c r="D7" s="64" t="inlineStr"/>
+      <c r="E7" s="64" t="inlineStr"/>
+      <c r="F7" s="64" t="inlineStr"/>
+      <c r="G7" s="64" t="inlineStr"/>
+      <c r="H7" s="64" t="inlineStr"/>
+      <c r="I7" s="64" t="inlineStr"/>
+      <c r="J7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="61" t="n">
+      <c r="K7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="64">
+      <c r="L7" s="65">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="65">
+      <c r="M7" s="66">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr"/>
-      <c r="B8" s="59" t="inlineStr"/>
-      <c r="C8" s="59" t="inlineStr"/>
-      <c r="D8" s="59" t="inlineStr"/>
-      <c r="E8" s="59" t="inlineStr"/>
-      <c r="F8" s="59" t="inlineStr"/>
-      <c r="G8" s="59" t="inlineStr"/>
-      <c r="H8" s="59" t="inlineStr"/>
-      <c r="I8" s="59" t="inlineStr"/>
-      <c r="J8" s="61" t="n">
+      <c r="A8" s="60" t="inlineStr"/>
+      <c r="B8" s="60" t="inlineStr"/>
+      <c r="C8" s="60" t="inlineStr"/>
+      <c r="D8" s="60" t="inlineStr"/>
+      <c r="E8" s="60" t="inlineStr"/>
+      <c r="F8" s="60" t="inlineStr"/>
+      <c r="G8" s="60" t="inlineStr"/>
+      <c r="H8" s="60" t="inlineStr"/>
+      <c r="I8" s="60" t="inlineStr"/>
+      <c r="J8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="61" t="n">
+      <c r="K8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="60">
+      <c r="L8" s="61">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="62">
+      <c r="M8" s="63">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="63" t="inlineStr"/>
-      <c r="B9" s="63" t="inlineStr"/>
-      <c r="C9" s="63" t="inlineStr"/>
-      <c r="D9" s="63" t="inlineStr"/>
-      <c r="E9" s="63" t="inlineStr"/>
-      <c r="F9" s="63" t="inlineStr"/>
-      <c r="G9" s="63" t="inlineStr"/>
-      <c r="H9" s="63" t="inlineStr"/>
-      <c r="I9" s="63" t="inlineStr"/>
-      <c r="J9" s="61" t="n">
+      <c r="A9" s="64" t="inlineStr"/>
+      <c r="B9" s="64" t="inlineStr"/>
+      <c r="C9" s="64" t="inlineStr"/>
+      <c r="D9" s="64" t="inlineStr"/>
+      <c r="E9" s="64" t="inlineStr"/>
+      <c r="F9" s="64" t="inlineStr"/>
+      <c r="G9" s="64" t="inlineStr"/>
+      <c r="H9" s="64" t="inlineStr"/>
+      <c r="I9" s="64" t="inlineStr"/>
+      <c r="J9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="61" t="n">
+      <c r="K9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="64">
+      <c r="L9" s="65">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="65">
+      <c r="M9" s="66">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr"/>
-      <c r="B10" s="59" t="inlineStr"/>
-      <c r="C10" s="59" t="inlineStr"/>
-      <c r="D10" s="59" t="inlineStr"/>
-      <c r="E10" s="59" t="inlineStr"/>
-      <c r="F10" s="59" t="inlineStr"/>
-      <c r="G10" s="59" t="inlineStr"/>
-      <c r="H10" s="59" t="inlineStr"/>
-      <c r="I10" s="59" t="inlineStr"/>
-      <c r="J10" s="61" t="n">
+      <c r="A10" s="60" t="inlineStr"/>
+      <c r="B10" s="60" t="inlineStr"/>
+      <c r="C10" s="60" t="inlineStr"/>
+      <c r="D10" s="60" t="inlineStr"/>
+      <c r="E10" s="60" t="inlineStr"/>
+      <c r="F10" s="60" t="inlineStr"/>
+      <c r="G10" s="60" t="inlineStr"/>
+      <c r="H10" s="60" t="inlineStr"/>
+      <c r="I10" s="60" t="inlineStr"/>
+      <c r="J10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="61" t="n">
+      <c r="K10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="60">
+      <c r="L10" s="61">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="62">
+      <c r="M10" s="63">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="63" t="inlineStr"/>
-      <c r="B11" s="63" t="inlineStr"/>
-      <c r="C11" s="63" t="inlineStr"/>
-      <c r="D11" s="63" t="inlineStr"/>
-      <c r="E11" s="63" t="inlineStr"/>
-      <c r="F11" s="63" t="inlineStr"/>
-      <c r="G11" s="63" t="inlineStr"/>
-      <c r="H11" s="63" t="inlineStr"/>
-      <c r="I11" s="63" t="inlineStr"/>
-      <c r="J11" s="61" t="n">
+      <c r="A11" s="64" t="inlineStr"/>
+      <c r="B11" s="64" t="inlineStr"/>
+      <c r="C11" s="64" t="inlineStr"/>
+      <c r="D11" s="64" t="inlineStr"/>
+      <c r="E11" s="64" t="inlineStr"/>
+      <c r="F11" s="64" t="inlineStr"/>
+      <c r="G11" s="64" t="inlineStr"/>
+      <c r="H11" s="64" t="inlineStr"/>
+      <c r="I11" s="64" t="inlineStr"/>
+      <c r="J11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="61" t="n">
+      <c r="K11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="64">
+      <c r="L11" s="65">
         <f>K11-J11</f>
         <v/>
       </c>
-      <c r="M11" s="65">
+      <c r="M11" s="66">
         <f>IF(J11=0,"",(K11-J11)/J11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr"/>
-      <c r="B12" s="59" t="inlineStr"/>
-      <c r="C12" s="59" t="inlineStr"/>
-      <c r="D12" s="59" t="inlineStr"/>
-      <c r="E12" s="59" t="inlineStr"/>
-      <c r="F12" s="59" t="inlineStr"/>
-      <c r="G12" s="59" t="inlineStr"/>
-      <c r="H12" s="59" t="inlineStr"/>
-      <c r="I12" s="59" t="inlineStr"/>
-      <c r="J12" s="61" t="n">
+      <c r="A12" s="60" t="inlineStr"/>
+      <c r="B12" s="60" t="inlineStr"/>
+      <c r="C12" s="60" t="inlineStr"/>
+      <c r="D12" s="60" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr"/>
+      <c r="F12" s="60" t="inlineStr"/>
+      <c r="G12" s="60" t="inlineStr"/>
+      <c r="H12" s="60" t="inlineStr"/>
+      <c r="I12" s="60" t="inlineStr"/>
+      <c r="J12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="61" t="n">
+      <c r="K12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="60">
+      <c r="L12" s="61">
         <f>K12-J12</f>
         <v/>
       </c>
-      <c r="M12" s="62">
+      <c r="M12" s="63">
         <f>IF(J12=0,"",(K12-J12)/J12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="63" t="inlineStr"/>
-      <c r="B13" s="63" t="inlineStr"/>
-      <c r="C13" s="63" t="inlineStr"/>
-      <c r="D13" s="63" t="inlineStr"/>
-      <c r="E13" s="63" t="inlineStr"/>
-      <c r="F13" s="63" t="inlineStr"/>
-      <c r="G13" s="63" t="inlineStr"/>
-      <c r="H13" s="63" t="inlineStr"/>
-      <c r="I13" s="63" t="inlineStr"/>
-      <c r="J13" s="61" t="n">
+      <c r="A13" s="64" t="inlineStr"/>
+      <c r="B13" s="64" t="inlineStr"/>
+      <c r="C13" s="64" t="inlineStr"/>
+      <c r="D13" s="64" t="inlineStr"/>
+      <c r="E13" s="64" t="inlineStr"/>
+      <c r="F13" s="64" t="inlineStr"/>
+      <c r="G13" s="64" t="inlineStr"/>
+      <c r="H13" s="64" t="inlineStr"/>
+      <c r="I13" s="64" t="inlineStr"/>
+      <c r="J13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="61" t="n">
+      <c r="K13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="64">
+      <c r="L13" s="65">
         <f>K13-J13</f>
         <v/>
       </c>
-      <c r="M13" s="65">
+      <c r="M13" s="66">
         <f>IF(J13=0,"",(K13-J13)/J13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="66" t="inlineStr">
+      <c r="A14" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="66" t="n"/>
-      <c r="C14" s="66" t="n"/>
-      <c r="D14" s="66" t="n"/>
-      <c r="E14" s="66" t="n"/>
-      <c r="F14" s="66" t="n"/>
-      <c r="G14" s="66" t="n"/>
-      <c r="H14" s="66" t="n"/>
-      <c r="I14" s="66" t="n"/>
-      <c r="J14" s="30">
+      <c r="B14" s="67" t="n"/>
+      <c r="C14" s="67" t="n"/>
+      <c r="D14" s="67" t="n"/>
+      <c r="E14" s="67" t="n"/>
+      <c r="F14" s="67" t="n"/>
+      <c r="G14" s="67" t="n"/>
+      <c r="H14" s="67" t="n"/>
+      <c r="I14" s="67" t="n"/>
+      <c r="J14" s="31">
         <f>SUM(J6:J13)</f>
         <v/>
       </c>
-      <c r="K14" s="30">
+      <c r="K14" s="31">
         <f>SUM(K6:K13)</f>
         <v/>
       </c>
-      <c r="L14" s="30">
+      <c r="L14" s="31">
         <f>K14-J14</f>
         <v/>
       </c>
-      <c r="M14" s="31">
+      <c r="M14" s="32">
         <f>IF(J14=0,"",(K14-J14)/J14)</f>
         <v/>
       </c>
@@ -13584,243 +13615,243 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Tipo de bien</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr"/>
-      <c r="B6" s="59" t="inlineStr"/>
-      <c r="C6" s="59" t="inlineStr"/>
-      <c r="D6" s="59" t="inlineStr"/>
-      <c r="E6" s="59" t="inlineStr"/>
-      <c r="F6" s="61" t="n">
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="60" t="inlineStr"/>
+      <c r="C6" s="60" t="inlineStr"/>
+      <c r="D6" s="60" t="inlineStr"/>
+      <c r="E6" s="60" t="inlineStr"/>
+      <c r="F6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="61" t="n">
+      <c r="G6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="60">
+      <c r="H6" s="61">
         <f>G6-F6</f>
         <v/>
       </c>
-      <c r="I6" s="62">
+      <c r="I6" s="63">
         <f>IF(F6=0,"",(G6-F6)/F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="63" t="inlineStr"/>
-      <c r="B7" s="63" t="inlineStr"/>
-      <c r="C7" s="63" t="inlineStr"/>
-      <c r="D7" s="63" t="inlineStr"/>
-      <c r="E7" s="63" t="inlineStr"/>
-      <c r="F7" s="61" t="n">
+      <c r="A7" s="64" t="inlineStr"/>
+      <c r="B7" s="64" t="inlineStr"/>
+      <c r="C7" s="64" t="inlineStr"/>
+      <c r="D7" s="64" t="inlineStr"/>
+      <c r="E7" s="64" t="inlineStr"/>
+      <c r="F7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="61" t="n">
+      <c r="G7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="64">
+      <c r="H7" s="65">
         <f>G7-F7</f>
         <v/>
       </c>
-      <c r="I7" s="65">
+      <c r="I7" s="66">
         <f>IF(F7=0,"",(G7-F7)/F7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr"/>
-      <c r="B8" s="59" t="inlineStr"/>
-      <c r="C8" s="59" t="inlineStr"/>
-      <c r="D8" s="59" t="inlineStr"/>
-      <c r="E8" s="59" t="inlineStr"/>
-      <c r="F8" s="61" t="n">
+      <c r="A8" s="60" t="inlineStr"/>
+      <c r="B8" s="60" t="inlineStr"/>
+      <c r="C8" s="60" t="inlineStr"/>
+      <c r="D8" s="60" t="inlineStr"/>
+      <c r="E8" s="60" t="inlineStr"/>
+      <c r="F8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="61" t="n">
+      <c r="G8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="60">
+      <c r="H8" s="61">
         <f>G8-F8</f>
         <v/>
       </c>
-      <c r="I8" s="62">
+      <c r="I8" s="63">
         <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="63" t="inlineStr"/>
-      <c r="B9" s="63" t="inlineStr"/>
-      <c r="C9" s="63" t="inlineStr"/>
-      <c r="D9" s="63" t="inlineStr"/>
-      <c r="E9" s="63" t="inlineStr"/>
-      <c r="F9" s="61" t="n">
+      <c r="A9" s="64" t="inlineStr"/>
+      <c r="B9" s="64" t="inlineStr"/>
+      <c r="C9" s="64" t="inlineStr"/>
+      <c r="D9" s="64" t="inlineStr"/>
+      <c r="E9" s="64" t="inlineStr"/>
+      <c r="F9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="61" t="n">
+      <c r="G9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="64">
+      <c r="H9" s="65">
         <f>G9-F9</f>
         <v/>
       </c>
-      <c r="I9" s="65">
+      <c r="I9" s="66">
         <f>IF(F9=0,"",(G9-F9)/F9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr"/>
-      <c r="B10" s="59" t="inlineStr"/>
-      <c r="C10" s="59" t="inlineStr"/>
-      <c r="D10" s="59" t="inlineStr"/>
-      <c r="E10" s="59" t="inlineStr"/>
-      <c r="F10" s="61" t="n">
+      <c r="A10" s="60" t="inlineStr"/>
+      <c r="B10" s="60" t="inlineStr"/>
+      <c r="C10" s="60" t="inlineStr"/>
+      <c r="D10" s="60" t="inlineStr"/>
+      <c r="E10" s="60" t="inlineStr"/>
+      <c r="F10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="61" t="n">
+      <c r="G10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="60">
+      <c r="H10" s="61">
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="62">
+      <c r="I10" s="63">
         <f>IF(F10=0,"",(G10-F10)/F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="63" t="inlineStr"/>
-      <c r="B11" s="63" t="inlineStr"/>
-      <c r="C11" s="63" t="inlineStr"/>
-      <c r="D11" s="63" t="inlineStr"/>
-      <c r="E11" s="63" t="inlineStr"/>
-      <c r="F11" s="61" t="n">
+      <c r="A11" s="64" t="inlineStr"/>
+      <c r="B11" s="64" t="inlineStr"/>
+      <c r="C11" s="64" t="inlineStr"/>
+      <c r="D11" s="64" t="inlineStr"/>
+      <c r="E11" s="64" t="inlineStr"/>
+      <c r="F11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="61" t="n">
+      <c r="G11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="64">
+      <c r="H11" s="65">
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="65">
+      <c r="I11" s="66">
         <f>IF(F11=0,"",(G11-F11)/F11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr"/>
-      <c r="B12" s="59" t="inlineStr"/>
-      <c r="C12" s="59" t="inlineStr"/>
-      <c r="D12" s="59" t="inlineStr"/>
-      <c r="E12" s="59" t="inlineStr"/>
-      <c r="F12" s="61" t="n">
+      <c r="A12" s="60" t="inlineStr"/>
+      <c r="B12" s="60" t="inlineStr"/>
+      <c r="C12" s="60" t="inlineStr"/>
+      <c r="D12" s="60" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr"/>
+      <c r="F12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="61" t="n">
+      <c r="G12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="60">
+      <c r="H12" s="61">
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="62">
+      <c r="I12" s="63">
         <f>IF(F12=0,"",(G12-F12)/F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="63" t="inlineStr"/>
-      <c r="B13" s="63" t="inlineStr"/>
-      <c r="C13" s="63" t="inlineStr"/>
-      <c r="D13" s="63" t="inlineStr"/>
-      <c r="E13" s="63" t="inlineStr"/>
-      <c r="F13" s="61" t="n">
+      <c r="A13" s="64" t="inlineStr"/>
+      <c r="B13" s="64" t="inlineStr"/>
+      <c r="C13" s="64" t="inlineStr"/>
+      <c r="D13" s="64" t="inlineStr"/>
+      <c r="E13" s="64" t="inlineStr"/>
+      <c r="F13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="61" t="n">
+      <c r="G13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="64">
+      <c r="H13" s="65">
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="65">
+      <c r="I13" s="66">
         <f>IF(F13=0,"",(G13-F13)/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="66" t="inlineStr">
+      <c r="A14" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="66" t="n"/>
-      <c r="C14" s="66" t="n"/>
-      <c r="D14" s="66" t="n"/>
-      <c r="E14" s="66" t="n"/>
-      <c r="F14" s="30">
+      <c r="B14" s="67" t="n"/>
+      <c r="C14" s="67" t="n"/>
+      <c r="D14" s="67" t="n"/>
+      <c r="E14" s="67" t="n"/>
+      <c r="F14" s="31">
         <f>SUM(F6:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="30">
+      <c r="G14" s="31">
         <f>SUM(G6:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="31">
         <f>G14-F14</f>
         <v/>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="32">
         <f>IF(F14=0,"",(G14-F14)/F14)</f>
         <v/>
       </c>
@@ -13888,195 +13919,195 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Tipo de vehiculo</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Registro / placa / chasis</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>1 - Vehiculos motorizados terrestres</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>PBO7092</t>
         </is>
       </c>
-      <c r="C6" s="59" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr"/>
-      <c r="F6" s="59" t="inlineStr"/>
-      <c r="G6" s="60" t="n">
+      <c r="E6" s="60" t="inlineStr"/>
+      <c r="F6" s="60" t="inlineStr"/>
+      <c r="G6" s="61" t="n">
         <v>12000</v>
       </c>
-      <c r="H6" s="61" t="n">
+      <c r="H6" s="62" t="n">
         <v>12000</v>
       </c>
-      <c r="I6" s="60">
+      <c r="I6" s="61">
         <f>H6-G6</f>
         <v/>
       </c>
-      <c r="J6" s="62">
+      <c r="J6" s="63">
         <f>IF(G6=0,"",(H6-G6)/G6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="63" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>1 - Vehiculos motorizados terrestres</t>
         </is>
       </c>
-      <c r="B7" s="63" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>PBF9690</t>
         </is>
       </c>
-      <c r="C7" s="63" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D7" s="63" t="inlineStr">
+      <c r="D7" s="64" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E7" s="63" t="inlineStr"/>
-      <c r="F7" s="63" t="inlineStr"/>
-      <c r="G7" s="64" t="n">
+      <c r="E7" s="64" t="inlineStr"/>
+      <c r="F7" s="64" t="inlineStr"/>
+      <c r="G7" s="65" t="n">
         <v>20000</v>
       </c>
-      <c r="H7" s="61" t="n">
+      <c r="H7" s="62" t="n">
         <v>20000</v>
       </c>
-      <c r="I7" s="64">
+      <c r="I7" s="65">
         <f>H7-G7</f>
         <v/>
       </c>
-      <c r="J7" s="65">
+      <c r="J7" s="66">
         <f>IF(G7=0,"",(H7-G7)/G7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>1 - Vehiculos motorizados terrestres</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>PFC8683</t>
         </is>
       </c>
-      <c r="C8" s="59" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D8" s="59" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E8" s="59" t="inlineStr"/>
-      <c r="F8" s="59" t="inlineStr"/>
-      <c r="G8" s="60" t="n">
+      <c r="E8" s="60" t="inlineStr"/>
+      <c r="F8" s="60" t="inlineStr"/>
+      <c r="G8" s="61" t="n">
         <v>32000</v>
       </c>
-      <c r="H8" s="61" t="n">
+      <c r="H8" s="62" t="n">
         <v>32000</v>
       </c>
-      <c r="I8" s="60">
+      <c r="I8" s="61">
         <f>H8-G8</f>
         <v/>
       </c>
-      <c r="J8" s="62">
+      <c r="J8" s="63">
         <f>IF(G8=0,"",(H8-G8)/G8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="66" t="inlineStr">
+      <c r="A9" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="66" t="n"/>
-      <c r="C9" s="66" t="n"/>
-      <c r="D9" s="66" t="n"/>
-      <c r="E9" s="66" t="n"/>
-      <c r="F9" s="66" t="n"/>
-      <c r="G9" s="30">
+      <c r="B9" s="67" t="n"/>
+      <c r="C9" s="67" t="n"/>
+      <c r="D9" s="67" t="n"/>
+      <c r="E9" s="67" t="n"/>
+      <c r="F9" s="67" t="n"/>
+      <c r="G9" s="31">
         <f>SUM(G6:G8)</f>
         <v/>
       </c>
-      <c r="H9" s="30">
+      <c r="H9" s="31">
         <f>SUM(H6:H8)</f>
         <v/>
       </c>
-      <c r="I9" s="30">
+      <c r="I9" s="31">
         <f>H9-G9</f>
         <v/>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="32">
         <f>IF(G9=0,"",(H9-G9)/G9)</f>
         <v/>
       </c>
@@ -14143,243 +14174,243 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Tipo de derecho</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr"/>
-      <c r="B6" s="59" t="inlineStr"/>
-      <c r="C6" s="59" t="inlineStr"/>
-      <c r="D6" s="59" t="inlineStr"/>
-      <c r="E6" s="59" t="inlineStr"/>
-      <c r="F6" s="61" t="n">
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="60" t="inlineStr"/>
+      <c r="C6" s="60" t="inlineStr"/>
+      <c r="D6" s="60" t="inlineStr"/>
+      <c r="E6" s="60" t="inlineStr"/>
+      <c r="F6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="61" t="n">
+      <c r="G6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="60">
+      <c r="H6" s="61">
         <f>G6-F6</f>
         <v/>
       </c>
-      <c r="I6" s="62">
+      <c r="I6" s="63">
         <f>IF(F6=0,"",(G6-F6)/F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="63" t="inlineStr"/>
-      <c r="B7" s="63" t="inlineStr"/>
-      <c r="C7" s="63" t="inlineStr"/>
-      <c r="D7" s="63" t="inlineStr"/>
-      <c r="E7" s="63" t="inlineStr"/>
-      <c r="F7" s="61" t="n">
+      <c r="A7" s="64" t="inlineStr"/>
+      <c r="B7" s="64" t="inlineStr"/>
+      <c r="C7" s="64" t="inlineStr"/>
+      <c r="D7" s="64" t="inlineStr"/>
+      <c r="E7" s="64" t="inlineStr"/>
+      <c r="F7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="61" t="n">
+      <c r="G7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="64">
+      <c r="H7" s="65">
         <f>G7-F7</f>
         <v/>
       </c>
-      <c r="I7" s="65">
+      <c r="I7" s="66">
         <f>IF(F7=0,"",(G7-F7)/F7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr"/>
-      <c r="B8" s="59" t="inlineStr"/>
-      <c r="C8" s="59" t="inlineStr"/>
-      <c r="D8" s="59" t="inlineStr"/>
-      <c r="E8" s="59" t="inlineStr"/>
-      <c r="F8" s="61" t="n">
+      <c r="A8" s="60" t="inlineStr"/>
+      <c r="B8" s="60" t="inlineStr"/>
+      <c r="C8" s="60" t="inlineStr"/>
+      <c r="D8" s="60" t="inlineStr"/>
+      <c r="E8" s="60" t="inlineStr"/>
+      <c r="F8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="61" t="n">
+      <c r="G8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="60">
+      <c r="H8" s="61">
         <f>G8-F8</f>
         <v/>
       </c>
-      <c r="I8" s="62">
+      <c r="I8" s="63">
         <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="63" t="inlineStr"/>
-      <c r="B9" s="63" t="inlineStr"/>
-      <c r="C9" s="63" t="inlineStr"/>
-      <c r="D9" s="63" t="inlineStr"/>
-      <c r="E9" s="63" t="inlineStr"/>
-      <c r="F9" s="61" t="n">
+      <c r="A9" s="64" t="inlineStr"/>
+      <c r="B9" s="64" t="inlineStr"/>
+      <c r="C9" s="64" t="inlineStr"/>
+      <c r="D9" s="64" t="inlineStr"/>
+      <c r="E9" s="64" t="inlineStr"/>
+      <c r="F9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="61" t="n">
+      <c r="G9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="64">
+      <c r="H9" s="65">
         <f>G9-F9</f>
         <v/>
       </c>
-      <c r="I9" s="65">
+      <c r="I9" s="66">
         <f>IF(F9=0,"",(G9-F9)/F9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr"/>
-      <c r="B10" s="59" t="inlineStr"/>
-      <c r="C10" s="59" t="inlineStr"/>
-      <c r="D10" s="59" t="inlineStr"/>
-      <c r="E10" s="59" t="inlineStr"/>
-      <c r="F10" s="61" t="n">
+      <c r="A10" s="60" t="inlineStr"/>
+      <c r="B10" s="60" t="inlineStr"/>
+      <c r="C10" s="60" t="inlineStr"/>
+      <c r="D10" s="60" t="inlineStr"/>
+      <c r="E10" s="60" t="inlineStr"/>
+      <c r="F10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="61" t="n">
+      <c r="G10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="60">
+      <c r="H10" s="61">
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="62">
+      <c r="I10" s="63">
         <f>IF(F10=0,"",(G10-F10)/F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="63" t="inlineStr"/>
-      <c r="B11" s="63" t="inlineStr"/>
-      <c r="C11" s="63" t="inlineStr"/>
-      <c r="D11" s="63" t="inlineStr"/>
-      <c r="E11" s="63" t="inlineStr"/>
-      <c r="F11" s="61" t="n">
+      <c r="A11" s="64" t="inlineStr"/>
+      <c r="B11" s="64" t="inlineStr"/>
+      <c r="C11" s="64" t="inlineStr"/>
+      <c r="D11" s="64" t="inlineStr"/>
+      <c r="E11" s="64" t="inlineStr"/>
+      <c r="F11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="61" t="n">
+      <c r="G11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="64">
+      <c r="H11" s="65">
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="65">
+      <c r="I11" s="66">
         <f>IF(F11=0,"",(G11-F11)/F11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr"/>
-      <c r="B12" s="59" t="inlineStr"/>
-      <c r="C12" s="59" t="inlineStr"/>
-      <c r="D12" s="59" t="inlineStr"/>
-      <c r="E12" s="59" t="inlineStr"/>
-      <c r="F12" s="61" t="n">
+      <c r="A12" s="60" t="inlineStr"/>
+      <c r="B12" s="60" t="inlineStr"/>
+      <c r="C12" s="60" t="inlineStr"/>
+      <c r="D12" s="60" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr"/>
+      <c r="F12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="61" t="n">
+      <c r="G12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="60">
+      <c r="H12" s="61">
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="62">
+      <c r="I12" s="63">
         <f>IF(F12=0,"",(G12-F12)/F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="63" t="inlineStr"/>
-      <c r="B13" s="63" t="inlineStr"/>
-      <c r="C13" s="63" t="inlineStr"/>
-      <c r="D13" s="63" t="inlineStr"/>
-      <c r="E13" s="63" t="inlineStr"/>
-      <c r="F13" s="61" t="n">
+      <c r="A13" s="64" t="inlineStr"/>
+      <c r="B13" s="64" t="inlineStr"/>
+      <c r="C13" s="64" t="inlineStr"/>
+      <c r="D13" s="64" t="inlineStr"/>
+      <c r="E13" s="64" t="inlineStr"/>
+      <c r="F13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="61" t="n">
+      <c r="G13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="64">
+      <c r="H13" s="65">
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="65">
+      <c r="I13" s="66">
         <f>IF(F13=0,"",(G13-F13)/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="66" t="inlineStr">
+      <c r="A14" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="66" t="n"/>
-      <c r="C14" s="66" t="n"/>
-      <c r="D14" s="66" t="n"/>
-      <c r="E14" s="66" t="n"/>
-      <c r="F14" s="30">
+      <c r="B14" s="67" t="n"/>
+      <c r="C14" s="67" t="n"/>
+      <c r="D14" s="67" t="n"/>
+      <c r="E14" s="67" t="n"/>
+      <c r="F14" s="31">
         <f>SUM(F6:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="30">
+      <c r="G14" s="31">
         <f>SUM(G6:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="31">
         <f>G14-F14</f>
         <v/>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="32">
         <f>IF(F14=0,"",(G14-F14)/F14)</f>
         <v/>
       </c>
@@ -14450,303 +14481,303 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Tipo de inmueble</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Provincia</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Canton</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Fecha de inscripcion</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Clave catastral</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr">
+      <c r="K5" s="26" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="L5" s="25" t="inlineStr">
+      <c r="L5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="M5" s="25" t="inlineStr">
+      <c r="M5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>3 - Terreno</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C6" s="59" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr">
+      <c r="E6" s="60" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F6" s="59" t="inlineStr">
+      <c r="F6" s="60" t="inlineStr">
         <is>
           <t>22/10/2008</t>
         </is>
       </c>
-      <c r="G6" s="59" t="inlineStr">
+      <c r="G6" s="60" t="inlineStr">
         <is>
           <t>1042203018</t>
         </is>
       </c>
-      <c r="H6" s="59" t="inlineStr"/>
-      <c r="I6" s="59" t="inlineStr"/>
-      <c r="J6" s="60" t="n">
+      <c r="H6" s="60" t="inlineStr"/>
+      <c r="I6" s="60" t="inlineStr"/>
+      <c r="J6" s="61" t="n">
         <v>267340.8</v>
       </c>
-      <c r="K6" s="61" t="n">
+      <c r="K6" s="62" t="n">
         <v>267340.8</v>
       </c>
-      <c r="L6" s="60">
+      <c r="L6" s="61">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="62">
+      <c r="M6" s="63">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="63" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>1 - Casa</t>
         </is>
       </c>
-      <c r="B7" s="63" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C7" s="63" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D7" s="63" t="inlineStr">
+      <c r="D7" s="64" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E7" s="63" t="inlineStr">
+      <c r="E7" s="64" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F7" s="63" t="inlineStr">
+      <c r="F7" s="64" t="inlineStr">
         <is>
           <t>13/03/1997</t>
         </is>
       </c>
-      <c r="G7" s="63" t="inlineStr">
+      <c r="G7" s="64" t="inlineStr">
         <is>
           <t>1012005008000000000</t>
         </is>
       </c>
-      <c r="H7" s="63" t="inlineStr"/>
-      <c r="I7" s="63" t="inlineStr"/>
-      <c r="J7" s="64" t="n">
+      <c r="H7" s="64" t="inlineStr"/>
+      <c r="I7" s="64" t="inlineStr"/>
+      <c r="J7" s="65" t="n">
         <v>198118.55</v>
       </c>
-      <c r="K7" s="61" t="n">
+      <c r="K7" s="62" t="n">
         <v>198118.55</v>
       </c>
-      <c r="L7" s="64">
+      <c r="L7" s="65">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="65">
+      <c r="M7" s="66">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>1 - Casa</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C8" s="59" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D8" s="59" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E8" s="59" t="inlineStr">
+      <c r="E8" s="60" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F8" s="59" t="inlineStr"/>
-      <c r="G8" s="59" t="inlineStr">
+      <c r="F8" s="60" t="inlineStr"/>
+      <c r="G8" s="60" t="inlineStr">
         <is>
           <t>1042203018</t>
         </is>
       </c>
-      <c r="H8" s="59" t="inlineStr"/>
-      <c r="I8" s="59" t="inlineStr"/>
-      <c r="J8" s="60" t="n">
+      <c r="H8" s="60" t="inlineStr"/>
+      <c r="I8" s="60" t="inlineStr"/>
+      <c r="J8" s="61" t="n">
         <v>33634.04</v>
       </c>
-      <c r="K8" s="61" t="n">
+      <c r="K8" s="62" t="n">
         <v>33634.04</v>
       </c>
-      <c r="L8" s="60">
+      <c r="L8" s="61">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="62">
+      <c r="M8" s="63">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="63" t="inlineStr">
+      <c r="A9" s="64" t="inlineStr">
         <is>
           <t>3 - Terreno</t>
         </is>
       </c>
-      <c r="B9" s="63" t="inlineStr">
+      <c r="B9" s="64" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C9" s="63" t="inlineStr">
+      <c r="C9" s="64" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D9" s="63" t="inlineStr">
+      <c r="D9" s="64" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E9" s="63" t="inlineStr">
+      <c r="E9" s="64" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F9" s="63" t="inlineStr"/>
-      <c r="G9" s="63" t="inlineStr">
+      <c r="F9" s="64" t="inlineStr"/>
+      <c r="G9" s="64" t="inlineStr">
         <is>
           <t>1012005008000000000</t>
         </is>
       </c>
-      <c r="H9" s="63" t="inlineStr"/>
-      <c r="I9" s="63" t="inlineStr"/>
-      <c r="J9" s="64" t="n">
+      <c r="H9" s="64" t="inlineStr"/>
+      <c r="I9" s="64" t="inlineStr"/>
+      <c r="J9" s="65" t="n">
         <v>82624.22</v>
       </c>
-      <c r="K9" s="61" t="n">
+      <c r="K9" s="62" t="n">
         <v>82624.22</v>
       </c>
-      <c r="L9" s="64">
+      <c r="L9" s="65">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="65">
+      <c r="M9" s="66">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="66" t="inlineStr">
+      <c r="A10" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B10" s="66" t="n"/>
-      <c r="C10" s="66" t="n"/>
-      <c r="D10" s="66" t="n"/>
-      <c r="E10" s="66" t="n"/>
-      <c r="F10" s="66" t="n"/>
-      <c r="G10" s="66" t="n"/>
-      <c r="H10" s="66" t="n"/>
-      <c r="I10" s="66" t="n"/>
-      <c r="J10" s="30">
+      <c r="B10" s="67" t="n"/>
+      <c r="C10" s="67" t="n"/>
+      <c r="D10" s="67" t="n"/>
+      <c r="E10" s="67" t="n"/>
+      <c r="F10" s="67" t="n"/>
+      <c r="G10" s="67" t="n"/>
+      <c r="H10" s="67" t="n"/>
+      <c r="I10" s="67" t="n"/>
+      <c r="J10" s="31">
         <f>SUM(J6:J9)</f>
         <v/>
       </c>
-      <c r="K10" s="30">
+      <c r="K10" s="31">
         <f>SUM(K6:K9)</f>
         <v/>
       </c>
-      <c r="L10" s="30">
+      <c r="L10" s="31">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="31">
+      <c r="M10" s="32">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
@@ -14819,243 +14850,243 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Pais</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Descripcion</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Regularizacion activos</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Anio fiscal adquisicion</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Valor 2025</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>Valor 2026</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Variacion</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Variacion %</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr"/>
-      <c r="B6" s="59" t="inlineStr"/>
-      <c r="C6" s="59" t="inlineStr"/>
-      <c r="D6" s="59" t="inlineStr"/>
-      <c r="E6" s="59" t="inlineStr"/>
-      <c r="F6" s="61" t="n">
+      <c r="A6" s="60" t="inlineStr"/>
+      <c r="B6" s="60" t="inlineStr"/>
+      <c r="C6" s="60" t="inlineStr"/>
+      <c r="D6" s="60" t="inlineStr"/>
+      <c r="E6" s="60" t="inlineStr"/>
+      <c r="F6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="61" t="n">
+      <c r="G6" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="60">
+      <c r="H6" s="61">
         <f>G6-F6</f>
         <v/>
       </c>
-      <c r="I6" s="62">
+      <c r="I6" s="63">
         <f>IF(F6=0,"",(G6-F6)/F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="63" t="inlineStr"/>
-      <c r="B7" s="63" t="inlineStr"/>
-      <c r="C7" s="63" t="inlineStr"/>
-      <c r="D7" s="63" t="inlineStr"/>
-      <c r="E7" s="63" t="inlineStr"/>
-      <c r="F7" s="61" t="n">
+      <c r="A7" s="64" t="inlineStr"/>
+      <c r="B7" s="64" t="inlineStr"/>
+      <c r="C7" s="64" t="inlineStr"/>
+      <c r="D7" s="64" t="inlineStr"/>
+      <c r="E7" s="64" t="inlineStr"/>
+      <c r="F7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="61" t="n">
+      <c r="G7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="64">
+      <c r="H7" s="65">
         <f>G7-F7</f>
         <v/>
       </c>
-      <c r="I7" s="65">
+      <c r="I7" s="66">
         <f>IF(F7=0,"",(G7-F7)/F7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr"/>
-      <c r="B8" s="59" t="inlineStr"/>
-      <c r="C8" s="59" t="inlineStr"/>
-      <c r="D8" s="59" t="inlineStr"/>
-      <c r="E8" s="59" t="inlineStr"/>
-      <c r="F8" s="61" t="n">
+      <c r="A8" s="60" t="inlineStr"/>
+      <c r="B8" s="60" t="inlineStr"/>
+      <c r="C8" s="60" t="inlineStr"/>
+      <c r="D8" s="60" t="inlineStr"/>
+      <c r="E8" s="60" t="inlineStr"/>
+      <c r="F8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="61" t="n">
+      <c r="G8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="60">
+      <c r="H8" s="61">
         <f>G8-F8</f>
         <v/>
       </c>
-      <c r="I8" s="62">
+      <c r="I8" s="63">
         <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="63" t="inlineStr"/>
-      <c r="B9" s="63" t="inlineStr"/>
-      <c r="C9" s="63" t="inlineStr"/>
-      <c r="D9" s="63" t="inlineStr"/>
-      <c r="E9" s="63" t="inlineStr"/>
-      <c r="F9" s="61" t="n">
+      <c r="A9" s="64" t="inlineStr"/>
+      <c r="B9" s="64" t="inlineStr"/>
+      <c r="C9" s="64" t="inlineStr"/>
+      <c r="D9" s="64" t="inlineStr"/>
+      <c r="E9" s="64" t="inlineStr"/>
+      <c r="F9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="61" t="n">
+      <c r="G9" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="64">
+      <c r="H9" s="65">
         <f>G9-F9</f>
         <v/>
       </c>
-      <c r="I9" s="65">
+      <c r="I9" s="66">
         <f>IF(F9=0,"",(G9-F9)/F9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr"/>
-      <c r="B10" s="59" t="inlineStr"/>
-      <c r="C10" s="59" t="inlineStr"/>
-      <c r="D10" s="59" t="inlineStr"/>
-      <c r="E10" s="59" t="inlineStr"/>
-      <c r="F10" s="61" t="n">
+      <c r="A10" s="60" t="inlineStr"/>
+      <c r="B10" s="60" t="inlineStr"/>
+      <c r="C10" s="60" t="inlineStr"/>
+      <c r="D10" s="60" t="inlineStr"/>
+      <c r="E10" s="60" t="inlineStr"/>
+      <c r="F10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="61" t="n">
+      <c r="G10" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="60">
+      <c r="H10" s="61">
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="62">
+      <c r="I10" s="63">
         <f>IF(F10=0,"",(G10-F10)/F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="63" t="inlineStr"/>
-      <c r="B11" s="63" t="inlineStr"/>
-      <c r="C11" s="63" t="inlineStr"/>
-      <c r="D11" s="63" t="inlineStr"/>
-      <c r="E11" s="63" t="inlineStr"/>
-      <c r="F11" s="61" t="n">
+      <c r="A11" s="64" t="inlineStr"/>
+      <c r="B11" s="64" t="inlineStr"/>
+      <c r="C11" s="64" t="inlineStr"/>
+      <c r="D11" s="64" t="inlineStr"/>
+      <c r="E11" s="64" t="inlineStr"/>
+      <c r="F11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="61" t="n">
+      <c r="G11" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="64">
+      <c r="H11" s="65">
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="65">
+      <c r="I11" s="66">
         <f>IF(F11=0,"",(G11-F11)/F11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr"/>
-      <c r="B12" s="59" t="inlineStr"/>
-      <c r="C12" s="59" t="inlineStr"/>
-      <c r="D12" s="59" t="inlineStr"/>
-      <c r="E12" s="59" t="inlineStr"/>
-      <c r="F12" s="61" t="n">
+      <c r="A12" s="60" t="inlineStr"/>
+      <c r="B12" s="60" t="inlineStr"/>
+      <c r="C12" s="60" t="inlineStr"/>
+      <c r="D12" s="60" t="inlineStr"/>
+      <c r="E12" s="60" t="inlineStr"/>
+      <c r="F12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="61" t="n">
+      <c r="G12" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="60">
+      <c r="H12" s="61">
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="62">
+      <c r="I12" s="63">
         <f>IF(F12=0,"",(G12-F12)/F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="63" t="inlineStr"/>
-      <c r="B13" s="63" t="inlineStr"/>
-      <c r="C13" s="63" t="inlineStr"/>
-      <c r="D13" s="63" t="inlineStr"/>
-      <c r="E13" s="63" t="inlineStr"/>
-      <c r="F13" s="61" t="n">
+      <c r="A13" s="64" t="inlineStr"/>
+      <c r="B13" s="64" t="inlineStr"/>
+      <c r="C13" s="64" t="inlineStr"/>
+      <c r="D13" s="64" t="inlineStr"/>
+      <c r="E13" s="64" t="inlineStr"/>
+      <c r="F13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="61" t="n">
+      <c r="G13" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="64">
+      <c r="H13" s="65">
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="65">
+      <c r="I13" s="66">
         <f>IF(F13=0,"",(G13-F13)/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="66" t="inlineStr">
+      <c r="A14" s="67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="66" t="n"/>
-      <c r="C14" s="66" t="n"/>
-      <c r="D14" s="66" t="n"/>
-      <c r="E14" s="66" t="n"/>
-      <c r="F14" s="30">
+      <c r="B14" s="67" t="n"/>
+      <c r="C14" s="67" t="n"/>
+      <c r="D14" s="67" t="n"/>
+      <c r="E14" s="67" t="n"/>
+      <c r="F14" s="31">
         <f>SUM(F6:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="30">
+      <c r="G14" s="31">
         <f>SUM(G6:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="31">
         <f>G14-F14</f>
         <v/>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="32">
         <f>IF(F14=0,"",(G14-F14)/F14)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat(tools): hoja de datos editable y reutilizable
La hoja "Datos del XML" ahora tiene celdas editables (amarillas) para la
identificacion del declarante y conyuge y el patrimonio declarado
(atribuible a hijos, sociedad conyugal, individual, anio anterior), con
listas desplegables del catalogo del SRI. Permite reutilizar la
plantilla cambiando los datos de la persona. Incluye el libro generado
con los datos del declarante GEDEON.

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -434,7 +434,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2341,7 +2341,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2351,13 +2351,20 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Edite las celdas amarillas para reutilizar la plantilla con otra persona; el XML se genera con estos datos</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="5" customHeight="1">
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="78" t="inlineStr">
         <is>
-          <t>IDENTIFICACION</t>
+          <t>IDENTIFICACION DEL DECLARANTE Y CONYUGE  (editable)</t>
         </is>
       </c>
     </row>
@@ -2458,129 +2465,127 @@
     <row r="14">
       <c r="A14" s="79" t="inlineStr">
         <is>
-          <t>Total creditos / cuentas por cobrar</t>
-        </is>
-      </c>
-      <c r="B14" s="61" t="n">
-        <v>0</v>
-      </c>
+          <t>Regularizacion de activos</t>
+        </is>
+      </c>
+      <c r="B14" s="80" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="78" t="inlineStr">
         <is>
-          <t>PATRIMONIO NETO (enlazado a la hoja Dashboard)</t>
+          <t>PATRIMONIO DECLARADO  (editable)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="79" t="inlineStr">
         <is>
-          <t>Patrimonio neto 2025</t>
-        </is>
-      </c>
-      <c r="B17" s="61">
-        <f>Dashboard!D31</f>
-        <v/>
+          <t>Patrimonio total declarado</t>
+        </is>
+      </c>
+      <c r="B17" s="61" t="n">
+        <v>883285.5600000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="79" t="inlineStr">
         <is>
-          <t>Patrimonio neto 2026 (proyectado)</t>
-        </is>
-      </c>
-      <c r="B18" s="61">
-        <f>Dashboard!E31</f>
-        <v/>
+          <t>Atribuible a hijos no emancipados</t>
+        </is>
+      </c>
+      <c r="B18" s="62" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="79" t="inlineStr">
         <is>
-          <t>Variacion proyectada</t>
-        </is>
-      </c>
-      <c r="B19" s="61">
-        <f>Dashboard!F31</f>
-        <v/>
+          <t>Patrimonio en la sociedad conyugal</t>
+        </is>
+      </c>
+      <c r="B19" s="62" t="n">
+        <v>883285.5600000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="79" t="inlineStr">
         <is>
-          <t>Variacion % proyectada</t>
-        </is>
-      </c>
-      <c r="B20" s="63">
-        <f>Dashboard!G31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="78" t="inlineStr">
-        <is>
-          <t>PATRIMONIO DECLARADO EN EL XML</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="79" t="inlineStr">
-        <is>
-          <t>Patrimonio total declarado</t>
-        </is>
-      </c>
-      <c r="B23" s="61" t="n">
-        <v>883285.5600000001</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="79" t="inlineStr">
-        <is>
-          <t>Atribuible a hijos no emancipados</t>
-        </is>
-      </c>
-      <c r="B24" s="61" t="n">
+          <t>Patrimonio individual del declarante</t>
+        </is>
+      </c>
+      <c r="B20" s="62" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="79" t="inlineStr">
+        <is>
+          <t>Patrimonio del anio anterior</t>
+        </is>
+      </c>
+      <c r="B21" s="62" t="n">
+        <v>801569.97</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="79" t="inlineStr">
+        <is>
+          <t>Crecimiento / decremento patrimonial</t>
+        </is>
+      </c>
+      <c r="B22" s="61" t="n">
+        <v>81715.59</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="78" t="inlineStr">
+        <is>
+          <t>PATRIMONIO NETO  (calculado - enlazado al Dashboard)</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
         <is>
-          <t>Patrimonio en la sociedad conyugal</t>
-        </is>
-      </c>
-      <c r="B25" s="61" t="n">
-        <v>883285.5600000001</v>
+          <t>Patrimonio neto 2025</t>
+        </is>
+      </c>
+      <c r="B25" s="61">
+        <f>Dashboard!D31</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
         <is>
-          <t>Patrimonio individual del declarante</t>
-        </is>
-      </c>
-      <c r="B26" s="61" t="n">
-        <v>0</v>
+          <t>Patrimonio neto 2026 (proyectado)</t>
+        </is>
+      </c>
+      <c r="B26" s="61">
+        <f>Dashboard!E31</f>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="79" t="inlineStr">
         <is>
-          <t>Patrimonio del anio anterior</t>
-        </is>
-      </c>
-      <c r="B27" s="61" t="n">
-        <v>801569.97</v>
+          <t>Variacion proyectada</t>
+        </is>
+      </c>
+      <c r="B27" s="61">
+        <f>Dashboard!F31</f>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="79" t="inlineStr">
         <is>
-          <t>Crecimiento / decremento patrimonial</t>
-        </is>
-      </c>
-      <c r="B28" s="61" t="n">
-        <v>81715.59</v>
+          <t>Variacion % proyectada</t>
+        </is>
+      </c>
+      <c r="B28" s="63">
+        <f>Dashboard!G31</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -2607,18 +2612,33 @@
     <row r="34">
       <c r="A34" s="59" t="inlineStr">
         <is>
-          <t>Catalogos del SRI integrados (Tablas 1-19 del archivo CATALOGO.xls). El XML se genera con generar_xml_sri.py.</t>
+          <t>Las celdas amarillas son editables; los totales de creditos y derechos se calculan automaticamente al generar el XML.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A22:B22"/>
   </mergeCells>
+  <dataValidations count="4">
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"IND - Individual,SCD - Sociedad,SOC - Sociedad conyugal o union de hecho"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"C - Cedula,E - Identificacion del exterior,P - Pasaporte,R - RUC"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"C - Cedula,E - Identificacion del exterior,P - Pasaporte,R - RUC"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 - Si,2 - No"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(tools): formato texto para numeros largos en columnas de identificacion
Las celdas de columnas de texto (claveCat, numIdent, placa, etc.) se
guardan con formato de texto ('@') para evitar que Excel las convierta
a notacion cientifica. El generador de XML (Python y VBA) ademas
formatea los numeros largos como entero plano antes de escribirlos.

https://claude.ai/code/session_01Vyh8FwP5vMboaeHUXVLaDC
</commit_message>
<xml_diff>
--- a/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
+++ b/tools/Declaracion_Patrimonial_2025_MARCO.xlsx
@@ -223,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -385,6 +385,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -395,6 +398,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1874,7 +1880,7 @@
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
+      <c r="D6" s="61" t="inlineStr">
         <is>
           <t>DINERS CLUB DEL ECUADOR</t>
         </is>
@@ -1884,97 +1890,97 @@
           <t>R - RUC</t>
         </is>
       </c>
-      <c r="F6" s="60" t="inlineStr">
+      <c r="F6" s="61" t="inlineStr">
         <is>
           <t>1792260957001</t>
         </is>
       </c>
-      <c r="G6" s="60" t="inlineStr"/>
+      <c r="G6" s="61" t="inlineStr"/>
       <c r="H6" s="60" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="I6" s="61" t="n">
+      <c r="I6" s="62" t="n">
         <v>4891.88</v>
       </c>
-      <c r="J6" s="62" t="n">
+      <c r="J6" s="63" t="n">
         <v>4891.88</v>
       </c>
-      <c r="K6" s="61">
+      <c r="K6" s="62">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="63">
+      <c r="L6" s="64">
         <f>IF(I6=0,"",(J6-I6)/I6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr">
+      <c r="A7" s="65" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B7" s="64" t="inlineStr">
+      <c r="B7" s="65" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C7" s="64" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D7" s="64" t="inlineStr">
+      <c r="D7" s="66" t="inlineStr">
         <is>
           <t>BANCO DEL PICHINCHA</t>
         </is>
       </c>
-      <c r="E7" s="64" t="inlineStr">
+      <c r="E7" s="65" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
-      <c r="F7" s="64" t="inlineStr">
+      <c r="F7" s="66" t="inlineStr">
         <is>
           <t>1790010937001</t>
         </is>
       </c>
-      <c r="G7" s="64" t="inlineStr"/>
-      <c r="H7" s="64" t="inlineStr">
+      <c r="G7" s="66" t="inlineStr"/>
+      <c r="H7" s="65" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="I7" s="65" t="n">
+      <c r="I7" s="67" t="n">
         <v>5547.31</v>
       </c>
-      <c r="J7" s="62" t="n">
+      <c r="J7" s="63" t="n">
         <v>5547.31</v>
       </c>
-      <c r="K7" s="65">
+      <c r="K7" s="67">
         <f>J7-I7</f>
         <v/>
       </c>
-      <c r="L7" s="66">
+      <c r="L7" s="68">
         <f>IF(I7=0,"",(J7-I7)/I7)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="68" t="inlineStr">
+      <c r="A8" s="70" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="68" t="n"/>
-      <c r="C8" s="68" t="n"/>
-      <c r="D8" s="68" t="n"/>
-      <c r="E8" s="68" t="n"/>
-      <c r="F8" s="68" t="n"/>
-      <c r="G8" s="68" t="n"/>
-      <c r="H8" s="68" t="n"/>
+      <c r="B8" s="70" t="n"/>
+      <c r="C8" s="70" t="n"/>
+      <c r="D8" s="70" t="n"/>
+      <c r="E8" s="70" t="n"/>
+      <c r="F8" s="70" t="n"/>
+      <c r="G8" s="70" t="n"/>
+      <c r="H8" s="70" t="n"/>
       <c r="I8" s="38">
         <f>SUM(I6:I7)</f>
         <v/>
@@ -2053,14 +2059,14 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="69" t="inlineStr">
+      <c r="B5" s="71" t="inlineStr">
         <is>
           <t>Incremento patrimonial declarado en el XML</t>
         </is>
       </c>
-      <c r="C5" s="70" t="n"/>
-      <c r="D5" s="70" t="n"/>
-      <c r="E5" s="71" t="n">
+      <c r="C5" s="72" t="n"/>
+      <c r="D5" s="72" t="n"/>
+      <c r="E5" s="73" t="n">
         <v>81715.59</v>
       </c>
     </row>
@@ -2077,84 +2083,84 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="72" t="inlineStr">
+      <c r="B8" s="74" t="inlineStr">
         <is>
           <t>1 - Ingresos locales</t>
         </is>
       </c>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="73" t="inlineStr">
+      <c r="E8" s="75" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="72" t="inlineStr">
+      <c r="B9" s="74" t="inlineStr">
         <is>
           <t>2 - Ingresos exterior</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
-      <c r="E9" s="73" t="inlineStr">
+      <c r="E9" s="75" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="72" t="inlineStr">
+      <c r="B10" s="74" t="inlineStr">
         <is>
           <t>3 - Herencias, legados o donaciones</t>
         </is>
       </c>
       <c r="C10" s="6" t="n"/>
       <c r="D10" s="6" t="n"/>
-      <c r="E10" s="73" t="inlineStr">
+      <c r="E10" s="75" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="72" t="inlineStr">
+      <c r="B11" s="74" t="inlineStr">
         <is>
           <t>4 - Loterias o rifas</t>
         </is>
       </c>
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
-      <c r="E11" s="73" t="inlineStr">
+      <c r="E11" s="75" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="72" t="inlineStr">
+      <c r="B12" s="74" t="inlineStr">
         <is>
           <t>5 - Ganancias de capital</t>
         </is>
       </c>
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="6" t="n"/>
-      <c r="E12" s="73" t="inlineStr">
+      <c r="E12" s="75" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="72" t="inlineStr">
+      <c r="B13" s="74" t="inlineStr">
         <is>
           <t>6 - Otros</t>
         </is>
       </c>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
-      <c r="E13" s="73" t="inlineStr">
+      <c r="E13" s="75" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
@@ -2224,7 +2230,7 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="74" t="inlineStr">
+      <c r="B5" s="76" t="inlineStr">
         <is>
           <t>►   GENERAR XML</t>
         </is>
@@ -2238,83 +2244,83 @@
       <c r="D6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="75" t="inlineStr">
+      <c r="B7" s="77" t="inlineStr">
         <is>
           <t>En el archivo .xlsm el boton verde ya esta vinculado a la macro GenerarXmlSRI.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="76" t="inlineStr">
+      <c r="B9" s="78" t="inlineStr">
         <is>
           <t>COMO USAR ESTE ARCHIVO</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="77" t="inlineStr">
+      <c r="B10" s="79" t="inlineStr">
         <is>
           <t>1. Al abrir el archivo .xlsm, pulse 'Habilitar contenido' en la barra de seguridad de Excel.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="77" t="inlineStr">
+      <c r="B11" s="79" t="inlineStr">
         <is>
           <t>2. Llene las columnas amarillas de cada modulo (Dinero, Vehiculos, etc.) y la hoja Justificacion.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="77" t="inlineStr">
+      <c r="B12" s="79" t="inlineStr">
         <is>
           <t>3. Pulse el boton verde GENERAR XML, indique el anio y elija donde guardar el archivo.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="77" t="inlineStr">
+      <c r="B13" s="79" t="inlineStr">
         <is>
           <t>4. El archivo .xml queda listo para subir al portal del SRI.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="77" t="inlineStr"/>
+      <c r="B14" s="79" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="76" t="inlineStr">
+      <c r="B15" s="78" t="inlineStr">
         <is>
           <t>SI EXCEL BLOQUEA LAS MACROS</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="77" t="inlineStr">
+      <c r="B16" s="79" t="inlineStr">
         <is>
           <t>- Cierre Excel. En el Explorador, clic derecho sobre el archivo &gt; Propiedades.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="77" t="inlineStr">
+      <c r="B17" s="79" t="inlineStr">
         <is>
           <t>- Al final de la pestana General marque 'Desbloquear' y pulse Aceptar.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="77" t="inlineStr">
+      <c r="B18" s="79" t="inlineStr">
         <is>
           <t>- Vuelva a abrirlo y pulse 'Habilitar contenido'. Conserve siempre la extension .xlsm.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="77" t="inlineStr"/>
+      <c r="B19" s="79" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="B20" s="77" t="inlineStr">
+      <c r="B20" s="79" t="inlineStr">
         <is>
           <t>Alternativa sin macros:  ejecutar  python tools/generar_xml_sri.py  desde la terminal.</t>
         </is>
@@ -2362,248 +2368,248 @@
       <c r="A3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="78" t="inlineStr">
+      <c r="A5" s="80" t="inlineStr">
         <is>
           <t>IDENTIFICACION DEL DECLARANTE Y CONYUGE  (editable)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="79" t="inlineStr">
+      <c r="A6" s="81" t="inlineStr">
         <is>
           <t>Anio de la declaracion</t>
         </is>
       </c>
-      <c r="B6" s="80" t="n">
+      <c r="B6" s="82" t="n">
         <v>2025</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="79" t="inlineStr">
+      <c r="A7" s="81" t="inlineStr">
         <is>
           <t>Tipo de declaracion</t>
         </is>
       </c>
-      <c r="B7" s="80" t="inlineStr">
+      <c r="B7" s="82" t="inlineStr">
         <is>
           <t>SOC - Sociedad conyugal o union de hecho</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="79" t="inlineStr">
+      <c r="A8" s="81" t="inlineStr">
         <is>
           <t>Tipo de identificacion</t>
         </is>
       </c>
-      <c r="B8" s="80" t="inlineStr">
+      <c r="B8" s="82" t="inlineStr">
         <is>
           <t>R - RUC</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="79" t="inlineStr">
+      <c r="A9" s="81" t="inlineStr">
         <is>
           <t>Numero de identificacion</t>
         </is>
       </c>
-      <c r="B9" s="80" t="inlineStr">
+      <c r="B9" s="82" t="inlineStr">
         <is>
           <t>1709164899001</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="79" t="inlineStr">
+      <c r="A10" s="81" t="inlineStr">
         <is>
           <t>Nombre del declarante</t>
         </is>
       </c>
-      <c r="B10" s="80" t="inlineStr">
+      <c r="B10" s="82" t="inlineStr">
         <is>
           <t>GONZALEZ NAVAS MARCO VINICIO</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="79" t="inlineStr">
+      <c r="A11" s="81" t="inlineStr">
         <is>
           <t>Identificacion del conyuge</t>
         </is>
       </c>
-      <c r="B11" s="80" t="inlineStr">
+      <c r="B11" s="82" t="inlineStr">
         <is>
           <t>C - Cedula</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="79" t="inlineStr">
+      <c r="A12" s="81" t="inlineStr">
         <is>
           <t>Numero ident. conyuge</t>
         </is>
       </c>
-      <c r="B12" s="80" t="inlineStr">
+      <c r="B12" s="82" t="inlineStr">
         <is>
           <t>1709784225</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="79" t="inlineStr">
+      <c r="A13" s="81" t="inlineStr">
         <is>
           <t>Nombre del conyuge</t>
         </is>
       </c>
-      <c r="B13" s="80" t="inlineStr">
+      <c r="B13" s="82" t="inlineStr">
         <is>
           <t>HIDALGO LOZA ROSA CONSUELO</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="79" t="inlineStr">
+      <c r="A14" s="81" t="inlineStr">
         <is>
           <t>Regularizacion de activos</t>
         </is>
       </c>
-      <c r="B14" s="80" t="inlineStr"/>
+      <c r="B14" s="82" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="78" t="inlineStr">
+      <c r="A16" s="80" t="inlineStr">
         <is>
           <t>PATRIMONIO DECLARADO  (editable)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="79" t="inlineStr">
+      <c r="A17" s="81" t="inlineStr">
         <is>
           <t>Patrimonio total declarado</t>
         </is>
       </c>
-      <c r="B17" s="61" t="n">
+      <c r="B17" s="62" t="n">
         <v>883285.5600000001</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="79" t="inlineStr">
+      <c r="A18" s="81" t="inlineStr">
         <is>
           <t>Atribuible a hijos no emancipados</t>
         </is>
       </c>
-      <c r="B18" s="62" t="n">
+      <c r="B18" s="63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="79" t="inlineStr">
+      <c r="A19" s="81" t="inlineStr">
         <is>
           <t>Patrimonio en la sociedad conyugal</t>
         </is>
       </c>
-      <c r="B19" s="62" t="n">
+      <c r="B19" s="63" t="n">
         <v>883285.5600000001</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="79" t="inlineStr">
+      <c r="A20" s="81" t="inlineStr">
         <is>
           <t>Patrimonio individual del declarante</t>
         </is>
       </c>
-      <c r="B20" s="62" t="n">
+      <c r="B20" s="63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="79" t="inlineStr">
+      <c r="A21" s="81" t="inlineStr">
         <is>
           <t>Patrimonio del anio anterior</t>
         </is>
       </c>
-      <c r="B21" s="62" t="n">
+      <c r="B21" s="63" t="n">
         <v>801569.97</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="79" t="inlineStr">
+      <c r="A22" s="81" t="inlineStr">
         <is>
           <t>Crecimiento / decremento patrimonial</t>
         </is>
       </c>
-      <c r="B22" s="61" t="n">
+      <c r="B22" s="62" t="n">
         <v>81715.59</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="78" t="inlineStr">
+      <c r="A24" s="80" t="inlineStr">
         <is>
           <t>PATRIMONIO NETO  (calculado - enlazado al Dashboard)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="79" t="inlineStr">
+      <c r="A25" s="81" t="inlineStr">
         <is>
           <t>Patrimonio neto 2025</t>
         </is>
       </c>
-      <c r="B25" s="61">
+      <c r="B25" s="62">
         <f>Dashboard!D31</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="79" t="inlineStr">
+      <c r="A26" s="81" t="inlineStr">
         <is>
           <t>Patrimonio neto 2026 (proyectado)</t>
         </is>
       </c>
-      <c r="B26" s="61">
+      <c r="B26" s="62">
         <f>Dashboard!E31</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="79" t="inlineStr">
+      <c r="A27" s="81" t="inlineStr">
         <is>
           <t>Variacion proyectada</t>
         </is>
       </c>
-      <c r="B27" s="61">
+      <c r="B27" s="62">
         <f>Dashboard!F31</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="79" t="inlineStr">
+      <c r="A28" s="81" t="inlineStr">
         <is>
           <t>Variacion % proyectada</t>
         </is>
       </c>
-      <c r="B28" s="63">
+      <c r="B28" s="64">
         <f>Dashboard!G31</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="76" t="inlineStr">
+      <c r="A30" s="78" t="inlineStr">
         <is>
           <t>Justificacion de la variacion (ver hoja Justificacion)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="77" t="inlineStr">
+      <c r="A31" s="79" t="inlineStr">
         <is>
           <t>- 1 - Ingresos locales</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="77" t="inlineStr">
+      <c r="A32" s="79" t="inlineStr">
         <is>
           <t>- 6 - Otros</t>
         </is>
@@ -5896,97 +5902,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="81" t="inlineStr">
+      <c r="A1" s="83" t="inlineStr">
         <is>
           <t>DINERO_EN</t>
         </is>
       </c>
-      <c r="B1" s="81" t="inlineStr">
+      <c r="B1" s="83" t="inlineStr">
         <is>
           <t>TIPO_INVERSION</t>
         </is>
       </c>
-      <c r="C1" s="81" t="inlineStr">
+      <c r="C1" s="83" t="inlineStr">
         <is>
           <t>UBICACION</t>
         </is>
       </c>
-      <c r="D1" s="81" t="inlineStr">
+      <c r="D1" s="83" t="inlineStr">
         <is>
           <t>PAIS</t>
         </is>
       </c>
-      <c r="E1" s="81" t="inlineStr">
+      <c r="E1" s="83" t="inlineStr">
         <is>
           <t>INSTITUCION_FINANCIERA</t>
         </is>
       </c>
-      <c r="F1" s="81" t="inlineStr">
+      <c r="F1" s="83" t="inlineStr">
         <is>
           <t>PARTES_RELACIONADAS</t>
         </is>
       </c>
-      <c r="G1" s="81" t="inlineStr">
+      <c r="G1" s="83" t="inlineStr">
         <is>
           <t>TIPO_DRC</t>
         </is>
       </c>
-      <c r="H1" s="81" t="inlineStr">
+      <c r="H1" s="83" t="inlineStr">
         <is>
           <t>TIPO_PERSONA</t>
         </is>
       </c>
-      <c r="I1" s="81" t="inlineStr">
+      <c r="I1" s="83" t="inlineStr">
         <is>
           <t>TIPO_BIEN_MUEBLE</t>
         </is>
       </c>
-      <c r="J1" s="81" t="inlineStr">
+      <c r="J1" s="83" t="inlineStr">
         <is>
           <t>TIPO_VEHICULO</t>
         </is>
       </c>
-      <c r="K1" s="81" t="inlineStr">
+      <c r="K1" s="83" t="inlineStr">
         <is>
           <t>TIPO_DERECHO</t>
         </is>
       </c>
-      <c r="L1" s="81" t="inlineStr">
+      <c r="L1" s="83" t="inlineStr">
         <is>
           <t>TIPO_INMUEBLE</t>
         </is>
       </c>
-      <c r="M1" s="81" t="inlineStr">
+      <c r="M1" s="83" t="inlineStr">
         <is>
           <t>PROVINCIA</t>
         </is>
       </c>
-      <c r="N1" s="81" t="inlineStr">
+      <c r="N1" s="83" t="inlineStr">
         <is>
           <t>CANTON</t>
         </is>
       </c>
-      <c r="O1" s="81" t="inlineStr">
+      <c r="O1" s="83" t="inlineStr">
         <is>
           <t>TIPO_ACREEDOR</t>
         </is>
       </c>
-      <c r="P1" s="81" t="inlineStr">
+      <c r="P1" s="83" t="inlineStr">
         <is>
           <t>TIPO_IDENTIFICACION</t>
         </is>
       </c>
-      <c r="Q1" s="81" t="inlineStr">
+      <c r="Q1" s="83" t="inlineStr">
         <is>
           <t>REGULARIZACION</t>
         </is>
       </c>
-      <c r="R1" s="81" t="inlineStr">
+      <c r="R1" s="83" t="inlineStr">
         <is>
           <t>JUSTIF_INCREMENTO</t>
         </is>
       </c>
-      <c r="S1" s="81" t="inlineStr">
+      <c r="S1" s="83" t="inlineStr">
         <is>
           <t>JUSTIF_DECREMENTO</t>
         </is>
@@ -12612,7 +12618,7 @@
           <t>1029 - BANCO PICHINCHA C.A.</t>
         </is>
       </c>
-      <c r="F6" s="60" t="inlineStr">
+      <c r="F6" s="61" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
@@ -12623,71 +12629,71 @@
         </is>
       </c>
       <c r="H6" s="60" t="inlineStr"/>
-      <c r="I6" s="60" t="inlineStr"/>
-      <c r="J6" s="61" t="n">
+      <c r="I6" s="61" t="inlineStr"/>
+      <c r="J6" s="62" t="n">
         <v>130.2</v>
       </c>
-      <c r="K6" s="62" t="n">
+      <c r="K6" s="63" t="n">
         <v>130.2</v>
       </c>
-      <c r="L6" s="61">
+      <c r="L6" s="62">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="63">
+      <c r="M6" s="64">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr">
+      <c r="A7" s="65" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B7" s="64" t="inlineStr">
+      <c r="B7" s="65" t="inlineStr">
         <is>
           <t>4 - Cuenta corriente</t>
         </is>
       </c>
-      <c r="C7" s="64" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D7" s="64" t="inlineStr">
+      <c r="D7" s="65" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E7" s="64" t="inlineStr">
+      <c r="E7" s="65" t="inlineStr">
         <is>
           <t>1029 - BANCO PICHINCHA C.A.</t>
         </is>
       </c>
-      <c r="F7" s="64" t="inlineStr">
+      <c r="F7" s="66" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G7" s="64" t="inlineStr">
+      <c r="G7" s="65" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H7" s="64" t="inlineStr"/>
-      <c r="I7" s="64" t="inlineStr"/>
-      <c r="J7" s="65" t="n">
+      <c r="H7" s="65" t="inlineStr"/>
+      <c r="I7" s="66" t="inlineStr"/>
+      <c r="J7" s="67" t="n">
         <v>5590.32</v>
       </c>
-      <c r="K7" s="62" t="n">
+      <c r="K7" s="63" t="n">
         <v>5590.32</v>
       </c>
-      <c r="L7" s="65">
+      <c r="L7" s="67">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="66">
+      <c r="M7" s="68">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
@@ -12718,7 +12724,7 @@
           <t>1418 - BANCO PROMERICA S.A.</t>
         </is>
       </c>
-      <c r="F8" s="60" t="inlineStr">
+      <c r="F8" s="61" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
@@ -12729,89 +12735,89 @@
         </is>
       </c>
       <c r="H8" s="60" t="inlineStr"/>
-      <c r="I8" s="60" t="inlineStr"/>
-      <c r="J8" s="61" t="n">
+      <c r="I8" s="61" t="inlineStr"/>
+      <c r="J8" s="62" t="n">
         <v>53237.31</v>
       </c>
-      <c r="K8" s="62" t="n">
+      <c r="K8" s="63" t="n">
         <v>53237.31</v>
       </c>
-      <c r="L8" s="61">
+      <c r="L8" s="62">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="63">
+      <c r="M8" s="64">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="64" t="inlineStr">
+      <c r="A9" s="65" t="inlineStr">
         <is>
           <t>IFI - Instituciones financieras</t>
         </is>
       </c>
-      <c r="B9" s="64" t="inlineStr">
+      <c r="B9" s="65" t="inlineStr">
         <is>
           <t>2 - Inversiones financieras</t>
         </is>
       </c>
-      <c r="C9" s="64" t="inlineStr">
+      <c r="C9" s="65" t="inlineStr">
         <is>
           <t>EXT - En el exterior</t>
         </is>
       </c>
-      <c r="D9" s="64" t="inlineStr">
+      <c r="D9" s="65" t="inlineStr">
         <is>
           <t>118 - PANAMA</t>
         </is>
       </c>
-      <c r="E9" s="64" t="inlineStr">
+      <c r="E9" s="65" t="inlineStr">
         <is>
           <t>BANCO PICHINCHA CA</t>
         </is>
       </c>
-      <c r="F9" s="64" t="inlineStr">
+      <c r="F9" s="66" t="inlineStr">
         <is>
           <t>DOLARES</t>
         </is>
       </c>
-      <c r="G9" s="64" t="inlineStr">
+      <c r="G9" s="65" t="inlineStr">
         <is>
           <t>2 - No</t>
         </is>
       </c>
-      <c r="H9" s="64" t="inlineStr"/>
-      <c r="I9" s="64" t="inlineStr"/>
-      <c r="J9" s="65" t="n">
+      <c r="H9" s="65" t="inlineStr"/>
+      <c r="I9" s="66" t="inlineStr"/>
+      <c r="J9" s="67" t="n">
         <v>189049.31</v>
       </c>
-      <c r="K9" s="62" t="n">
+      <c r="K9" s="63" t="n">
         <v>189049.31</v>
       </c>
-      <c r="L9" s="65">
+      <c r="L9" s="67">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="66">
+      <c r="M9" s="68">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="67" t="inlineStr">
+      <c r="A10" s="69" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B10" s="67" t="n"/>
-      <c r="C10" s="67" t="n"/>
-      <c r="D10" s="67" t="n"/>
-      <c r="E10" s="67" t="n"/>
-      <c r="F10" s="67" t="n"/>
-      <c r="G10" s="67" t="n"/>
-      <c r="H10" s="67" t="n"/>
-      <c r="I10" s="67" t="n"/>
+      <c r="B10" s="69" t="n"/>
+      <c r="C10" s="69" t="n"/>
+      <c r="D10" s="69" t="n"/>
+      <c r="E10" s="69" t="n"/>
+      <c r="F10" s="69" t="n"/>
+      <c r="G10" s="69" t="n"/>
+      <c r="H10" s="69" t="n"/>
+      <c r="I10" s="69" t="n"/>
       <c r="J10" s="31">
         <f>SUM(J6:J9)</f>
         <v/>
@@ -12974,48 +12980,48 @@
       <c r="A6" s="60" t="inlineStr"/>
       <c r="B6" s="60" t="inlineStr"/>
       <c r="C6" s="60" t="inlineStr"/>
-      <c r="D6" s="60" t="inlineStr"/>
-      <c r="E6" s="60" t="inlineStr"/>
-      <c r="F6" s="60" t="inlineStr"/>
+      <c r="D6" s="61" t="inlineStr"/>
+      <c r="E6" s="61" t="inlineStr"/>
+      <c r="F6" s="61" t="inlineStr"/>
       <c r="G6" s="60" t="inlineStr"/>
       <c r="H6" s="60" t="inlineStr"/>
-      <c r="I6" s="60" t="inlineStr"/>
-      <c r="J6" s="62" t="n">
+      <c r="I6" s="61" t="inlineStr"/>
+      <c r="J6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="62" t="n">
+      <c r="K6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="61">
+      <c r="L6" s="62">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="63">
+      <c r="M6" s="64">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr"/>
-      <c r="B7" s="64" t="inlineStr"/>
-      <c r="C7" s="64" t="inlineStr"/>
-      <c r="D7" s="64" t="inlineStr"/>
-      <c r="E7" s="64" t="inlineStr"/>
-      <c r="F7" s="64" t="inlineStr"/>
-      <c r="G7" s="64" t="inlineStr"/>
-      <c r="H7" s="64" t="inlineStr"/>
-      <c r="I7" s="64" t="inlineStr"/>
-      <c r="J7" s="62" t="n">
+      <c r="A7" s="65" t="inlineStr"/>
+      <c r="B7" s="65" t="inlineStr"/>
+      <c r="C7" s="65" t="inlineStr"/>
+      <c r="D7" s="66" t="inlineStr"/>
+      <c r="E7" s="66" t="inlineStr"/>
+      <c r="F7" s="66" t="inlineStr"/>
+      <c r="G7" s="65" t="inlineStr"/>
+      <c r="H7" s="65" t="inlineStr"/>
+      <c r="I7" s="66" t="inlineStr"/>
+      <c r="J7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="62" t="n">
+      <c r="K7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="65">
+      <c r="L7" s="67">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="66">
+      <c r="M7" s="68">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
@@ -13024,48 +13030,48 @@
       <c r="A8" s="60" t="inlineStr"/>
       <c r="B8" s="60" t="inlineStr"/>
       <c r="C8" s="60" t="inlineStr"/>
-      <c r="D8" s="60" t="inlineStr"/>
-      <c r="E8" s="60" t="inlineStr"/>
-      <c r="F8" s="60" t="inlineStr"/>
+      <c r="D8" s="61" t="inlineStr"/>
+      <c r="E8" s="61" t="inlineStr"/>
+      <c r="F8" s="61" t="inlineStr"/>
       <c r="G8" s="60" t="inlineStr"/>
       <c r="H8" s="60" t="inlineStr"/>
-      <c r="I8" s="60" t="inlineStr"/>
-      <c r="J8" s="62" t="n">
+      <c r="I8" s="61" t="inlineStr"/>
+      <c r="J8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="62" t="n">
+      <c r="K8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="61">
+      <c r="L8" s="62">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="63">
+      <c r="M8" s="64">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="64" t="inlineStr"/>
-      <c r="B9" s="64" t="inlineStr"/>
-      <c r="C9" s="64" t="inlineStr"/>
-      <c r="D9" s="64" t="inlineStr"/>
-      <c r="E9" s="64" t="inlineStr"/>
-      <c r="F9" s="64" t="inlineStr"/>
-      <c r="G9" s="64" t="inlineStr"/>
-      <c r="H9" s="64" t="inlineStr"/>
-      <c r="I9" s="64" t="inlineStr"/>
-      <c r="J9" s="62" t="n">
+      <c r="A9" s="65" t="inlineStr"/>
+      <c r="B9" s="65" t="inlineStr"/>
+      <c r="C9" s="65" t="inlineStr"/>
+      <c r="D9" s="66" t="inlineStr"/>
+      <c r="E9" s="66" t="inlineStr"/>
+      <c r="F9" s="66" t="inlineStr"/>
+      <c r="G9" s="65" t="inlineStr"/>
+      <c r="H9" s="65" t="inlineStr"/>
+      <c r="I9" s="66" t="inlineStr"/>
+      <c r="J9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="62" t="n">
+      <c r="K9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="65">
+      <c r="L9" s="67">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="66">
+      <c r="M9" s="68">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
@@ -13074,48 +13080,48 @@
       <c r="A10" s="60" t="inlineStr"/>
       <c r="B10" s="60" t="inlineStr"/>
       <c r="C10" s="60" t="inlineStr"/>
-      <c r="D10" s="60" t="inlineStr"/>
-      <c r="E10" s="60" t="inlineStr"/>
-      <c r="F10" s="60" t="inlineStr"/>
+      <c r="D10" s="61" t="inlineStr"/>
+      <c r="E10" s="61" t="inlineStr"/>
+      <c r="F10" s="61" t="inlineStr"/>
       <c r="G10" s="60" t="inlineStr"/>
       <c r="H10" s="60" t="inlineStr"/>
-      <c r="I10" s="60" t="inlineStr"/>
-      <c r="J10" s="62" t="n">
+      <c r="I10" s="61" t="inlineStr"/>
+      <c r="J10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="62" t="n">
+      <c r="K10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="61">
+      <c r="L10" s="62">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="63">
+      <c r="M10" s="64">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="64" t="inlineStr"/>
-      <c r="B11" s="64" t="inlineStr"/>
-      <c r="C11" s="64" t="inlineStr"/>
-      <c r="D11" s="64" t="inlineStr"/>
-      <c r="E11" s="64" t="inlineStr"/>
-      <c r="F11" s="64" t="inlineStr"/>
-      <c r="G11" s="64" t="inlineStr"/>
-      <c r="H11" s="64" t="inlineStr"/>
-      <c r="I11" s="64" t="inlineStr"/>
-      <c r="J11" s="62" t="n">
+      <c r="A11" s="65" t="inlineStr"/>
+      <c r="B11" s="65" t="inlineStr"/>
+      <c r="C11" s="65" t="inlineStr"/>
+      <c r="D11" s="66" t="inlineStr"/>
+      <c r="E11" s="66" t="inlineStr"/>
+      <c r="F11" s="66" t="inlineStr"/>
+      <c r="G11" s="65" t="inlineStr"/>
+      <c r="H11" s="65" t="inlineStr"/>
+      <c r="I11" s="66" t="inlineStr"/>
+      <c r="J11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="62" t="n">
+      <c r="K11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="65">
+      <c r="L11" s="67">
         <f>K11-J11</f>
         <v/>
       </c>
-      <c r="M11" s="66">
+      <c r="M11" s="68">
         <f>IF(J11=0,"",(K11-J11)/J11)</f>
         <v/>
       </c>
@@ -13124,66 +13130,66 @@
       <c r="A12" s="60" t="inlineStr"/>
       <c r="B12" s="60" t="inlineStr"/>
       <c r="C12" s="60" t="inlineStr"/>
-      <c r="D12" s="60" t="inlineStr"/>
-      <c r="E12" s="60" t="inlineStr"/>
-      <c r="F12" s="60" t="inlineStr"/>
+      <c r="D12" s="61" t="inlineStr"/>
+      <c r="E12" s="61" t="inlineStr"/>
+      <c r="F12" s="61" t="inlineStr"/>
       <c r="G12" s="60" t="inlineStr"/>
       <c r="H12" s="60" t="inlineStr"/>
-      <c r="I12" s="60" t="inlineStr"/>
-      <c r="J12" s="62" t="n">
+      <c r="I12" s="61" t="inlineStr"/>
+      <c r="J12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="62" t="n">
+      <c r="K12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="61">
+      <c r="L12" s="62">
         <f>K12-J12</f>
         <v/>
       </c>
-      <c r="M12" s="63">
+      <c r="M12" s="64">
         <f>IF(J12=0,"",(K12-J12)/J12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="64" t="inlineStr"/>
-      <c r="B13" s="64" t="inlineStr"/>
-      <c r="C13" s="64" t="inlineStr"/>
-      <c r="D13" s="64" t="inlineStr"/>
-      <c r="E13" s="64" t="inlineStr"/>
-      <c r="F13" s="64" t="inlineStr"/>
-      <c r="G13" s="64" t="inlineStr"/>
-      <c r="H13" s="64" t="inlineStr"/>
-      <c r="I13" s="64" t="inlineStr"/>
-      <c r="J13" s="62" t="n">
+      <c r="A13" s="65" t="inlineStr"/>
+      <c r="B13" s="65" t="inlineStr"/>
+      <c r="C13" s="65" t="inlineStr"/>
+      <c r="D13" s="66" t="inlineStr"/>
+      <c r="E13" s="66" t="inlineStr"/>
+      <c r="F13" s="66" t="inlineStr"/>
+      <c r="G13" s="65" t="inlineStr"/>
+      <c r="H13" s="65" t="inlineStr"/>
+      <c r="I13" s="66" t="inlineStr"/>
+      <c r="J13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="62" t="n">
+      <c r="K13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="65">
+      <c r="L13" s="67">
         <f>K13-J13</f>
         <v/>
       </c>
-      <c r="M13" s="66">
+      <c r="M13" s="68">
         <f>IF(J13=0,"",(K13-J13)/J13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="67" t="inlineStr">
+      <c r="A14" s="69" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="67" t="n"/>
-      <c r="C14" s="67" t="n"/>
-      <c r="D14" s="67" t="n"/>
-      <c r="E14" s="67" t="n"/>
-      <c r="F14" s="67" t="n"/>
-      <c r="G14" s="67" t="n"/>
-      <c r="H14" s="67" t="n"/>
-      <c r="I14" s="67" t="n"/>
+      <c r="B14" s="69" t="n"/>
+      <c r="C14" s="69" t="n"/>
+      <c r="D14" s="69" t="n"/>
+      <c r="E14" s="69" t="n"/>
+      <c r="F14" s="69" t="n"/>
+      <c r="G14" s="69" t="n"/>
+      <c r="H14" s="69" t="n"/>
+      <c r="I14" s="69" t="n"/>
       <c r="J14" s="31">
         <f>SUM(J6:J13)</f>
         <v/>
@@ -13337,219 +13343,219 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="60" t="inlineStr"/>
+      <c r="A6" s="61" t="inlineStr"/>
       <c r="B6" s="60" t="inlineStr"/>
       <c r="C6" s="60" t="inlineStr"/>
-      <c r="D6" s="60" t="inlineStr"/>
+      <c r="D6" s="61" t="inlineStr"/>
       <c r="E6" s="60" t="inlineStr"/>
       <c r="F6" s="60" t="inlineStr"/>
       <c r="G6" s="60" t="inlineStr"/>
       <c r="H6" s="60" t="inlineStr"/>
-      <c r="I6" s="60" t="inlineStr"/>
-      <c r="J6" s="62" t="n">
+      <c r="I6" s="61" t="inlineStr"/>
+      <c r="J6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="62" t="n">
+      <c r="K6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="61">
+      <c r="L6" s="62">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="63">
+      <c r="M6" s="64">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr"/>
-      <c r="B7" s="64" t="inlineStr"/>
-      <c r="C7" s="64" t="inlineStr"/>
-      <c r="D7" s="64" t="inlineStr"/>
-      <c r="E7" s="64" t="inlineStr"/>
-      <c r="F7" s="64" t="inlineStr"/>
-      <c r="G7" s="64" t="inlineStr"/>
-      <c r="H7" s="64" t="inlineStr"/>
-      <c r="I7" s="64" t="inlineStr"/>
-      <c r="J7" s="62" t="n">
+      <c r="A7" s="66" t="inlineStr"/>
+      <c r="B7" s="65" t="inlineStr"/>
+      <c r="C7" s="65" t="inlineStr"/>
+      <c r="D7" s="66" t="inlineStr"/>
+      <c r="E7" s="65" t="inlineStr"/>
+      <c r="F7" s="65" t="inlineStr"/>
+      <c r="G7" s="65" t="inlineStr"/>
+      <c r="H7" s="65" t="inlineStr"/>
+      <c r="I7" s="66" t="inlineStr"/>
+      <c r="J7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="62" t="n">
+      <c r="K7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="65">
+      <c r="L7" s="67">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="66">
+      <c r="M7" s="68">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="60" t="inlineStr"/>
+      <c r="A8" s="61" t="inlineStr"/>
       <c r="B8" s="60" t="inlineStr"/>
       <c r="C8" s="60" t="inlineStr"/>
-      <c r="D8" s="60" t="inlineStr"/>
+      <c r="D8" s="61" t="inlineStr"/>
       <c r="E8" s="60" t="inlineStr"/>
       <c r="F8" s="60" t="inlineStr"/>
       <c r="G8" s="60" t="inlineStr"/>
       <c r="H8" s="60" t="inlineStr"/>
-      <c r="I8" s="60" t="inlineStr"/>
-      <c r="J8" s="62" t="n">
+      <c r="I8" s="61" t="inlineStr"/>
+      <c r="J8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="62" t="n">
+      <c r="K8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="61">
+      <c r="L8" s="62">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="63">
+      <c r="M8" s="64">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="64" t="inlineStr"/>
-      <c r="B9" s="64" t="inlineStr"/>
-      <c r="C9" s="64" t="inlineStr"/>
-      <c r="D9" s="64" t="inlineStr"/>
-      <c r="E9" s="64" t="inlineStr"/>
-      <c r="F9" s="64" t="inlineStr"/>
-      <c r="G9" s="64" t="inlineStr"/>
-      <c r="H9" s="64" t="inlineStr"/>
-      <c r="I9" s="64" t="inlineStr"/>
-      <c r="J9" s="62" t="n">
+      <c r="A9" s="66" t="inlineStr"/>
+      <c r="B9" s="65" t="inlineStr"/>
+      <c r="C9" s="65" t="inlineStr"/>
+      <c r="D9" s="66" t="inlineStr"/>
+      <c r="E9" s="65" t="inlineStr"/>
+      <c r="F9" s="65" t="inlineStr"/>
+      <c r="G9" s="65" t="inlineStr"/>
+      <c r="H9" s="65" t="inlineStr"/>
+      <c r="I9" s="66" t="inlineStr"/>
+      <c r="J9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="62" t="n">
+      <c r="K9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="65">
+      <c r="L9" s="67">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="66">
+      <c r="M9" s="68">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="60" t="inlineStr"/>
+      <c r="A10" s="61" t="inlineStr"/>
       <c r="B10" s="60" t="inlineStr"/>
       <c r="C10" s="60" t="inlineStr"/>
-      <c r="D10" s="60" t="inlineStr"/>
+      <c r="D10" s="61" t="inlineStr"/>
       <c r="E10" s="60" t="inlineStr"/>
       <c r="F10" s="60" t="inlineStr"/>
       <c r="G10" s="60" t="inlineStr"/>
       <c r="H10" s="60" t="inlineStr"/>
-      <c r="I10" s="60" t="inlineStr"/>
-      <c r="J10" s="62" t="n">
+      <c r="I10" s="61" t="inlineStr"/>
+      <c r="J10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="62" t="n">
+      <c r="K10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="61">
+      <c r="L10" s="62">
         <f>K10-J10</f>
         <v/>
       </c>
-      <c r="M10" s="63">
+      <c r="M10" s="64">
         <f>IF(J10=0,"",(K10-J10)/J10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="64" t="inlineStr"/>
-      <c r="B11" s="64" t="inlineStr"/>
-      <c r="C11" s="64" t="inlineStr"/>
-      <c r="D11" s="64" t="inlineStr"/>
-      <c r="E11" s="64" t="inlineStr"/>
-      <c r="F11" s="64" t="inlineStr"/>
-      <c r="G11" s="64" t="inlineStr"/>
-      <c r="H11" s="64" t="inlineStr"/>
-      <c r="I11" s="64" t="inlineStr"/>
-      <c r="J11" s="62" t="n">
+      <c r="A11" s="66" t="inlineStr"/>
+      <c r="B11" s="65" t="inlineStr"/>
+      <c r="C11" s="65" t="inlineStr"/>
+      <c r="D11" s="66" t="inlineStr"/>
+      <c r="E11" s="65" t="inlineStr"/>
+      <c r="F11" s="65" t="inlineStr"/>
+      <c r="G11" s="65" t="inlineStr"/>
+      <c r="H11" s="65" t="inlineStr"/>
+      <c r="I11" s="66" t="inlineStr"/>
+      <c r="J11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="62" t="n">
+      <c r="K11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="65">
+      <c r="L11" s="67">
         <f>K11-J11</f>
         <v/>
       </c>
-      <c r="M11" s="66">
+      <c r="M11" s="68">
         <f>IF(J11=0,"",(K11-J11)/J11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="60" t="inlineStr"/>
+      <c r="A12" s="61" t="inlineStr"/>
       <c r="B12" s="60" t="inlineStr"/>
       <c r="C12" s="60" t="inlineStr"/>
-      <c r="D12" s="60" t="inlineStr"/>
+      <c r="D12" s="61" t="inlineStr"/>
       <c r="E12" s="60" t="inlineStr"/>
       <c r="F12" s="60" t="inlineStr"/>
       <c r="G12" s="60" t="inlineStr"/>
       <c r="H12" s="60" t="inlineStr"/>
-      <c r="I12" s="60" t="inlineStr"/>
-      <c r="J12" s="62" t="n">
+      <c r="I12" s="61" t="inlineStr"/>
+      <c r="J12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="62" t="n">
+      <c r="K12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="61">
+      <c r="L12" s="62">
         <f>K12-J12</f>
         <v/>
       </c>
-      <c r="M12" s="63">
+      <c r="M12" s="64">
         <f>IF(J12=0,"",(K12-J12)/J12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="64" t="inlineStr"/>
-      <c r="B13" s="64" t="inlineStr"/>
-      <c r="C13" s="64" t="inlineStr"/>
-      <c r="D13" s="64" t="inlineStr"/>
-      <c r="E13" s="64" t="inlineStr"/>
-      <c r="F13" s="64" t="inlineStr"/>
-      <c r="G13" s="64" t="inlineStr"/>
-      <c r="H13" s="64" t="inlineStr"/>
-      <c r="I13" s="64" t="inlineStr"/>
-      <c r="J13" s="62" t="n">
+      <c r="A13" s="66" t="inlineStr"/>
+      <c r="B13" s="65" t="inlineStr"/>
+      <c r="C13" s="65" t="inlineStr"/>
+      <c r="D13" s="66" t="inlineStr"/>
+      <c r="E13" s="65" t="inlineStr"/>
+      <c r="F13" s="65" t="inlineStr"/>
+      <c r="G13" s="65" t="inlineStr"/>
+      <c r="H13" s="65" t="inlineStr"/>
+      <c r="I13" s="66" t="inlineStr"/>
+      <c r="J13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="62" t="n">
+      <c r="K13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="65">
+      <c r="L13" s="67">
         <f>K13-J13</f>
         <v/>
       </c>
-      <c r="M13" s="66">
+      <c r="M13" s="68">
         <f>IF(J13=0,"",(K13-J13)/J13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="67" t="inlineStr">
+      <c r="A14" s="69" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="67" t="n"/>
-      <c r="C14" s="67" t="n"/>
-      <c r="D14" s="67" t="n"/>
-      <c r="E14" s="67" t="n"/>
-      <c r="F14" s="67" t="n"/>
-      <c r="G14" s="67" t="n"/>
-      <c r="H14" s="67" t="n"/>
-      <c r="I14" s="67" t="n"/>
+      <c r="B14" s="69" t="n"/>
+      <c r="C14" s="69" t="n"/>
+      <c r="D14" s="69" t="n"/>
+      <c r="E14" s="69" t="n"/>
+      <c r="F14" s="69" t="n"/>
+      <c r="G14" s="69" t="n"/>
+      <c r="H14" s="69" t="n"/>
+      <c r="I14" s="69" t="n"/>
       <c r="J14" s="31">
         <f>SUM(J6:J13)</f>
         <v/>
@@ -13686,39 +13692,39 @@
       <c r="B6" s="60" t="inlineStr"/>
       <c r="C6" s="60" t="inlineStr"/>
       <c r="D6" s="60" t="inlineStr"/>
-      <c r="E6" s="60" t="inlineStr"/>
-      <c r="F6" s="62" t="n">
+      <c r="E6" s="61" t="inlineStr"/>
+      <c r="F6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="62" t="n">
+      <c r="G6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="61">
+      <c r="H6" s="62">
         <f>G6-F6</f>
         <v/>
       </c>
-      <c r="I6" s="63">
+      <c r="I6" s="64">
         <f>IF(F6=0,"",(G6-F6)/F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr"/>
-      <c r="B7" s="64" t="inlineStr"/>
-      <c r="C7" s="64" t="inlineStr"/>
-      <c r="D7" s="64" t="inlineStr"/>
-      <c r="E7" s="64" t="inlineStr"/>
-      <c r="F7" s="62" t="n">
+      <c r="A7" s="65" t="inlineStr"/>
+      <c r="B7" s="65" t="inlineStr"/>
+      <c r="C7" s="65" t="inlineStr"/>
+      <c r="D7" s="65" t="inlineStr"/>
+      <c r="E7" s="66" t="inlineStr"/>
+      <c r="F7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="62" t="n">
+      <c r="G7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="65">
+      <c r="H7" s="67">
         <f>G7-F7</f>
         <v/>
       </c>
-      <c r="I7" s="66">
+      <c r="I7" s="68">
         <f>IF(F7=0,"",(G7-F7)/F7)</f>
         <v/>
       </c>
@@ -13728,39 +13734,39 @@
       <c r="B8" s="60" t="inlineStr"/>
       <c r="C8" s="60" t="inlineStr"/>
       <c r="D8" s="60" t="inlineStr"/>
-      <c r="E8" s="60" t="inlineStr"/>
-      <c r="F8" s="62" t="n">
+      <c r="E8" s="61" t="inlineStr"/>
+      <c r="F8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="62" t="n">
+      <c r="G8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="61">
+      <c r="H8" s="62">
         <f>G8-F8</f>
         <v/>
       </c>
-      <c r="I8" s="63">
+      <c r="I8" s="64">
         <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="64" t="inlineStr"/>
-      <c r="B9" s="64" t="inlineStr"/>
-      <c r="C9" s="64" t="inlineStr"/>
-      <c r="D9" s="64" t="inlineStr"/>
-      <c r="E9" s="64" t="inlineStr"/>
-      <c r="F9" s="62" t="n">
+      <c r="A9" s="65" t="inlineStr"/>
+      <c r="B9" s="65" t="inlineStr"/>
+      <c r="C9" s="65" t="inlineStr"/>
+      <c r="D9" s="65" t="inlineStr"/>
+      <c r="E9" s="66" t="inlineStr"/>
+      <c r="F9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="62" t="n">
+      <c r="G9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="65">
+      <c r="H9" s="67">
         <f>G9-F9</f>
         <v/>
       </c>
-      <c r="I9" s="66">
+      <c r="I9" s="68">
         <f>IF(F9=0,"",(G9-F9)/F9)</f>
         <v/>
       </c>
@@ -13770,39 +13776,39 @@
       <c r="B10" s="60" t="inlineStr"/>
       <c r="C10" s="60" t="inlineStr"/>
       <c r="D10" s="60" t="inlineStr"/>
-      <c r="E10" s="60" t="inlineStr"/>
-      <c r="F10" s="62" t="n">
+      <c r="E10" s="61" t="inlineStr"/>
+      <c r="F10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="62" t="n">
+      <c r="G10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="61">
+      <c r="H10" s="62">
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="63">
+      <c r="I10" s="64">
         <f>IF(F10=0,"",(G10-F10)/F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="64" t="inlineStr"/>
-      <c r="B11" s="64" t="inlineStr"/>
-      <c r="C11" s="64" t="inlineStr"/>
-      <c r="D11" s="64" t="inlineStr"/>
-      <c r="E11" s="64" t="inlineStr"/>
-      <c r="F11" s="62" t="n">
+      <c r="A11" s="65" t="inlineStr"/>
+      <c r="B11" s="65" t="inlineStr"/>
+      <c r="C11" s="65" t="inlineStr"/>
+      <c r="D11" s="65" t="inlineStr"/>
+      <c r="E11" s="66" t="inlineStr"/>
+      <c r="F11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="62" t="n">
+      <c r="G11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="65">
+      <c r="H11" s="67">
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="66">
+      <c r="I11" s="68">
         <f>IF(F11=0,"",(G11-F11)/F11)</f>
         <v/>
       </c>
@@ -13812,53 +13818,53 @@
       <c r="B12" s="60" t="inlineStr"/>
       <c r="C12" s="60" t="inlineStr"/>
       <c r="D12" s="60" t="inlineStr"/>
-      <c r="E12" s="60" t="inlineStr"/>
-      <c r="F12" s="62" t="n">
+      <c r="E12" s="61" t="inlineStr"/>
+      <c r="F12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="62" t="n">
+      <c r="G12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="61">
+      <c r="H12" s="62">
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="63">
+      <c r="I12" s="64">
         <f>IF(F12=0,"",(G12-F12)/F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="64" t="inlineStr"/>
-      <c r="B13" s="64" t="inlineStr"/>
-      <c r="C13" s="64" t="inlineStr"/>
-      <c r="D13" s="64" t="inlineStr"/>
-      <c r="E13" s="64" t="inlineStr"/>
-      <c r="F13" s="62" t="n">
+      <c r="A13" s="65" t="inlineStr"/>
+      <c r="B13" s="65" t="inlineStr"/>
+      <c r="C13" s="65" t="inlineStr"/>
+      <c r="D13" s="65" t="inlineStr"/>
+      <c r="E13" s="66" t="inlineStr"/>
+      <c r="F13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="62" t="n">
+      <c r="G13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="65">
+      <c r="H13" s="67">
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="66">
+      <c r="I13" s="68">
         <f>IF(F13=0,"",(G13-F13)/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="67" t="inlineStr">
+      <c r="A14" s="69" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="67" t="n"/>
-      <c r="C14" s="67" t="n"/>
-      <c r="D14" s="67" t="n"/>
-      <c r="E14" s="67" t="n"/>
+      <c r="B14" s="69" t="n"/>
+      <c r="C14" s="69" t="n"/>
+      <c r="D14" s="69" t="n"/>
+      <c r="E14" s="69" t="n"/>
       <c r="F14" s="31">
         <f>SUM(F6:F13)</f>
         <v/>
@@ -13996,7 +14002,7 @@
           <t>1 - Vehiculos motorizados terrestres</t>
         </is>
       </c>
-      <c r="B6" s="60" t="inlineStr">
+      <c r="B6" s="61" t="inlineStr">
         <is>
           <t>PBO7092</t>
         </is>
@@ -14012,56 +14018,56 @@
         </is>
       </c>
       <c r="E6" s="60" t="inlineStr"/>
-      <c r="F6" s="60" t="inlineStr"/>
-      <c r="G6" s="61" t="n">
+      <c r="F6" s="61" t="inlineStr"/>
+      <c r="G6" s="62" t="n">
         <v>12000</v>
       </c>
-      <c r="H6" s="62" t="n">
+      <c r="H6" s="63" t="n">
         <v>12000</v>
       </c>
-      <c r="I6" s="61">
+      <c r="I6" s="62">
         <f>H6-G6</f>
         <v/>
       </c>
-      <c r="J6" s="63">
+      <c r="J6" s="64">
         <f>IF(G6=0,"",(H6-G6)/G6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr">
+      <c r="A7" s="65" t="inlineStr">
         <is>
           <t>1 - Vehiculos motorizados terrestres</t>
         </is>
       </c>
-      <c r="B7" s="64" t="inlineStr">
+      <c r="B7" s="66" t="inlineStr">
         <is>
           <t>PBF9690</t>
         </is>
       </c>
-      <c r="C7" s="64" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="D7" s="64" t="inlineStr">
+      <c r="D7" s="65" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="E7" s="64" t="inlineStr"/>
-      <c r="F7" s="64" t="inlineStr"/>
-      <c r="G7" s="65" t="n">
+      <c r="E7" s="65" t="inlineStr"/>
+      <c r="F7" s="66" t="inlineStr"/>
+      <c r="G7" s="67" t="n">
         <v>20000</v>
       </c>
-      <c r="H7" s="62" t="n">
+      <c r="H7" s="63" t="n">
         <v>20000</v>
       </c>
-      <c r="I7" s="65">
+      <c r="I7" s="67">
         <f>H7-G7</f>
         <v/>
       </c>
-      <c r="J7" s="66">
+      <c r="J7" s="68">
         <f>IF(G7=0,"",(H7-G7)/G7)</f>
         <v/>
       </c>
@@ -14072,7 +14078,7 @@
           <t>1 - Vehiculos motorizados terrestres</t>
         </is>
       </c>
-      <c r="B8" s="60" t="inlineStr">
+      <c r="B8" s="61" t="inlineStr">
         <is>
           <t>PFC8683</t>
         </is>
@@ -14088,33 +14094,33 @@
         </is>
       </c>
       <c r="E8" s="60" t="inlineStr"/>
-      <c r="F8" s="60" t="inlineStr"/>
-      <c r="G8" s="61" t="n">
+      <c r="F8" s="61" t="inlineStr"/>
+      <c r="G8" s="62" t="n">
         <v>32000</v>
       </c>
-      <c r="H8" s="62" t="n">
+      <c r="H8" s="63" t="n">
         <v>32000</v>
       </c>
-      <c r="I8" s="61">
+      <c r="I8" s="62">
         <f>H8-G8</f>
         <v/>
       </c>
-      <c r="J8" s="63">
+      <c r="J8" s="64">
         <f>IF(G8=0,"",(H8-G8)/G8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="67" t="inlineStr">
+      <c r="A9" s="69" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="67" t="n"/>
-      <c r="C9" s="67" t="n"/>
-      <c r="D9" s="67" t="n"/>
-      <c r="E9" s="67" t="n"/>
-      <c r="F9" s="67" t="n"/>
+      <c r="B9" s="69" t="n"/>
+      <c r="C9" s="69" t="n"/>
+      <c r="D9" s="69" t="n"/>
+      <c r="E9" s="69" t="n"/>
+      <c r="F9" s="69" t="n"/>
       <c r="G9" s="31">
         <f>SUM(G6:G8)</f>
         <v/>
@@ -14245,39 +14251,39 @@
       <c r="B6" s="60" t="inlineStr"/>
       <c r="C6" s="60" t="inlineStr"/>
       <c r="D6" s="60" t="inlineStr"/>
-      <c r="E6" s="60" t="inlineStr"/>
-      <c r="F6" s="62" t="n">
+      <c r="E6" s="61" t="inlineStr"/>
+      <c r="F6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="62" t="n">
+      <c r="G6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="61">
+      <c r="H6" s="62">
         <f>G6-F6</f>
         <v/>
       </c>
-      <c r="I6" s="63">
+      <c r="I6" s="64">
         <f>IF(F6=0,"",(G6-F6)/F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr"/>
-      <c r="B7" s="64" t="inlineStr"/>
-      <c r="C7" s="64" t="inlineStr"/>
-      <c r="D7" s="64" t="inlineStr"/>
-      <c r="E7" s="64" t="inlineStr"/>
-      <c r="F7" s="62" t="n">
+      <c r="A7" s="65" t="inlineStr"/>
+      <c r="B7" s="65" t="inlineStr"/>
+      <c r="C7" s="65" t="inlineStr"/>
+      <c r="D7" s="65" t="inlineStr"/>
+      <c r="E7" s="66" t="inlineStr"/>
+      <c r="F7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="62" t="n">
+      <c r="G7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="65">
+      <c r="H7" s="67">
         <f>G7-F7</f>
         <v/>
       </c>
-      <c r="I7" s="66">
+      <c r="I7" s="68">
         <f>IF(F7=0,"",(G7-F7)/F7)</f>
         <v/>
       </c>
@@ -14287,39 +14293,39 @@
       <c r="B8" s="60" t="inlineStr"/>
       <c r="C8" s="60" t="inlineStr"/>
       <c r="D8" s="60" t="inlineStr"/>
-      <c r="E8" s="60" t="inlineStr"/>
-      <c r="F8" s="62" t="n">
+      <c r="E8" s="61" t="inlineStr"/>
+      <c r="F8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="62" t="n">
+      <c r="G8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="61">
+      <c r="H8" s="62">
         <f>G8-F8</f>
         <v/>
       </c>
-      <c r="I8" s="63">
+      <c r="I8" s="64">
         <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="64" t="inlineStr"/>
-      <c r="B9" s="64" t="inlineStr"/>
-      <c r="C9" s="64" t="inlineStr"/>
-      <c r="D9" s="64" t="inlineStr"/>
-      <c r="E9" s="64" t="inlineStr"/>
-      <c r="F9" s="62" t="n">
+      <c r="A9" s="65" t="inlineStr"/>
+      <c r="B9" s="65" t="inlineStr"/>
+      <c r="C9" s="65" t="inlineStr"/>
+      <c r="D9" s="65" t="inlineStr"/>
+      <c r="E9" s="66" t="inlineStr"/>
+      <c r="F9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="62" t="n">
+      <c r="G9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="65">
+      <c r="H9" s="67">
         <f>G9-F9</f>
         <v/>
       </c>
-      <c r="I9" s="66">
+      <c r="I9" s="68">
         <f>IF(F9=0,"",(G9-F9)/F9)</f>
         <v/>
       </c>
@@ -14329,39 +14335,39 @@
       <c r="B10" s="60" t="inlineStr"/>
       <c r="C10" s="60" t="inlineStr"/>
       <c r="D10" s="60" t="inlineStr"/>
-      <c r="E10" s="60" t="inlineStr"/>
-      <c r="F10" s="62" t="n">
+      <c r="E10" s="61" t="inlineStr"/>
+      <c r="F10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="62" t="n">
+      <c r="G10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="61">
+      <c r="H10" s="62">
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="63">
+      <c r="I10" s="64">
         <f>IF(F10=0,"",(G10-F10)/F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="64" t="inlineStr"/>
-      <c r="B11" s="64" t="inlineStr"/>
-      <c r="C11" s="64" t="inlineStr"/>
-      <c r="D11" s="64" t="inlineStr"/>
-      <c r="E11" s="64" t="inlineStr"/>
-      <c r="F11" s="62" t="n">
+      <c r="A11" s="65" t="inlineStr"/>
+      <c r="B11" s="65" t="inlineStr"/>
+      <c r="C11" s="65" t="inlineStr"/>
+      <c r="D11" s="65" t="inlineStr"/>
+      <c r="E11" s="66" t="inlineStr"/>
+      <c r="F11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="62" t="n">
+      <c r="G11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="65">
+      <c r="H11" s="67">
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="66">
+      <c r="I11" s="68">
         <f>IF(F11=0,"",(G11-F11)/F11)</f>
         <v/>
       </c>
@@ -14371,53 +14377,53 @@
       <c r="B12" s="60" t="inlineStr"/>
       <c r="C12" s="60" t="inlineStr"/>
       <c r="D12" s="60" t="inlineStr"/>
-      <c r="E12" s="60" t="inlineStr"/>
-      <c r="F12" s="62" t="n">
+      <c r="E12" s="61" t="inlineStr"/>
+      <c r="F12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="62" t="n">
+      <c r="G12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="61">
+      <c r="H12" s="62">
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="63">
+      <c r="I12" s="64">
         <f>IF(F12=0,"",(G12-F12)/F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="64" t="inlineStr"/>
-      <c r="B13" s="64" t="inlineStr"/>
-      <c r="C13" s="64" t="inlineStr"/>
-      <c r="D13" s="64" t="inlineStr"/>
-      <c r="E13" s="64" t="inlineStr"/>
-      <c r="F13" s="62" t="n">
+      <c r="A13" s="65" t="inlineStr"/>
+      <c r="B13" s="65" t="inlineStr"/>
+      <c r="C13" s="65" t="inlineStr"/>
+      <c r="D13" s="65" t="inlineStr"/>
+      <c r="E13" s="66" t="inlineStr"/>
+      <c r="F13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="62" t="n">
+      <c r="G13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="65">
+      <c r="H13" s="67">
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="66">
+      <c r="I13" s="68">
         <f>IF(F13=0,"",(G13-F13)/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="67" t="inlineStr">
+      <c r="A14" s="69" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="67" t="n"/>
-      <c r="C14" s="67" t="n"/>
-      <c r="D14" s="67" t="n"/>
-      <c r="E14" s="67" t="n"/>
+      <c r="B14" s="69" t="n"/>
+      <c r="C14" s="69" t="n"/>
+      <c r="D14" s="69" t="n"/>
+      <c r="E14" s="69" t="n"/>
       <c r="F14" s="31">
         <f>SUM(F6:F13)</f>
         <v/>
@@ -14593,82 +14599,82 @@
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F6" s="60" t="inlineStr">
+      <c r="F6" s="61" t="inlineStr">
         <is>
           <t>22/10/2008</t>
         </is>
       </c>
-      <c r="G6" s="60" t="inlineStr">
+      <c r="G6" s="61" t="inlineStr">
         <is>
           <t>1042203018</t>
         </is>
       </c>
       <c r="H6" s="60" t="inlineStr"/>
-      <c r="I6" s="60" t="inlineStr"/>
-      <c r="J6" s="61" t="n">
+      <c r="I6" s="61" t="inlineStr"/>
+      <c r="J6" s="62" t="n">
         <v>267340.8</v>
       </c>
-      <c r="K6" s="62" t="n">
+      <c r="K6" s="63" t="n">
         <v>267340.8</v>
       </c>
-      <c r="L6" s="61">
+      <c r="L6" s="62">
         <f>K6-J6</f>
         <v/>
       </c>
-      <c r="M6" s="63">
+      <c r="M6" s="64">
         <f>IF(J6=0,"",(K6-J6)/J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr">
+      <c r="A7" s="65" t="inlineStr">
         <is>
           <t>1 - Casa</t>
         </is>
       </c>
-      <c r="B7" s="64" t="inlineStr">
+      <c r="B7" s="65" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C7" s="64" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D7" s="64" t="inlineStr">
+      <c r="D7" s="65" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E7" s="64" t="inlineStr">
+      <c r="E7" s="65" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F7" s="64" t="inlineStr">
+      <c r="F7" s="66" t="inlineStr">
         <is>
           <t>13/03/1997</t>
         </is>
       </c>
-      <c r="G7" s="64" t="inlineStr">
+      <c r="G7" s="66" t="inlineStr">
         <is>
           <t>1012005008000000000</t>
         </is>
       </c>
-      <c r="H7" s="64" t="inlineStr"/>
-      <c r="I7" s="64" t="inlineStr"/>
-      <c r="J7" s="65" t="n">
+      <c r="H7" s="65" t="inlineStr"/>
+      <c r="I7" s="66" t="inlineStr"/>
+      <c r="J7" s="67" t="n">
         <v>198118.55</v>
       </c>
-      <c r="K7" s="62" t="n">
+      <c r="K7" s="63" t="n">
         <v>198118.55</v>
       </c>
-      <c r="L7" s="65">
+      <c r="L7" s="67">
         <f>K7-J7</f>
         <v/>
       </c>
-      <c r="M7" s="66">
+      <c r="M7" s="68">
         <f>IF(J7=0,"",(K7-J7)/J7)</f>
         <v/>
       </c>
@@ -14699,92 +14705,92 @@
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F8" s="60" t="inlineStr"/>
-      <c r="G8" s="60" t="inlineStr">
+      <c r="F8" s="61" t="inlineStr"/>
+      <c r="G8" s="61" t="inlineStr">
         <is>
           <t>1042203018</t>
         </is>
       </c>
       <c r="H8" s="60" t="inlineStr"/>
-      <c r="I8" s="60" t="inlineStr"/>
-      <c r="J8" s="61" t="n">
+      <c r="I8" s="61" t="inlineStr"/>
+      <c r="J8" s="62" t="n">
         <v>33634.04</v>
       </c>
-      <c r="K8" s="62" t="n">
+      <c r="K8" s="63" t="n">
         <v>33634.04</v>
       </c>
-      <c r="L8" s="61">
+      <c r="L8" s="62">
         <f>K8-J8</f>
         <v/>
       </c>
-      <c r="M8" s="63">
+      <c r="M8" s="64">
         <f>IF(J8=0,"",(K8-J8)/J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="64" t="inlineStr">
+      <c r="A9" s="65" t="inlineStr">
         <is>
           <t>3 - Terreno</t>
         </is>
       </c>
-      <c r="B9" s="64" t="inlineStr">
+      <c r="B9" s="65" t="inlineStr">
         <is>
           <t>ECU - En el Ecuador</t>
         </is>
       </c>
-      <c r="C9" s="64" t="inlineStr">
+      <c r="C9" s="65" t="inlineStr">
         <is>
           <t>593 - ECUADOR</t>
         </is>
       </c>
-      <c r="D9" s="64" t="inlineStr">
+      <c r="D9" s="65" t="inlineStr">
         <is>
           <t>217 - PICHINCHA</t>
         </is>
       </c>
-      <c r="E9" s="64" t="inlineStr">
+      <c r="E9" s="65" t="inlineStr">
         <is>
           <t>21701 - QUITO</t>
         </is>
       </c>
-      <c r="F9" s="64" t="inlineStr"/>
-      <c r="G9" s="64" t="inlineStr">
+      <c r="F9" s="66" t="inlineStr"/>
+      <c r="G9" s="66" t="inlineStr">
         <is>
           <t>1012005008000000000</t>
         </is>
       </c>
-      <c r="H9" s="64" t="inlineStr"/>
-      <c r="I9" s="64" t="inlineStr"/>
-      <c r="J9" s="65" t="n">
+      <c r="H9" s="65" t="inlineStr"/>
+      <c r="I9" s="66" t="inlineStr"/>
+      <c r="J9" s="67" t="n">
         <v>82624.22</v>
       </c>
-      <c r="K9" s="62" t="n">
+      <c r="K9" s="63" t="n">
         <v>82624.22</v>
       </c>
-      <c r="L9" s="65">
+      <c r="L9" s="67">
         <f>K9-J9</f>
         <v/>
       </c>
-      <c r="M9" s="66">
+      <c r="M9" s="68">
         <f>IF(J9=0,"",(K9-J9)/J9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="67" t="inlineStr">
+      <c r="A10" s="69" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B10" s="67" t="n"/>
-      <c r="C10" s="67" t="n"/>
-      <c r="D10" s="67" t="n"/>
-      <c r="E10" s="67" t="n"/>
-      <c r="F10" s="67" t="n"/>
-      <c r="G10" s="67" t="n"/>
-      <c r="H10" s="67" t="n"/>
-      <c r="I10" s="67" t="n"/>
+      <c r="B10" s="69" t="n"/>
+      <c r="C10" s="69" t="n"/>
+      <c r="D10" s="69" t="n"/>
+      <c r="E10" s="69" t="n"/>
+      <c r="F10" s="69" t="n"/>
+      <c r="G10" s="69" t="n"/>
+      <c r="H10" s="69" t="n"/>
+      <c r="I10" s="69" t="n"/>
       <c r="J10" s="31">
         <f>SUM(J6:J9)</f>
         <v/>
@@ -14919,41 +14925,41 @@
     <row r="6">
       <c r="A6" s="60" t="inlineStr"/>
       <c r="B6" s="60" t="inlineStr"/>
-      <c r="C6" s="60" t="inlineStr"/>
+      <c r="C6" s="61" t="inlineStr"/>
       <c r="D6" s="60" t="inlineStr"/>
-      <c r="E6" s="60" t="inlineStr"/>
-      <c r="F6" s="62" t="n">
+      <c r="E6" s="61" t="inlineStr"/>
+      <c r="F6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="62" t="n">
+      <c r="G6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="61">
+      <c r="H6" s="62">
         <f>G6-F6</f>
         <v/>
       </c>
-      <c r="I6" s="63">
+      <c r="I6" s="64">
         <f>IF(F6=0,"",(G6-F6)/F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr"/>
-      <c r="B7" s="64" t="inlineStr"/>
-      <c r="C7" s="64" t="inlineStr"/>
-      <c r="D7" s="64" t="inlineStr"/>
-      <c r="E7" s="64" t="inlineStr"/>
-      <c r="F7" s="62" t="n">
+      <c r="A7" s="65" t="inlineStr"/>
+      <c r="B7" s="65" t="inlineStr"/>
+      <c r="C7" s="66" t="inlineStr"/>
+      <c r="D7" s="65" t="inlineStr"/>
+      <c r="E7" s="66" t="inlineStr"/>
+      <c r="F7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="62" t="n">
+      <c r="G7" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="65">
+      <c r="H7" s="67">
         <f>G7-F7</f>
         <v/>
       </c>
-      <c r="I7" s="66">
+      <c r="I7" s="68">
         <f>IF(F7=0,"",(G7-F7)/F7)</f>
         <v/>
       </c>
@@ -14961,41 +14967,41 @@
     <row r="8">
       <c r="A8" s="60" t="inlineStr"/>
       <c r="B8" s="60" t="inlineStr"/>
-      <c r="C8" s="60" t="inlineStr"/>
+      <c r="C8" s="61" t="inlineStr"/>
       <c r="D8" s="60" t="inlineStr"/>
-      <c r="E8" s="60" t="inlineStr"/>
-      <c r="F8" s="62" t="n">
+      <c r="E8" s="61" t="inlineStr"/>
+      <c r="F8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="62" t="n">
+      <c r="G8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="61">
+      <c r="H8" s="62">
         <f>G8-F8</f>
         <v/>
       </c>
-      <c r="I8" s="63">
+      <c r="I8" s="64">
         <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="64" t="inlineStr"/>
-      <c r="B9" s="64" t="inlineStr"/>
-      <c r="C9" s="64" t="inlineStr"/>
-      <c r="D9" s="64" t="inlineStr"/>
-      <c r="E9" s="64" t="inlineStr"/>
-      <c r="F9" s="62" t="n">
+      <c r="A9" s="65" t="inlineStr"/>
+      <c r="B9" s="65" t="inlineStr"/>
+      <c r="C9" s="66" t="inlineStr"/>
+      <c r="D9" s="65" t="inlineStr"/>
+      <c r="E9" s="66" t="inlineStr"/>
+      <c r="F9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="62" t="n">
+      <c r="G9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="65">
+      <c r="H9" s="67">
         <f>G9-F9</f>
         <v/>
       </c>
-      <c r="I9" s="66">
+      <c r="I9" s="68">
         <f>IF(F9=0,"",(G9-F9)/F9)</f>
         <v/>
       </c>
@@ -15003,41 +15009,41 @@
     <row r="10">
       <c r="A10" s="60" t="inlineStr"/>
       <c r="B10" s="60" t="inlineStr"/>
-      <c r="C10" s="60" t="inlineStr"/>
+      <c r="C10" s="61" t="inlineStr"/>
       <c r="D10" s="60" t="inlineStr"/>
-      <c r="E10" s="60" t="inlineStr"/>
-      <c r="F10" s="62" t="n">
+      <c r="E10" s="61" t="inlineStr"/>
+      <c r="F10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="62" t="n">
+      <c r="G10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="61">
+      <c r="H10" s="62">
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="63">
+      <c r="I10" s="64">
         <f>IF(F10=0,"",(G10-F10)/F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="64" t="inlineStr"/>
-      <c r="B11" s="64" t="inlineStr"/>
-      <c r="C11" s="64" t="inlineStr"/>
-      <c r="D11" s="64" t="inlineStr"/>
-      <c r="E11" s="64" t="inlineStr"/>
-      <c r="F11" s="62" t="n">
+      <c r="A11" s="65" t="inlineStr"/>
+      <c r="B11" s="65" t="inlineStr"/>
+      <c r="C11" s="66" t="inlineStr"/>
+      <c r="D11" s="65" t="inlineStr"/>
+      <c r="E11" s="66" t="inlineStr"/>
+      <c r="F11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="62" t="n">
+      <c r="G11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="65">
+      <c r="H11" s="67">
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="66">
+      <c r="I11" s="68">
         <f>IF(F11=0,"",(G11-F11)/F11)</f>
         <v/>
       </c>
@@ -15045,55 +15051,55 @@
     <row r="12">
       <c r="A12" s="60" t="inlineStr"/>
       <c r="B12" s="60" t="inlineStr"/>
-      <c r="C12" s="60" t="inlineStr"/>
+      <c r="C12" s="61" t="inlineStr"/>
       <c r="D12" s="60" t="inlineStr"/>
-      <c r="E12" s="60" t="inlineStr"/>
-      <c r="F12" s="62" t="n">
+      <c r="E12" s="61" t="inlineStr"/>
+      <c r="F12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="62" t="n">
+      <c r="G12" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="61">
+      <c r="H12" s="62">
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="63">
+      <c r="I12" s="64">
         <f>IF(F12=0,"",(G12-F12)/F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="64" t="inlineStr"/>
-      <c r="B13" s="64" t="inlineStr"/>
-      <c r="C13" s="64" t="inlineStr"/>
-      <c r="D13" s="64" t="inlineStr"/>
-      <c r="E13" s="64" t="inlineStr"/>
-      <c r="F13" s="62" t="n">
+      <c r="A13" s="65" t="inlineStr"/>
+      <c r="B13" s="65" t="inlineStr"/>
+      <c r="C13" s="66" t="inlineStr"/>
+      <c r="D13" s="65" t="inlineStr"/>
+      <c r="E13" s="66" t="inlineStr"/>
+      <c r="F13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="62" t="n">
+      <c r="G13" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="65">
+      <c r="H13" s="67">
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="66">
+      <c r="I13" s="68">
         <f>IF(F13=0,"",(G13-F13)/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="67" t="inlineStr">
+      <c r="A14" s="69" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="67" t="n"/>
-      <c r="C14" s="67" t="n"/>
-      <c r="D14" s="67" t="n"/>
-      <c r="E14" s="67" t="n"/>
+      <c r="B14" s="69" t="n"/>
+      <c r="C14" s="69" t="n"/>
+      <c r="D14" s="69" t="n"/>
+      <c r="E14" s="69" t="n"/>
       <c r="F14" s="31">
         <f>SUM(F6:F13)</f>
         <v/>

</xml_diff>